<commit_message>
Update Excel file floor 1,2
</commit_message>
<xml_diff>
--- a/assets/floor_1_data.xlsx
+++ b/assets/floor_1_data.xlsx
@@ -529,7 +529,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -556,65 +556,65 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>WIFI-AP-Lobby</v>
+        <v>SRV-DC-01</v>
       </c>
       <c r="B2" t="str">
-        <v>AP</v>
+        <v>Server</v>
       </c>
       <c r="C2">
-        <v>-800</v>
+        <v>-1500</v>
       </c>
       <c r="D2">
-        <v>1200</v>
+        <v>-1300</v>
       </c>
       <c r="E2" t="str">
-        <v>Main entrance access point</v>
+        <v>Domain Controller 1</v>
       </c>
       <c r="F2" t="str">
         <v>Active</v>
       </c>
-      <c r="G2" s="1">
-        <v>44927</v>
+      <c r="G2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>WIFI-AP-Canteen</v>
+        <v>SRV-FS-01</v>
       </c>
       <c r="B3" t="str">
-        <v>AP</v>
+        <v>Server</v>
       </c>
       <c r="C3">
-        <v>550</v>
+        <v>-1550</v>
       </c>
       <c r="D3">
-        <v>900</v>
+        <v>-1300</v>
       </c>
       <c r="E3" t="str">
-        <v>Cafeteria coverage</v>
+        <v>File Server 1</v>
       </c>
       <c r="F3" t="str">
-        <v>Inactive</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
+        <v>Active</v>
+      </c>
+      <c r="G3" s="1">
+        <v>44927</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>SRV-DC-01</v>
+        <v>SW-IDF-01</v>
       </c>
       <c r="B4" t="str">
-        <v>Server</v>
+        <v>Switch</v>
       </c>
       <c r="C4">
-        <v>-1500</v>
+        <v>-1450</v>
       </c>
       <c r="D4">
-        <v>-1300</v>
+        <v>-1350</v>
       </c>
       <c r="E4" t="str">
-        <v>Domain Controller 1</v>
+        <v>Main Distribution Frame Switch</v>
       </c>
       <c r="F4" t="str">
         <v>Active</v>
@@ -625,19 +625,19 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>SRV-FS-01</v>
+        <v>AP-001</v>
       </c>
       <c r="B5" t="str">
-        <v>Server</v>
+        <v>AP</v>
       </c>
       <c r="C5">
-        <v>-1550</v>
+        <v>-1293</v>
       </c>
       <c r="D5">
-        <v>-1300</v>
+        <v>519</v>
       </c>
       <c r="E5" t="str">
-        <v>File Server 1</v>
+        <v>Main entrance access point</v>
       </c>
       <c r="F5" t="str">
         <v>Active</v>
@@ -648,30 +648,329 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>SW-IDF-01</v>
+        <v>AP-002</v>
       </c>
       <c r="B6" t="str">
-        <v>Switch</v>
+        <v>AP</v>
       </c>
       <c r="C6">
-        <v>-1450</v>
+        <v>-614</v>
       </c>
       <c r="D6">
-        <v>-1350</v>
+        <v>71</v>
       </c>
       <c r="E6" t="str">
-        <v>Main Distribution Frame Switch</v>
+        <v>Cafeteria coverage</v>
       </c>
       <c r="F6" t="str">
         <v>Active</v>
       </c>
       <c r="G6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>AP-003</v>
+      </c>
+      <c r="B7" t="str">
+        <v>AP</v>
+      </c>
+      <c r="C7">
+        <v>-339</v>
+      </c>
+      <c r="D7">
+        <v>-1235</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>AP-004</v>
+      </c>
+      <c r="B8" t="str">
+        <v>AP</v>
+      </c>
+      <c r="C8">
+        <v>587</v>
+      </c>
+      <c r="D8">
+        <v>-1129</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>AP-005</v>
+      </c>
+      <c r="B9" t="str">
+        <v>AP</v>
+      </c>
+      <c r="C9">
+        <v>558</v>
+      </c>
+      <c r="D9">
+        <v>-186</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>AP-006</v>
+      </c>
+      <c r="B10" t="str">
+        <v>AP</v>
+      </c>
+      <c r="C10">
+        <v>1002</v>
+      </c>
+      <c r="D10">
+        <v>-426</v>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>AP-007</v>
+      </c>
+      <c r="B11" t="str">
+        <v>AP</v>
+      </c>
+      <c r="C11">
+        <v>995</v>
+      </c>
+      <c r="D11">
+        <v>-774</v>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>AP-008</v>
+      </c>
+      <c r="B12" t="str">
+        <v>AP</v>
+      </c>
+      <c r="C12">
+        <v>1268</v>
+      </c>
+      <c r="D12">
+        <v>-648</v>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>AP-009</v>
+      </c>
+      <c r="B13" t="str">
+        <v>AP</v>
+      </c>
+      <c r="C13">
+        <v>1252</v>
+      </c>
+      <c r="D13">
+        <v>-33</v>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>AP-010</v>
+      </c>
+      <c r="B14" t="str">
+        <v>AP</v>
+      </c>
+      <c r="C14">
+        <v>1545</v>
+      </c>
+      <c r="D14">
+        <v>-1153</v>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>AP-011</v>
+      </c>
+      <c r="B15" t="str">
+        <v>AP</v>
+      </c>
+      <c r="C15">
+        <v>2102</v>
+      </c>
+      <c r="D15">
+        <v>-391</v>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>AP-012</v>
+      </c>
+      <c r="B16" t="str">
+        <v>AP</v>
+      </c>
+      <c r="C16">
+        <v>2003</v>
+      </c>
+      <c r="D16">
+        <v>-1086</v>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>AP-013</v>
+      </c>
+      <c r="B17" t="str">
+        <v>AP</v>
+      </c>
+      <c r="C17">
+        <v>2309</v>
+      </c>
+      <c r="D17">
+        <v>38</v>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>AP-014</v>
+      </c>
+      <c r="B18" t="str">
+        <v>AP</v>
+      </c>
+      <c r="C18">
+        <v>2347</v>
+      </c>
+      <c r="D18">
+        <v>-552</v>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>AP-015</v>
+      </c>
+      <c r="B19" t="str">
+        <v>AP</v>
+      </c>
+      <c r="C19">
+        <v>2645</v>
+      </c>
+      <c r="D19">
+        <v>559</v>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G19" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G19"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Paper Form asset
</commit_message>
<xml_diff>
--- a/assets/floor_1_data.xlsx
+++ b/assets/floor_1_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\M.Mead\5.FactoryView\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FD85265-95B9-4E70-9455-E41AB33E9222}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{574D2672-E366-4828-BAF2-79CA0670337C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25260" yWindow="2460" windowWidth="21600" windowHeight="11295" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loc_name" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="pers_lap" sheetId="4" r:id="rId4"/>
     <sheet name="weight" sheetId="5" r:id="rId5"/>
     <sheet name="cam" sheetId="6" r:id="rId6"/>
+    <sheet name="paper" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="79">
   <si>
     <t>Name</t>
   </si>
@@ -258,6 +259,15 @@
   </si>
   <si>
     <t>Salmon</t>
+  </si>
+  <si>
+    <t>T.Slip</t>
+  </si>
+  <si>
+    <t>Test Paper</t>
+  </si>
+  <si>
+    <t>Paper</t>
   </si>
 </sst>
 </file>
@@ -1775,4 +1785,57 @@
     <ignoredError sqref="A1:H4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB643B34-7A2A-4A47-AF69-189BDD7E5EC7}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C2">
+        <v>-450</v>
+      </c>
+      <c r="D2">
+        <v>-220</v>
+      </c>
+      <c r="E2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add display custom fields, start with it layer, update Excel source
</commit_message>
<xml_diff>
--- a/assets/floor_1_data.xlsx
+++ b/assets/floor_1_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\M.Mead\5.FactoryView\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\M.Mead\9.FactoryView\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{574D2672-E366-4828-BAF2-79CA0670337C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E6CDD60-9DF1-434E-8F69-75648D7BE864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25260" yWindow="2460" windowWidth="21600" windowHeight="11295" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loc_name" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="149">
   <si>
     <t>Name</t>
   </si>
@@ -96,9 +96,6 @@
     <t>Truck Loading Area</t>
   </si>
   <si>
-    <t>AP-001</t>
-  </si>
-  <si>
     <t>AP</t>
   </si>
   <si>
@@ -108,57 +105,15 @@
     <t>Orange</t>
   </si>
   <si>
-    <t>AP-002</t>
-  </si>
-  <si>
     <t>Cafeteria coverage</t>
   </si>
   <si>
-    <t>AP-003</t>
-  </si>
-  <si>
     <t>Violet</t>
   </si>
   <si>
-    <t>AP-004</t>
-  </si>
-  <si>
-    <t>AP-005</t>
-  </si>
-  <si>
-    <t>AP-006</t>
-  </si>
-  <si>
-    <t>AP-007</t>
-  </si>
-  <si>
-    <t>AP-008</t>
-  </si>
-  <si>
-    <t>AP-009</t>
-  </si>
-  <si>
-    <t>AP-010</t>
-  </si>
-  <si>
-    <t>AP-011</t>
-  </si>
-  <si>
     <t>Blue</t>
   </si>
   <si>
-    <t>AP-012</t>
-  </si>
-  <si>
-    <t>AP-013</t>
-  </si>
-  <si>
-    <t>AP-014</t>
-  </si>
-  <si>
-    <t>AP-015</t>
-  </si>
-  <si>
     <t>AP01c</t>
   </si>
   <si>
@@ -268,6 +223,261 @@
   </si>
   <si>
     <t>Paper</t>
+  </si>
+  <si>
+    <t>AP-01</t>
+  </si>
+  <si>
+    <t>AP-02</t>
+  </si>
+  <si>
+    <t>AP-03</t>
+  </si>
+  <si>
+    <t>AP-04</t>
+  </si>
+  <si>
+    <t>AP-05</t>
+  </si>
+  <si>
+    <t>AP-06</t>
+  </si>
+  <si>
+    <t>AP-07</t>
+  </si>
+  <si>
+    <t>AP-08</t>
+  </si>
+  <si>
+    <t>AP-09</t>
+  </si>
+  <si>
+    <t>AP-10</t>
+  </si>
+  <si>
+    <t>AP-11</t>
+  </si>
+  <si>
+    <t>AP-12</t>
+  </si>
+  <si>
+    <t>AP-13</t>
+  </si>
+  <si>
+    <t>AP-14</t>
+  </si>
+  <si>
+    <t>AP-15</t>
+  </si>
+  <si>
+    <t>IP Address</t>
+  </si>
+  <si>
+    <t>MAC Address</t>
+  </si>
+  <si>
+    <t>Platform</t>
+  </si>
+  <si>
+    <t>Serial Number</t>
+  </si>
+  <si>
+    <t>10.198.85.151</t>
+  </si>
+  <si>
+    <t>f8:14:dd:a2:62:00</t>
+  </si>
+  <si>
+    <t>CW9176I</t>
+  </si>
+  <si>
+    <t>WVN29470BSP</t>
+  </si>
+  <si>
+    <t>10.198.85.154</t>
+  </si>
+  <si>
+    <t>f8:14:dd:a2:64:40</t>
+  </si>
+  <si>
+    <t>WVN29470BT7</t>
+  </si>
+  <si>
+    <t>10.198.85.146</t>
+  </si>
+  <si>
+    <t>f8:14:dd:a2:60:80</t>
+  </si>
+  <si>
+    <t>WVN29470BSB</t>
+  </si>
+  <si>
+    <t>10.198.85.145</t>
+  </si>
+  <si>
+    <t>f8:14:dd:a2:66:60</t>
+  </si>
+  <si>
+    <t>WVN29470BTQ</t>
+  </si>
+  <si>
+    <t>10.198.85.152</t>
+  </si>
+  <si>
+    <t>f8:14:dd:a2:52:a0</t>
+  </si>
+  <si>
+    <t>WVN29470BP2</t>
+  </si>
+  <si>
+    <t>10.198.85.147</t>
+  </si>
+  <si>
+    <t>f8:14:dd:a2:82:00</t>
+  </si>
+  <si>
+    <t>WVN29470C07</t>
+  </si>
+  <si>
+    <t>10.198.85.149</t>
+  </si>
+  <si>
+    <t>f8:14:dd:a2:82:20</t>
+  </si>
+  <si>
+    <t>WVN29470C08</t>
+  </si>
+  <si>
+    <t>10.198.85.150</t>
+  </si>
+  <si>
+    <t>f8:14:dd:a2:57:60</t>
+  </si>
+  <si>
+    <t>WVN29470BQ6</t>
+  </si>
+  <si>
+    <t>10.198.85.148</t>
+  </si>
+  <si>
+    <t>f8:14:dd:a2:63:60</t>
+  </si>
+  <si>
+    <t>WVN29470BT0</t>
+  </si>
+  <si>
+    <t>10.198.85.153</t>
+  </si>
+  <si>
+    <t>f8:14:dd:a2:42:a0</t>
+  </si>
+  <si>
+    <t>WVN29470BKA</t>
+  </si>
+  <si>
+    <t>10.198.85.155</t>
+  </si>
+  <si>
+    <t>f8:14:dd:a2:60:c0</t>
+  </si>
+  <si>
+    <t>WVN29470BSD</t>
+  </si>
+  <si>
+    <t>10.198.85.163</t>
+  </si>
+  <si>
+    <t>f8:14:dd:a2:65:40</t>
+  </si>
+  <si>
+    <t>WVN29470BTF</t>
+  </si>
+  <si>
+    <t>10.198.85.161</t>
+  </si>
+  <si>
+    <t>f8:14:dd:a2:5d:20</t>
+  </si>
+  <si>
+    <t>WVN29470BRJ</t>
+  </si>
+  <si>
+    <t>10.198.85.160</t>
+  </si>
+  <si>
+    <t>f8:14:dd:a2:57:40</t>
+  </si>
+  <si>
+    <t>WVN29470BQ5</t>
+  </si>
+  <si>
+    <t>10.198.85.162</t>
+  </si>
+  <si>
+    <t>f8:14:dd:a2:89:80</t>
+  </si>
+  <si>
+    <t>WVN29470C1Z</t>
+  </si>
+  <si>
+    <t>Switch Detail</t>
+  </si>
+  <si>
+    <t>Port Details</t>
+  </si>
+  <si>
+    <t>THJMNMCHOTH01S04</t>
+  </si>
+  <si>
+    <t>Gi2/0/4</t>
+  </si>
+  <si>
+    <t>Gi2/0/5</t>
+  </si>
+  <si>
+    <t>THCHON-CCB-AS10</t>
+  </si>
+  <si>
+    <t>G1/0/12</t>
+  </si>
+  <si>
+    <t>G1/0/13</t>
+  </si>
+  <si>
+    <t>G1/0/14</t>
+  </si>
+  <si>
+    <t>G1/0/15</t>
+  </si>
+  <si>
+    <t>G1/0/16</t>
+  </si>
+  <si>
+    <t>G1/0/17</t>
+  </si>
+  <si>
+    <t>G1/0/18</t>
+  </si>
+  <si>
+    <t>G1/0/19</t>
+  </si>
+  <si>
+    <t>THJMNMCHOTH01S02</t>
+  </si>
+  <si>
+    <t>Gi1/0/29</t>
+  </si>
+  <si>
+    <t>Gi1/0/30</t>
+  </si>
+  <si>
+    <t>Gi1/0/31</t>
+  </si>
+  <si>
+    <t>Gi1/0/32</t>
+  </si>
+  <si>
+    <t>Gi1/0/33</t>
   </si>
 </sst>
 </file>
@@ -283,15 +493,33 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -299,13 +527,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -788,10 +1040,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="5" max="5" width="19.88671875" customWidth="1"/>
+    <col min="9" max="9" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -816,13 +1077,31 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I1" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" t="s">
         <v>21</v>
-      </c>
-      <c r="B2" t="s">
-        <v>22</v>
       </c>
       <c r="C2">
         <v>-1293</v>
@@ -831,7 +1110,7 @@
         <v>519</v>
       </c>
       <c r="E2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F2" t="s">
         <v>11</v>
@@ -840,15 +1119,33 @@
         <v>44927</v>
       </c>
       <c r="H2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="N2" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C3">
         <v>-614</v>
@@ -857,7 +1154,7 @@
         <v>71</v>
       </c>
       <c r="E3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F3" t="s">
         <v>11</v>
@@ -866,15 +1163,33 @@
         <v>12</v>
       </c>
       <c r="H3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>66</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C4">
         <v>-339</v>
@@ -892,15 +1207,33 @@
         <v>12</v>
       </c>
       <c r="H4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="N4" s="6" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>67</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C5">
         <v>587</v>
@@ -918,15 +1251,33 @@
         <v>12</v>
       </c>
       <c r="H5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C6">
         <v>558</v>
@@ -944,15 +1295,33 @@
         <v>12</v>
       </c>
       <c r="H6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>69</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C7">
         <v>1002</v>
@@ -970,15 +1339,33 @@
         <v>12</v>
       </c>
       <c r="H7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="N7" s="6" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C8">
         <v>995</v>
@@ -996,15 +1383,33 @@
         <v>12</v>
       </c>
       <c r="H8" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="N8" s="6" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C9">
         <v>1268</v>
@@ -1022,15 +1427,33 @@
         <v>12</v>
       </c>
       <c r="H9" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="M9" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="N9" s="6" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C10">
         <v>1252</v>
@@ -1048,15 +1471,33 @@
         <v>12</v>
       </c>
       <c r="H10" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="M10" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="N10" s="6" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>35</v>
+        <v>73</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C11">
         <v>1545</v>
@@ -1074,15 +1515,33 @@
         <v>12</v>
       </c>
       <c r="H11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="M11" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="N11" s="6" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C12">
         <v>2102</v>
@@ -1100,15 +1559,33 @@
         <v>12</v>
       </c>
       <c r="H12" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="M12" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="N12" s="6" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>38</v>
+        <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C13">
         <v>2003</v>
@@ -1126,15 +1603,33 @@
         <v>12</v>
       </c>
       <c r="H13" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="M13" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="N13" s="6" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>39</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C14">
         <v>2309</v>
@@ -1152,15 +1647,33 @@
         <v>12</v>
       </c>
       <c r="H14" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="M14" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="N14" s="6" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>40</v>
+        <v>77</v>
       </c>
       <c r="B15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C15">
         <v>2347</v>
@@ -1178,15 +1691,33 @@
         <v>12</v>
       </c>
       <c r="H15" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="M15" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="N15" s="6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="B16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C16">
         <v>2645</v>
@@ -1204,15 +1735,33 @@
         <v>12</v>
       </c>
       <c r="H16" t="s">
-        <v>37</v>
+        <v>26</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="L16" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="M16" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="N16" s="6" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C17">
         <v>-2111</v>
@@ -1224,21 +1773,21 @@
         <v>12</v>
       </c>
       <c r="F17" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="G17" t="s">
         <v>12</v>
       </c>
       <c r="H17" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C18">
         <v>-2407</v>
@@ -1250,21 +1799,21 @@
         <v>12</v>
       </c>
       <c r="F18" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="G18" t="s">
         <v>12</v>
       </c>
       <c r="H18" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="B19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C19">
         <v>-1884</v>
@@ -1276,21 +1825,21 @@
         <v>12</v>
       </c>
       <c r="F19" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="G19" t="s">
         <v>12</v>
       </c>
       <c r="H19" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="B20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C20">
         <v>-2019</v>
@@ -1302,21 +1851,21 @@
         <v>12</v>
       </c>
       <c r="F20" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="G20" t="s">
         <v>12</v>
       </c>
       <c r="H20" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="B21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C21">
         <v>-2394</v>
@@ -1328,21 +1877,21 @@
         <v>12</v>
       </c>
       <c r="F21" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="G21" t="s">
         <v>12</v>
       </c>
       <c r="H21" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="B22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C22">
         <v>-1925</v>
@@ -1354,19 +1903,19 @@
         <v>12</v>
       </c>
       <c r="F22" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="G22" t="s">
         <v>12</v>
       </c>
       <c r="H22" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:H16 A22:G22 A17:G17 A18:G18 A19:G19 A20:G20 A21:G21" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:H1 A22:G22 A17:G17 A18:G18 A19:G19 A20:G20 A21:G21 B16:H16 B2:H2 B3:H3 B4:H4 B5:H5 B6:H6 B7:H7 B8:H8 B9:H9 B10:H10 B11:H11 B12:H12 B13:H13 B14:H14 B15:H15" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1404,10 +1953,10 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="C2">
         <v>-450</v>
@@ -1416,7 +1965,7 @@
         <v>-200</v>
       </c>
       <c r="E2" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F2" t="s">
         <v>11</v>
@@ -1430,10 +1979,10 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="C3">
         <v>150</v>
@@ -1442,7 +1991,7 @@
         <v>-600</v>
       </c>
       <c r="E3" t="s">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="F3" t="s">
         <v>11</v>
@@ -1456,10 +2005,10 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="C4">
         <v>800</v>
@@ -1468,10 +2017,10 @@
         <v>250</v>
       </c>
       <c r="E4" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="F4" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="G4" t="s">
         <v>12</v>
@@ -1521,10 +2070,10 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="C2">
         <v>-336</v>
@@ -1533,13 +2082,13 @@
         <v>-446</v>
       </c>
       <c r="E2" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="F2" t="s">
         <v>11</v>
       </c>
       <c r="G2" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="H2" t="s">
         <v>12</v>
@@ -1586,10 +2135,10 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="C2">
         <v>1280</v>
@@ -1598,7 +2147,7 @@
         <v>-343</v>
       </c>
       <c r="E2" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="F2" t="s">
         <v>11</v>
@@ -1612,10 +2161,10 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="C3">
         <v>1289</v>
@@ -1624,7 +2173,7 @@
         <v>-243</v>
       </c>
       <c r="E3" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="F3" t="s">
         <v>11</v>
@@ -1638,10 +2187,10 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="B4" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="C4">
         <v>1349</v>
@@ -1650,7 +2199,7 @@
         <v>-130</v>
       </c>
       <c r="E4" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="F4" t="s">
         <v>11</v>
@@ -1703,10 +2252,10 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="B2" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="C2">
         <v>-900</v>
@@ -1715,7 +2264,7 @@
         <v>1250</v>
       </c>
       <c r="E2" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="F2" t="s">
         <v>11</v>
@@ -1729,10 +2278,10 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1741,7 +2290,7 @@
         <v>-1400</v>
       </c>
       <c r="E3" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="F3" t="s">
         <v>11</v>
@@ -1755,10 +2304,10 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="B4" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="C4">
         <v>600</v>
@@ -1767,7 +2316,7 @@
         <v>850</v>
       </c>
       <c r="E4" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="F4" t="s">
         <v>11</v>
@@ -1820,10 +2369,10 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="C2">
         <v>-450</v>
@@ -1832,7 +2381,7 @@
         <v>-220</v>
       </c>
       <c r="E2" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add animated flow paths layer for material flow visualization
New 'flow' renderType: CatmullRomCurve3 smooth paths with animated
LineDashedMaterial (dashOffset driven by delta time). 14 flow paths
for floor 1 covering warehouse outlet through tipping, blending,
pouch fillers/x-ray, and can filler/conveyor routes.

- AssetFactory: createFlowVisual() parses semicolon-delimited Points
- LayerManager: flow branch in addItem(), updateFlowAnimations(delta)
- Application: delta time tracking, calls updateFlowAnimations each frame
- DataLoader: Points/Speed/DashSize/GapSize added to STANDARD_COLS

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/floor_1_data.xlsx
+++ b/assets/floor_1_data.xlsx
@@ -14,6 +14,7 @@
     <sheet name="cam" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="paper" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="zones" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="flow" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -571,8 +572,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -601,8 +600,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -631,8 +628,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -661,8 +656,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -852,7 +845,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Orange</t>
@@ -906,13 +898,11 @@
       <c r="D4" t="n">
         <v>-1235</v>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>Violet</t>
@@ -966,13 +956,11 @@
       <c r="D5" t="n">
         <v>-1129</v>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>Violet</t>
@@ -1026,13 +1014,11 @@
       <c r="D6" t="n">
         <v>-186</v>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Violet</t>
@@ -1086,13 +1072,11 @@
       <c r="D7" t="n">
         <v>-426</v>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>Violet</t>
@@ -1146,13 +1130,11 @@
       <c r="D8" t="n">
         <v>-774</v>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Violet</t>
@@ -1206,13 +1188,11 @@
       <c r="D9" t="n">
         <v>-648</v>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>Violet</t>
@@ -1266,13 +1246,11 @@
       <c r="D10" t="n">
         <v>-33</v>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>Violet</t>
@@ -1326,13 +1304,11 @@
       <c r="D11" t="n">
         <v>-1153</v>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>Violet</t>
@@ -1386,13 +1362,11 @@
       <c r="D12" t="n">
         <v>-391</v>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>Blue</t>
@@ -1446,13 +1420,11 @@
       <c r="D13" t="n">
         <v>-1086</v>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>Blue</t>
@@ -1506,13 +1478,11 @@
       <c r="D14" t="n">
         <v>38</v>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>Blue</t>
@@ -1566,13 +1536,11 @@
       <c r="D15" t="n">
         <v>-552</v>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>Blue</t>
@@ -1626,13 +1594,11 @@
       <c r="D16" t="n">
         <v>559</v>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>Blue</t>
@@ -1686,13 +1652,11 @@
       <c r="D17" t="n">
         <v>-511</v>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>Inactive</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>Salmon</t>
@@ -1716,13 +1680,11 @@
       <c r="D18" t="n">
         <v>-310</v>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>Inactive</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>Salmon</t>
@@ -1746,13 +1708,11 @@
       <c r="D19" t="n">
         <v>-250</v>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>Inactive</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>Salmon</t>
@@ -1776,13 +1736,11 @@
       <c r="D20" t="n">
         <v>-52</v>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>Inactive</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>Salmon</t>
@@ -1806,13 +1764,11 @@
       <c r="D21" t="n">
         <v>674</v>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>Inactive</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>Salmon</t>
@@ -1836,13 +1792,11 @@
       <c r="D22" t="n">
         <v>653</v>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>Inactive</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>Salmon</t>
@@ -1932,8 +1886,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1962,8 +1914,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1992,8 +1942,6 @@
           <t>Inactive</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2083,7 +2031,6 @@
           <t>2025-12-15</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2168,8 +2115,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2198,8 +2143,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2228,8 +2171,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2314,8 +2255,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2344,8 +2283,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2374,8 +2311,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2565,4 +2500,414 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>DashSize</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>GapSize</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Outlet→Stack</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>450,-993;550,-855</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>#FF6600</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F2" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Stack→Tipping#1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>550,-855;579,-1020;750,-1020;1176,-1020</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>#FF6600</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F3" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Stack→Tipping#2</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>550,-855;579,-856;720,-1020;1176,-856</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>#FF6600</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>30</v>
+      </c>
+      <c r="F4" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Stack→Tipping#3</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>550,-855;579,-675;720,-1020;1176,-675</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>#FF6600</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F5" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Stack→Tipping#4</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>550,-855;579,-270;750,-1020;1176,-270</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>#FF6600</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>30</v>
+      </c>
+      <c r="F6" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Tipping#1→Blend</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1176,-1020;1220,-1020;1220,-578;1070,-578</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>#FF6600</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F7" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Tipping#2→Blend</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1176,-865;1216,-865;1216,-578;1070,-578</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>#FF6600</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F8" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Tipping#3→Blend</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1176,-675;1212,-675;1212,-578;1070,-578</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>#FF6600</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>30</v>
+      </c>
+      <c r="F9" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Tipping#4→Blend</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1176,-270;1210,-270;1210,-578;1070,-578</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>#FF6600</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>30</v>
+      </c>
+      <c r="F10" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PouchFiller#1→XRay#1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1380,-688;1559,-688</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>#FF6600</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>30</v>
+      </c>
+      <c r="F11" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PouchFiller#2→XRay#2</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1380,-554;1551,-554</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>#FF6600</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>30</v>
+      </c>
+      <c r="F12" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PouchFiller#3→XRay#3</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1380,-417;1520,-417;1568,-457</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>#FF6600</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>30</v>
+      </c>
+      <c r="F13" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>PouchFiller#4→XRay#4</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1380,-278;1586,-688</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>#FF6600</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F14" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CanFiller→Conveyor</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1203,-137;1386,-137</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>#FFCC00</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>30</v>
+      </c>
+      <c r="F15" t="n">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix flow animation via onBeforeRender hook; add Tension to Excel
Replace _flowMaterials loop with line.onBeforeRender, which Three.js
calls immediately before uploading uniforms for each object — guaranteeing
dashOffset is always current. Uses absolute time offset (no delta drift).

Tension column added to floor_1_data.xlsx flow sheet (default 0.3).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/floor_1_data.xlsx
+++ b/assets/floor_1_data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4140" yWindow="2265" windowWidth="21600" windowHeight="11295" tabRatio="600" firstSheet="0" activeTab="8" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="loc_name" sheetId="1" state="visible" r:id="rId1"/>
@@ -2508,8 +2508,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20.109375" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="38.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="8.33203125" bestFit="1" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2542,6 +2547,11 @@
           <t>GapSize</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2568,6 +2578,9 @@
       <c r="F2" t="n">
         <v>15</v>
       </c>
+      <c r="G2" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2594,6 +2607,9 @@
       <c r="F3" t="n">
         <v>15</v>
       </c>
+      <c r="G3" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2603,7 +2619,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>550,-855;579,-856;720,-1020;1176,-856</t>
+          <t>550,-855;579,-856;720,-865;1176,-856</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2620,6 +2636,9 @@
       <c r="F4" t="n">
         <v>15</v>
       </c>
+      <c r="G4" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2629,7 +2648,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>550,-855;579,-675;720,-1020;1176,-675</t>
+          <t>550,-855;579,-675;720,-675;1176,-675</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2646,6 +2665,9 @@
       <c r="F5" t="n">
         <v>15</v>
       </c>
+      <c r="G5" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2655,7 +2677,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>550,-855;579,-270;750,-1020;1176,-270</t>
+          <t>550,-855;579,-270;750,-270;1176,-270</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2672,6 +2694,9 @@
       <c r="F6" t="n">
         <v>15</v>
       </c>
+      <c r="G6" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2698,6 +2723,9 @@
       <c r="F7" t="n">
         <v>15</v>
       </c>
+      <c r="G7" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2724,6 +2752,9 @@
       <c r="F8" t="n">
         <v>15</v>
       </c>
+      <c r="G8" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2750,6 +2781,9 @@
       <c r="F9" t="n">
         <v>15</v>
       </c>
+      <c r="G9" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2776,6 +2810,9 @@
       <c r="F10" t="n">
         <v>15</v>
       </c>
+      <c r="G10" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2802,6 +2839,9 @@
       <c r="F11" t="n">
         <v>15</v>
       </c>
+      <c r="G11" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2828,6 +2868,9 @@
       <c r="F12" t="n">
         <v>15</v>
       </c>
+      <c r="G12" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2854,6 +2897,9 @@
       <c r="F13" t="n">
         <v>15</v>
       </c>
+      <c r="G13" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2863,7 +2909,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1380,-278;1586,-688</t>
+          <t>1380,-278;1586,-278</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2880,6 +2926,9 @@
       <c r="F14" t="n">
         <v>15</v>
       </c>
+      <c r="G14" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2905,6 +2954,9 @@
       </c>
       <c r="F15" t="n">
         <v>15</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix flow pause, scale pallet 1.5x, slow human walk speed
- Pause button: switch from early-return to frozen-time approach
  (_lastFlowT stores t when running; loop always executes with frozen t
  when paused, so pulses stay in place without skipping the position update)
- Pallet pulse: all geometry and positions scaled 1.5× for better visibility
- Human walk: speed multiplier 0.025 → 0.005 (0.2× of previous value)
- Also includes prior session: pulse shapes (pallet, human), path hover
  tooltip via invisible TubeGeometry hit mesh, ShowLine toggle, edge tint,
  zone corner format (X1/Y1/X2/Y2), layer grouping, settings panel,
  cross-floor flow support, pause button UI

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/floor_1_data.xlsx
+++ b/assets/floor_1_data.xlsx
@@ -8,20 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\M.Mead\9.FactoryView\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E952E23-ECC9-4388-86A9-A461D9B5CF1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67ACDF8D-E423-4E33-B015-EF822FB14D68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loc_name" sheetId="1" r:id="rId1"/>
     <sheet name="it_dev" sheetId="2" r:id="rId2"/>
-    <sheet name="dept_desk" sheetId="3" r:id="rId3"/>
-    <sheet name="pers_lap" sheetId="4" r:id="rId4"/>
-    <sheet name="weight" sheetId="5" r:id="rId5"/>
-    <sheet name="cam" sheetId="6" r:id="rId6"/>
-    <sheet name="paper" sheetId="7" r:id="rId7"/>
-    <sheet name="zones" sheetId="8" r:id="rId8"/>
-    <sheet name="flow" sheetId="9" r:id="rId9"/>
+    <sheet name="prod_comp" sheetId="4" r:id="rId3"/>
+    <sheet name="machine" sheetId="5" r:id="rId4"/>
+    <sheet name="inspect" sheetId="6" r:id="rId5"/>
+    <sheet name="paper" sheetId="8" r:id="rId6"/>
+    <sheet name="zones" sheetId="9" r:id="rId7"/>
+    <sheet name="flow" sheetId="10" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -38,7 +37,7 @@
     <author>User</author>
   </authors>
   <commentList>
-    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0800-000001000000}">
+    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0900-000001000000}">
       <text>
         <r>
           <rPr>
@@ -56,26 +55,17 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{7A046D8A-5163-4222-B23D-65813CE5672D}">
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0900-000002000000}">
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
+            <sz val="12"/>
+            <color theme="1"/>
             <rFont val="Tahoma"/>
-            <charset val="222"/>
+            <family val="2"/>
+            <scheme val="minor"/>
           </rPr>
-          <t>User:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="222"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>User:
 box, small_box, can, sack, powder</t>
         </r>
       </text>
@@ -85,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="221">
   <si>
     <t>Name</t>
   </si>
@@ -111,69 +101,36 @@
     <t>Color</t>
   </si>
   <si>
-    <t>Entrance Staff</t>
-  </si>
-  <si>
-    <t>Door</t>
-  </si>
-  <si>
-    <t>Main Staff Entrance</t>
+    <t>IP Address</t>
+  </si>
+  <si>
+    <t>MAC Address</t>
+  </si>
+  <si>
+    <t>Platform</t>
+  </si>
+  <si>
+    <t>Serial Number</t>
+  </si>
+  <si>
+    <t>Switch Detail</t>
+  </si>
+  <si>
+    <t>Port Details</t>
+  </si>
+  <si>
+    <t>AP-01</t>
+  </si>
+  <si>
+    <t>AP</t>
+  </si>
+  <si>
+    <t>Main entrance access point</t>
   </si>
   <si>
     <t>Active</t>
   </si>
   <si>
-    <t>Assembly Zone</t>
-  </si>
-  <si>
-    <t>Zone</t>
-  </si>
-  <si>
-    <t>Final Assembly Area</t>
-  </si>
-  <si>
-    <t>Manager Office</t>
-  </si>
-  <si>
-    <t>Room</t>
-  </si>
-  <si>
-    <t>Restricted Access</t>
-  </si>
-  <si>
-    <t>Loading Bay</t>
-  </si>
-  <si>
-    <t>Truck Loading Area</t>
-  </si>
-  <si>
-    <t>IP Address</t>
-  </si>
-  <si>
-    <t>MAC Address</t>
-  </si>
-  <si>
-    <t>Platform</t>
-  </si>
-  <si>
-    <t>Serial Number</t>
-  </si>
-  <si>
-    <t>Switch Detail</t>
-  </si>
-  <si>
-    <t>Port Details</t>
-  </si>
-  <si>
-    <t>AP-01</t>
-  </si>
-  <si>
-    <t>AP</t>
-  </si>
-  <si>
-    <t>Main entrance access point</t>
-  </si>
-  <si>
     <t>Orange</t>
   </si>
   <si>
@@ -444,82 +401,76 @@
     <t>AP06c</t>
   </si>
   <si>
-    <t>RND-Desk-01</t>
-  </si>
-  <si>
-    <t>R&amp;D</t>
-  </si>
-  <si>
-    <t>Senior Developer Desk</t>
-  </si>
-  <si>
-    <t>QA-Desk-05</t>
-  </si>
-  <si>
-    <t>QA</t>
-  </si>
-  <si>
-    <t>Test Station 5</t>
-  </si>
-  <si>
-    <t>PROD-Desk-11</t>
-  </si>
-  <si>
-    <t>Production</t>
-  </si>
-  <si>
-    <t>Production Line PC</t>
-  </si>
-  <si>
-    <t>LT</t>
-  </si>
-  <si>
-    <t>Standard</t>
-  </si>
-  <si>
     <t>Added via Editor</t>
   </si>
   <si>
     <t>2025-12-15</t>
   </si>
   <si>
-    <t>Vitamin A</t>
-  </si>
-  <si>
-    <t>Analog Scale</t>
-  </si>
-  <si>
-    <t>Vitamin B</t>
-  </si>
-  <si>
-    <t>Digital Scale</t>
-  </si>
-  <si>
-    <t>Vitamin C</t>
-  </si>
-  <si>
-    <t>CAM-Lobby-01</t>
-  </si>
-  <si>
-    <t>Dome</t>
-  </si>
-  <si>
-    <t>Covers main entrance</t>
-  </si>
-  <si>
-    <t>CAM-Exit-North</t>
-  </si>
-  <si>
-    <t>Bullet</t>
-  </si>
-  <si>
-    <t>Covers north emergency exit</t>
-  </si>
-  <si>
-    <t>CAM-Canteen-01</t>
-  </si>
-  <si>
-    <t>Monitors cafeteria seating area</t>
+    <t>Stripping #1</t>
+  </si>
+  <si>
+    <t>Machine</t>
+  </si>
+  <si>
+    <t>2026-04-13</t>
+  </si>
+  <si>
+    <t>Stripping #2</t>
+  </si>
+  <si>
+    <t>Stripping #4</t>
+  </si>
+  <si>
+    <t>Stripping #3</t>
+  </si>
+  <si>
+    <t>Tipping#1</t>
+  </si>
+  <si>
+    <t>Tipping#2</t>
+  </si>
+  <si>
+    <t>Tipping#3</t>
+  </si>
+  <si>
+    <t>Tipping#4</t>
+  </si>
+  <si>
+    <t>Blend-A</t>
+  </si>
+  <si>
+    <t>Blend-B</t>
+  </si>
+  <si>
+    <t>Blend-C</t>
+  </si>
+  <si>
+    <t>Blend-D</t>
+  </si>
+  <si>
+    <t>Filler#1</t>
+  </si>
+  <si>
+    <t>Filler#2</t>
+  </si>
+  <si>
+    <t>Filler#3</t>
+  </si>
+  <si>
+    <t>Filler#4</t>
+  </si>
+  <si>
+    <t>X-Ray</t>
+  </si>
+  <si>
+    <t>Inspect</t>
+  </si>
+  <si>
+    <t>i-Weight</t>
+  </si>
+  <si>
+    <t>Cam</t>
   </si>
   <si>
     <t>T.Slip</t>
@@ -531,19 +482,22 @@
     <t>Test Paper</t>
   </si>
   <si>
-    <t>Width</t>
-  </si>
-  <si>
-    <t>Height</t>
+    <t>X1</t>
+  </si>
+  <si>
+    <t>Y1</t>
+  </si>
+  <si>
+    <t>X2</t>
+  </si>
+  <si>
+    <t>Y2</t>
   </si>
   <si>
     <t>Opacity</t>
   </si>
   <si>
-    <t>BorderColor</t>
-  </si>
-  <si>
-    <t>BorderThickness</t>
+    <t>FontSize</t>
   </si>
   <si>
     <t>Production Zone</t>
@@ -552,7 +506,58 @@
     <t>#FF6600</t>
   </si>
   <si>
-    <t>Main production area</t>
+    <t>Blending and Tipping</t>
+  </si>
+  <si>
+    <t>Pouch Filler</t>
+  </si>
+  <si>
+    <t>Can Area</t>
+  </si>
+  <si>
+    <t>Pouch Packing</t>
+  </si>
+  <si>
+    <t>Can Packing</t>
+  </si>
+  <si>
+    <t>#d4c26a</t>
+  </si>
+  <si>
+    <t>Empty Can</t>
+  </si>
+  <si>
+    <t>#d4bb3f</t>
+  </si>
+  <si>
+    <t>Raw Mat Warehouse</t>
+  </si>
+  <si>
+    <t>#aa7ed6</t>
+  </si>
+  <si>
+    <t>Finish Goods Warehouse</t>
+  </si>
+  <si>
+    <t>#6d4794</t>
+  </si>
+  <si>
+    <t>Receiving</t>
+  </si>
+  <si>
+    <t>#553280</t>
+  </si>
+  <si>
+    <t>RTD</t>
+  </si>
+  <si>
+    <t>#db6978</t>
+  </si>
+  <si>
+    <t>QA Lab</t>
+  </si>
+  <si>
+    <t>#428a5b</t>
   </si>
   <si>
     <t>Points</t>
@@ -573,12 +578,21 @@
     <t>Shape</t>
   </si>
   <si>
+    <t>ShowLine</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
     <t>Outlet→Stack</t>
   </si>
   <si>
     <t>450,-993;550,-855</t>
   </si>
   <si>
+    <t>sack</t>
+  </si>
+  <si>
     <t>Stack→Tipping#1</t>
   </si>
   <si>
@@ -609,6 +623,9 @@
     <t>1176,-1020;1220,-1020;1220,-578;1070,-578</t>
   </si>
   <si>
+    <t>powder</t>
+  </si>
+  <si>
     <t>Tipping#2→Blend</t>
   </si>
   <si>
@@ -624,18 +641,60 @@
     <t>Tipping#4→Blend</t>
   </si>
   <si>
+    <t>1176,-270;1210,-270;1210,-578;1070,-578;1070,-578,150</t>
+  </si>
+  <si>
     <t>PouchFiller#1→XRay#1</t>
   </si>
   <si>
+    <t>1380,-688;1559,-688;2038,-684;2037,-755;1758,-759;1758,-835;2093,-832;2095,-942;1890,-945;1890,-1108;1329,-1108;1244,-1192;633,-1191;491,-1051;-336,-1052;-358,-1070;-418,-1066;-435,-1090;-411,-1110;-392,-1084;-433,-1066;-431,-1166;-293,-1166</t>
+  </si>
+  <si>
+    <t>#348ceb</t>
+  </si>
+  <si>
+    <t>small_box</t>
+  </si>
+  <si>
     <t>PouchFiller#2→XRay#2</t>
   </si>
   <si>
+    <t>1380,-554;1551,-554;1620,-557;1644,-578;2024,-570;2003,-526;1984,-550;2007,-573;2025,-547;2024,-423;1982,-444;2002,-467;2025,-448;2021,-272;1697,-275;1696,-228;2091,-229;2095,-941;1891,-946;1891,-1126;1335,-1126;1253,-1213;623,-1213;481,-1069;156,-1072;153,-1155;175,-1182;200,-1154;176,-1136;158,-1177;324,-1177</t>
+  </si>
+  <si>
+    <t>#396ca3</t>
+  </si>
+  <si>
     <t>PouchFiller#3→XRay#3</t>
   </si>
   <si>
+    <t>1380,-417;1520,-417;1568,-457;1604,-500;1642,-486;1645,-383;1797,-382;1797,-364;2002,-369;2022,-312;2021,-273;1698,-273;1700,-227;2090,-229;2094,-940;1891,-944;1890,-1108;1331,-1108;1244,-1189;631,-1193;485,-1050;138,-1047;122,-1070;-169,-1075;-175,-1148;-155,-1168;-130,-1147;-151,-1127;-174,-1169;-50,-1167</t>
+  </si>
+  <si>
+    <t>#77852c</t>
+  </si>
+  <si>
     <t>PouchFiller#4→XRay#4</t>
   </si>
   <si>
+    <t>1380,-278;1586,-278;1624,-277;1621,-156;2001,-153;2004,-92;1640,-98;1637,-51;2092,-51;2095,-941;1892,-944;1893,-1125;1337,-1126;1252,-1213;630,-1213;481,-1071;158,-1071;152,-1152;176,-1176;198,-1157;178,-1132;159,-1177;290,-1176</t>
+  </si>
+  <si>
+    <t>#89ad49</t>
+  </si>
+  <si>
+    <t>Pouch-&gt;Box</t>
+  </si>
+  <si>
+    <t>266,-1265;-946,-1270;-946,-1132</t>
+  </si>
+  <si>
+    <t>#7a522a</t>
+  </si>
+  <si>
+    <t>box</t>
+  </si>
+  <si>
     <t>CanFiller→Conveyor</t>
   </si>
   <si>
@@ -645,50 +704,47 @@
     <t>#FFCC00</t>
   </si>
   <si>
-    <t>sack</t>
-  </si>
-  <si>
-    <t>powder</t>
-  </si>
-  <si>
-    <t>small_box</t>
-  </si>
-  <si>
     <t>can</t>
   </si>
   <si>
-    <t>1176,-270;1210,-270;1210,-578;1070,-578;1070,-578,150</t>
-  </si>
-  <si>
-    <t>1380,-688;1559,-688;2038,-684;2037,-755;1758,-759;1758,-835;2093,-832;2095,-942;1890,-945;1890,-1108;1329,-1108;1244,-1192;633,-1191;491,-1051;-336,-1052;-358,-1070;-418,-1066;-435,-1090;-411,-1110;-392,-1084;-433,-1066;-431,-1166;-293,-1166</t>
-  </si>
-  <si>
-    <t>#348ceb</t>
-  </si>
-  <si>
-    <t>1380,-554;1551,-554;1620,-557;1644,-578;2024,-570;2003,-526;1984,-550;2007,-573;2025,-547;2024,-423;1982,-444;2002,-467;2025,-448;2021,-272;1697,-275;1696,-228;2091,-229;2095,-941;1891,-946;1891,-1126;1335,-1126;1253,-1213;623,-1213;481,-1069;156,-1072;153,-1155;175,-1182;200,-1154;176,-1136;158,-1177;324,-1177</t>
-  </si>
-  <si>
-    <t>#396ca3</t>
-  </si>
-  <si>
-    <t>1380,-417;1520,-417;1568,-457;1604,-500;1642,-486;1645,-383;1797,-382;1797,-364;2002,-369;2022,-312;2021,-273;1698,-273;1700,-227;2090,-229;2094,-940;1891,-944;1890,-1108;1331,-1108;1244,-1189;631,-1193;485,-1050;138,-1047;122,-1070;-169,-1075;-175,-1148;-155,-1168;-130,-1147;-151,-1127;-174,-1169;-50,-1167</t>
-  </si>
-  <si>
-    <t>#77852c</t>
-  </si>
-  <si>
-    <t>1380,-278;1586,-278;1624,-277;1621,-156;2001,-153;2004,-92;1640,-98;1637,-51;2092,-51;2095,-941;1892,-944;1893,-1125;1337,-1126;1252,-1213;630,-1213;481,-1071;158,-1071;152,-1152;176,-1176;198,-1157;178,-1132;159,-1177;290,-1176</t>
-  </si>
-  <si>
-    <t>#89ad49</t>
+    <t>Empty Can Input</t>
+  </si>
+  <si>
+    <t>601,198;603,255;654,256;651,-129;1095,-133;1094,-58;1115,-58;1112,-132;1203,-137</t>
+  </si>
+  <si>
+    <t>#766f6b</t>
+  </si>
+  <si>
+    <t>GWINS</t>
+  </si>
+  <si>
+    <t>gwins</t>
+  </si>
+  <si>
+    <t>-722,-1085;-1348,-1085</t>
+  </si>
+  <si>
+    <t>pallet</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Palette-&gt;Out</t>
+  </si>
+  <si>
+    <t>Empty Can -&gt; In</t>
+  </si>
+  <si>
+    <t>238,187;609,187</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -697,17 +753,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="222"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="222"/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="FkGroteskNeue"/>
     </font>
   </fonts>
   <fills count="5">
@@ -736,7 +784,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -759,11 +807,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -775,6 +834,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1114,10 +1176,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1141,86 +1207,6 @@
       </c>
       <c r="H1" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2">
-        <v>-550</v>
-      </c>
-      <c r="D2">
-        <v>-200</v>
-      </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3">
-        <v>200</v>
-      </c>
-      <c r="D3">
-        <v>100</v>
-      </c>
-      <c r="E3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4">
-        <v>800</v>
-      </c>
-      <c r="D4">
-        <v>-400</v>
-      </c>
-      <c r="E4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5">
-        <v>-400</v>
-      </c>
-      <c r="D5">
-        <v>400</v>
-      </c>
-      <c r="E5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1231,7 +1217,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:N22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="5" max="5" width="19.88671875" customWidth="1"/>
     <col min="9" max="9" width="12.6640625" bestFit="1" customWidth="1"/>
@@ -1242,7 +1228,7 @@
     <col min="14" max="14" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1268,30 +1254,30 @@
         <v>7</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C2">
         <v>-1293</v>
@@ -1300,42 +1286,42 @@
         <v>519</v>
       </c>
       <c r="E2" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="F2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G2" s="1">
         <v>44927</v>
       </c>
       <c r="H2" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="N2" s="6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C3">
         <v>-614</v>
@@ -1344,39 +1330,39 @@
         <v>71</v>
       </c>
       <c r="E3" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="F3" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L3" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="I3" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>40</v>
-      </c>
       <c r="M3" s="5" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C4">
         <v>-339</v>
@@ -1385,36 +1371,36 @@
         <v>-1235</v>
       </c>
       <c r="F4" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H4" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C5">
         <v>587</v>
@@ -1423,36 +1409,36 @@
         <v>-1129</v>
       </c>
       <c r="F5" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H5" t="s">
+        <v>32</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" t="s">
         <v>43</v>
       </c>
-      <c r="I5" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="M5" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="N5" s="6" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>54</v>
-      </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C6">
         <v>558</v>
@@ -1461,36 +1447,36 @@
         <v>-186</v>
       </c>
       <c r="F6" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H6" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="M6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="N6" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="N6" s="6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:14">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C7">
         <v>1002</v>
@@ -1499,36 +1485,36 @@
         <v>-426</v>
       </c>
       <c r="F7" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H7" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="N7" s="6" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
       <c r="A8" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C8">
         <v>995</v>
@@ -1537,36 +1523,36 @@
         <v>-774</v>
       </c>
       <c r="F8" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H8" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="M8" s="5" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="N8" s="6" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C9">
         <v>1268</v>
@@ -1575,36 +1561,36 @@
         <v>-648</v>
       </c>
       <c r="F9" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H9" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="M9" s="5" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
       <c r="A10" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C10">
         <v>1252</v>
@@ -1613,36 +1599,36 @@
         <v>-33</v>
       </c>
       <c r="F10" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H10" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="L10" s="4" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="N10" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
       <c r="A11" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C11">
         <v>1545</v>
@@ -1651,36 +1637,36 @@
         <v>-1153</v>
       </c>
       <c r="F11" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H11" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
       <c r="A12" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C12">
         <v>2102</v>
@@ -1689,36 +1675,36 @@
         <v>-391</v>
       </c>
       <c r="F12" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H12" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
       <c r="A13" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C13">
         <v>2003</v>
@@ -1727,36 +1713,36 @@
         <v>-1086</v>
       </c>
       <c r="F13" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H13" t="s">
+        <v>74</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="M13" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="N13" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14" t="s">
         <v>85</v>
       </c>
-      <c r="I13" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="K13" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="L13" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="M13" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="N13" s="6" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>96</v>
-      </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C14">
         <v>2309</v>
@@ -1765,36 +1751,36 @@
         <v>38</v>
       </c>
       <c r="F14" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H14" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="M14" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="N14" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="N14" s="6" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="1:14">
       <c r="A15" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C15">
         <v>2347</v>
@@ -1803,36 +1789,36 @@
         <v>-552</v>
       </c>
       <c r="F15" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H15" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="L15" s="4" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="N15" s="6" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
       <c r="A16" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C16">
         <v>2645</v>
@@ -1841,36 +1827,36 @@
         <v>559</v>
       </c>
       <c r="F16" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H16" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="L16" s="4" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="B17" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C17">
         <v>-2111</v>
@@ -1879,18 +1865,18 @@
         <v>-511</v>
       </c>
       <c r="F17" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="H17" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="B18" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C18">
         <v>-2407</v>
@@ -1899,18 +1885,18 @@
         <v>-310</v>
       </c>
       <c r="F18" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="H18" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="B19" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C19">
         <v>-1884</v>
@@ -1919,18 +1905,18 @@
         <v>-250</v>
       </c>
       <c r="F19" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="H19" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="B20" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C20">
         <v>-2019</v>
@@ -1939,18 +1925,18 @@
         <v>-52</v>
       </c>
       <c r="F20" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="H20" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="B21" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C21">
         <v>-2394</v>
@@ -1959,18 +1945,18 @@
         <v>674</v>
       </c>
       <c r="F21" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="H21" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="B22" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C22">
         <v>-1925</v>
@@ -1979,10 +1965,10 @@
         <v>653</v>
       </c>
       <c r="F22" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="H22" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -1991,11 +1977,14 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="7" max="7" width="10.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2021,64 +2010,27 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B2" t="s">
-        <v>120</v>
+        <v>214</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>213</v>
       </c>
       <c r="C2">
-        <v>-450</v>
+        <v>-336</v>
       </c>
       <c r="D2">
-        <v>-200</v>
+        <v>-446</v>
       </c>
       <c r="E2" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>122</v>
-      </c>
-      <c r="B3" t="s">
-        <v>123</v>
-      </c>
-      <c r="C3">
-        <v>150</v>
-      </c>
-      <c r="D3">
-        <v>-600</v>
-      </c>
-      <c r="E3" t="s">
-        <v>124</v>
-      </c>
-      <c r="F3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>125</v>
-      </c>
-      <c r="B4" t="s">
-        <v>126</v>
-      </c>
-      <c r="C4">
-        <v>800</v>
-      </c>
-      <c r="D4">
-        <v>250</v>
-      </c>
-      <c r="E4" t="s">
-        <v>127</v>
-      </c>
-      <c r="F4" t="s">
-        <v>112</v>
+        <v>17</v>
+      </c>
+      <c r="G2" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -2087,11 +2039,16 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.109375" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2117,27 +2074,336 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="B2" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="C2">
-        <v>-336</v>
+        <v>793</v>
       </c>
       <c r="D2">
-        <v>-446</v>
+        <v>-1020</v>
       </c>
       <c r="E2" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="F2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G2" t="s">
-        <v>131</v>
+        <v>112</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3">
+        <v>763</v>
+      </c>
+      <c r="D3">
+        <v>-854</v>
+      </c>
+      <c r="E3" t="s">
+        <v>108</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C4">
+        <v>773</v>
+      </c>
+      <c r="D4">
+        <v>-675</v>
+      </c>
+      <c r="E4" t="s">
+        <v>108</v>
+      </c>
+      <c r="F4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C5">
+        <v>800</v>
+      </c>
+      <c r="D5">
+        <v>-270</v>
+      </c>
+      <c r="E5" t="s">
+        <v>108</v>
+      </c>
+      <c r="F5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
+        <v>116</v>
+      </c>
+      <c r="B6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C6">
+        <v>1157</v>
+      </c>
+      <c r="D6">
+        <v>-1020</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
+        <v>117</v>
+      </c>
+      <c r="B7" t="s">
+        <v>111</v>
+      </c>
+      <c r="C7">
+        <v>1157</v>
+      </c>
+      <c r="D7">
+        <v>-854</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
+        <v>118</v>
+      </c>
+      <c r="B8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C8">
+        <v>1157</v>
+      </c>
+      <c r="D8">
+        <v>-675</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B9" t="s">
+        <v>111</v>
+      </c>
+      <c r="C9">
+        <v>1157</v>
+      </c>
+      <c r="D9">
+        <v>-270</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
+        <v>120</v>
+      </c>
+      <c r="B10" t="s">
+        <v>111</v>
+      </c>
+      <c r="C10">
+        <v>1019</v>
+      </c>
+      <c r="D10">
+        <v>-504</v>
+      </c>
+      <c r="E10" t="s">
+        <v>108</v>
+      </c>
+      <c r="F10" t="s">
+        <v>17</v>
+      </c>
+      <c r="G10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
+        <v>121</v>
+      </c>
+      <c r="B11" t="s">
+        <v>111</v>
+      </c>
+      <c r="C11">
+        <v>914</v>
+      </c>
+      <c r="D11">
+        <v>-504</v>
+      </c>
+      <c r="E11" t="s">
+        <v>108</v>
+      </c>
+      <c r="F11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" t="s">
+        <v>122</v>
+      </c>
+      <c r="B12" t="s">
+        <v>111</v>
+      </c>
+      <c r="C12">
+        <v>798</v>
+      </c>
+      <c r="D12">
+        <v>-504</v>
+      </c>
+      <c r="E12" t="s">
+        <v>108</v>
+      </c>
+      <c r="F12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" t="s">
+        <v>123</v>
+      </c>
+      <c r="B13" t="s">
+        <v>111</v>
+      </c>
+      <c r="C13">
+        <v>653</v>
+      </c>
+      <c r="D13">
+        <v>-501</v>
+      </c>
+      <c r="E13" t="s">
+        <v>108</v>
+      </c>
+      <c r="F13" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" t="s">
+        <v>124</v>
+      </c>
+      <c r="B14" t="s">
+        <v>111</v>
+      </c>
+      <c r="C14">
+        <v>1354</v>
+      </c>
+      <c r="D14">
+        <v>-688</v>
+      </c>
+      <c r="E14" t="s">
+        <v>108</v>
+      </c>
+      <c r="F14" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" t="s">
+        <v>125</v>
+      </c>
+      <c r="B15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C15">
+        <v>1354</v>
+      </c>
+      <c r="D15">
+        <v>-553</v>
+      </c>
+      <c r="E15" t="s">
+        <v>108</v>
+      </c>
+      <c r="F15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G15" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" t="s">
+        <v>126</v>
+      </c>
+      <c r="B16" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16">
+        <v>1354</v>
+      </c>
+      <c r="D16">
+        <v>-420</v>
+      </c>
+      <c r="E16" t="s">
+        <v>108</v>
+      </c>
+      <c r="F16" t="s">
+        <v>17</v>
+      </c>
+      <c r="G16" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>127</v>
+      </c>
+      <c r="B17" t="s">
+        <v>111</v>
+      </c>
+      <c r="C17">
+        <v>1354</v>
+      </c>
+      <c r="D17">
+        <v>-279</v>
+      </c>
+      <c r="E17" t="s">
+        <v>108</v>
+      </c>
+      <c r="F17" t="s">
+        <v>17</v>
+      </c>
+      <c r="G17" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -2146,11 +2412,11 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2176,64 +2442,172 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C2">
-        <v>1280</v>
+        <v>1560</v>
       </c>
       <c r="D2">
-        <v>-343</v>
-      </c>
-      <c r="E2" t="s">
+        <v>-691</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C3">
+        <v>1552</v>
+      </c>
+      <c r="D3">
+        <v>-560</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B4" t="s">
+        <v>129</v>
+      </c>
+      <c r="C4">
+        <v>1567</v>
+      </c>
+      <c r="D4">
+        <v>-456</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>128</v>
+      </c>
+      <c r="B5" t="s">
+        <v>129</v>
+      </c>
+      <c r="C5">
+        <v>1587</v>
+      </c>
+      <c r="D5">
+        <v>-280</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
         <v>130</v>
       </c>
-      <c r="F2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>134</v>
-      </c>
-      <c r="B3" t="s">
-        <v>135</v>
-      </c>
-      <c r="C3">
-        <v>1289</v>
-      </c>
-      <c r="D3">
-        <v>-243</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="B6" t="s">
+        <v>129</v>
+      </c>
+      <c r="C6">
+        <v>1498</v>
+      </c>
+      <c r="D6">
+        <v>-689</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
         <v>130</v>
       </c>
-      <c r="F3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>136</v>
-      </c>
-      <c r="B4" t="s">
-        <v>135</v>
-      </c>
-      <c r="C4">
-        <v>1349</v>
-      </c>
-      <c r="D4">
-        <v>-130</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="B7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C7">
+        <v>1498</v>
+      </c>
+      <c r="D7">
+        <v>-556</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
         <v>130</v>
       </c>
-      <c r="F4" t="s">
-        <v>11</v>
+      <c r="B8" t="s">
+        <v>129</v>
+      </c>
+      <c r="C8">
+        <v>1498</v>
+      </c>
+      <c r="D8">
+        <v>-419</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>131</v>
+      </c>
+      <c r="B9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C9">
+        <v>1965</v>
+      </c>
+      <c r="D9">
+        <v>-770</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
+        <v>131</v>
+      </c>
+      <c r="B10" t="s">
+        <v>129</v>
+      </c>
+      <c r="C10">
+        <v>1777</v>
+      </c>
+      <c r="D10">
+        <v>-292</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
+        <v>131</v>
+      </c>
+      <c r="B11" t="s">
+        <v>129</v>
+      </c>
+      <c r="C11">
+        <v>1757</v>
+      </c>
+      <c r="D11">
+        <v>-117</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" t="s">
+        <v>128</v>
+      </c>
+      <c r="B12" t="s">
+        <v>129</v>
+      </c>
+      <c r="C12">
+        <v>799</v>
+      </c>
+      <c r="D12">
+        <v>-50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" t="s">
+        <v>131</v>
+      </c>
+      <c r="B13" t="s">
+        <v>129</v>
+      </c>
+      <c r="C13">
+        <v>1393</v>
+      </c>
+      <c r="D13">
+        <v>-51</v>
       </c>
     </row>
   </sheetData>
@@ -2242,11 +2616,11 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2272,64 +2646,21 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C2">
-        <v>-900</v>
+        <v>-450</v>
       </c>
       <c r="D2">
-        <v>1250</v>
+        <v>-220</v>
       </c>
       <c r="E2" t="s">
-        <v>139</v>
-      </c>
-      <c r="F2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>140</v>
-      </c>
-      <c r="B3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>-1400</v>
-      </c>
-      <c r="E3" t="s">
-        <v>142</v>
-      </c>
-      <c r="F3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>143</v>
-      </c>
-      <c r="B4" t="s">
-        <v>138</v>
-      </c>
-      <c r="C4">
-        <v>600</v>
-      </c>
-      <c r="D4">
-        <v>850</v>
-      </c>
-      <c r="E4" t="s">
-        <v>144</v>
-      </c>
-      <c r="F4" t="s">
-        <v>11</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -2338,125 +2669,354 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="21.44140625" customWidth="1"/>
+    <col min="8" max="8" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.5546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>135</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>136</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>137</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>145</v>
-      </c>
-      <c r="B2" t="s">
-        <v>146</v>
-      </c>
-      <c r="C2">
-        <v>-450</v>
-      </c>
-      <c r="D2">
-        <v>-220</v>
-      </c>
-      <c r="E2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:J2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" t="s">
-        <v>148</v>
-      </c>
-      <c r="E1" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="F1" t="s">
         <v>7</v>
       </c>
       <c r="G1" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
       <c r="H1" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="I1" t="s">
-        <v>152</v>
-      </c>
-      <c r="J1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>589</v>
       </c>
       <c r="C2">
-        <v>-100</v>
+        <v>-1104</v>
       </c>
       <c r="D2">
-        <v>1400</v>
+        <v>1229</v>
       </c>
       <c r="E2">
-        <v>700</v>
+        <v>-190</v>
       </c>
       <c r="F2" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="G2">
         <v>0.2</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2">
+        <v>14</v>
+      </c>
+      <c r="I2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="B3">
+        <v>1229</v>
+      </c>
+      <c r="C3">
+        <v>-759</v>
+      </c>
+      <c r="D3">
+        <v>1511</v>
+      </c>
+      <c r="E3">
+        <v>-190</v>
+      </c>
+      <c r="F3" t="s">
+        <v>142</v>
+      </c>
+      <c r="G3">
+        <v>0.2</v>
+      </c>
+      <c r="H3">
+        <v>14</v>
+      </c>
+      <c r="I3" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="B4">
+        <v>217</v>
+      </c>
+      <c r="C4">
+        <v>-190</v>
+      </c>
+      <c r="D4">
+        <v>1585</v>
+      </c>
+      <c r="E4">
+        <v>-5</v>
+      </c>
+      <c r="F4" t="s">
+        <v>142</v>
+      </c>
+      <c r="G4">
+        <v>0.2</v>
+      </c>
+      <c r="H4">
+        <v>14</v>
+      </c>
+      <c r="I4" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>146</v>
+      </c>
+      <c r="B5">
+        <v>-1374</v>
+      </c>
+      <c r="C5">
+        <v>-1303</v>
+      </c>
+      <c r="D5">
+        <v>452</v>
+      </c>
+      <c r="E5">
+        <v>-971</v>
+      </c>
+      <c r="F5" t="s">
+        <v>142</v>
+      </c>
+      <c r="G5">
+        <v>0.2</v>
+      </c>
+      <c r="H5">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>147</v>
+      </c>
+      <c r="B6">
+        <v>-173</v>
+      </c>
+      <c r="C6">
+        <v>-193</v>
+      </c>
+      <c r="D6">
+        <v>216</v>
+      </c>
+      <c r="E6">
+        <v>-5</v>
+      </c>
+      <c r="F6" t="s">
+        <v>148</v>
+      </c>
+      <c r="G6">
+        <v>0.2</v>
+      </c>
+      <c r="H6">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>149</v>
+      </c>
+      <c r="B7">
+        <v>173</v>
+      </c>
+      <c r="C7">
+        <v>-5</v>
+      </c>
+      <c r="D7">
+        <v>726</v>
+      </c>
+      <c r="E7">
+        <v>320</v>
+      </c>
+      <c r="F7" t="s">
+        <v>150</v>
+      </c>
+      <c r="G7">
+        <v>0.2</v>
+      </c>
+      <c r="H7">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>151</v>
+      </c>
+      <c r="B8">
+        <v>-468</v>
+      </c>
+      <c r="C8">
+        <v>-971</v>
+      </c>
+      <c r="D8">
+        <v>591</v>
+      </c>
+      <c r="E8">
+        <v>-190</v>
+      </c>
+      <c r="F8" t="s">
+        <v>152</v>
+      </c>
+      <c r="G8">
+        <v>0.2</v>
+      </c>
+      <c r="H8">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>153</v>
+      </c>
+      <c r="B9">
+        <v>-1540</v>
+      </c>
+      <c r="C9">
+        <v>-971</v>
+      </c>
+      <c r="D9">
+        <v>-468</v>
+      </c>
+      <c r="E9">
+        <v>-190</v>
+      </c>
+      <c r="F9" t="s">
         <v>154</v>
       </c>
-      <c r="I2">
-        <v>15</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="G9">
+        <v>0.2</v>
+      </c>
+      <c r="H9">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
         <v>155</v>
+      </c>
+      <c r="B10">
+        <v>-206</v>
+      </c>
+      <c r="C10">
+        <v>-8</v>
+      </c>
+      <c r="D10">
+        <v>119</v>
+      </c>
+      <c r="E10">
+        <v>728</v>
+      </c>
+      <c r="F10" t="s">
+        <v>156</v>
+      </c>
+      <c r="G10">
+        <v>0.2</v>
+      </c>
+      <c r="H10">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="B11">
+        <v>119</v>
+      </c>
+      <c r="C11">
+        <v>488</v>
+      </c>
+      <c r="D11">
+        <v>535</v>
+      </c>
+      <c r="E11">
+        <v>728</v>
+      </c>
+      <c r="F11" t="s">
+        <v>156</v>
+      </c>
+      <c r="G11">
+        <v>0.2</v>
+      </c>
+      <c r="H11">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" t="s">
+        <v>157</v>
+      </c>
+      <c r="B12">
+        <v>-2703</v>
+      </c>
+      <c r="C12">
+        <v>-584</v>
+      </c>
+      <c r="D12">
+        <v>-1785</v>
+      </c>
+      <c r="E12">
+        <v>1308</v>
+      </c>
+      <c r="F12" t="s">
+        <v>158</v>
+      </c>
+      <c r="G12">
+        <v>0.2</v>
+      </c>
+      <c r="H12">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" t="s">
+        <v>159</v>
+      </c>
+      <c r="B13">
+        <v>2121</v>
+      </c>
+      <c r="C13">
+        <v>-1169</v>
+      </c>
+      <c r="D13">
+        <v>2645</v>
+      </c>
+      <c r="E13">
+        <v>6</v>
+      </c>
+      <c r="F13" t="s">
+        <v>160</v>
+      </c>
+      <c r="G13">
+        <v>0.2</v>
+      </c>
+      <c r="H13">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -2464,51 +3024,57 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:J19"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="219.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C1" t="s">
         <v>7</v>
       </c>
       <c r="D1" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="E1" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F1" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="G1" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="H1" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+        <v>166</v>
+      </c>
+      <c r="I1" t="s">
+        <v>167</v>
+      </c>
+      <c r="J1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="B2" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C2" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -2523,18 +3089,21 @@
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+        <v>171</v>
+      </c>
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="B3" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="C3" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -2549,18 +3118,21 @@
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+        <v>171</v>
+      </c>
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="B4" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="C4" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -2575,18 +3147,21 @@
         <v>0</v>
       </c>
       <c r="H4" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+        <v>171</v>
+      </c>
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="B5" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="C5" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -2601,18 +3176,21 @@
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+        <v>171</v>
+      </c>
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="B6" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="C6" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -2627,18 +3205,21 @@
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+        <v>171</v>
+      </c>
+      <c r="I6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="B7" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="C7" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -2653,18 +3234,21 @@
         <v>0</v>
       </c>
       <c r="H7" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+        <v>182</v>
+      </c>
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="B8" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="C8" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -2679,18 +3263,21 @@
         <v>0</v>
       </c>
       <c r="H8" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+        <v>182</v>
+      </c>
+      <c r="I8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="B9" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="C9" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -2705,18 +3292,21 @@
         <v>0</v>
       </c>
       <c r="H9" t="s">
+        <v>182</v>
+      </c>
+      <c r="I9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>178</v>
-      </c>
       <c r="B10" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C10" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -2731,18 +3321,21 @@
         <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+        <v>182</v>
+      </c>
+      <c r="I10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="B11" t="s">
+        <v>190</v>
+      </c>
+      <c r="C11" t="s">
         <v>191</v>
-      </c>
-      <c r="C11" t="s">
-        <v>192</v>
       </c>
       <c r="D11">
         <v>0.5</v>
@@ -2757,18 +3350,21 @@
         <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="I11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="B12" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C12" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D12">
         <v>0.3</v>
@@ -2783,18 +3379,21 @@
         <v>0</v>
       </c>
       <c r="H12" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="I12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
       <c r="B13" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C13" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D13">
         <v>0.2</v>
@@ -2809,18 +3408,21 @@
         <v>0</v>
       </c>
       <c r="H13" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="I13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>182</v>
+        <v>199</v>
       </c>
       <c r="B14" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="C14" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D14">
         <v>0.3</v>
@@ -2835,18 +3437,21 @@
         <v>0</v>
       </c>
       <c r="H14" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="I14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="B15" t="s">
-        <v>184</v>
+        <v>203</v>
       </c>
       <c r="C15" t="s">
-        <v>185</v>
+        <v>204</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -2861,7 +3466,132 @@
         <v>0</v>
       </c>
       <c r="H15" t="s">
-        <v>189</v>
+        <v>205</v>
+      </c>
+      <c r="I15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="A16" t="s">
+        <v>206</v>
+      </c>
+      <c r="B16" t="s">
+        <v>207</v>
+      </c>
+      <c r="C16" t="s">
+        <v>208</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>30</v>
+      </c>
+      <c r="F16">
+        <v>15</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16" t="s">
+        <v>209</v>
+      </c>
+      <c r="I16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10">
+      <c r="A17" t="s">
+        <v>210</v>
+      </c>
+      <c r="B17" t="s">
+        <v>211</v>
+      </c>
+      <c r="C17" t="s">
+        <v>212</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>30</v>
+      </c>
+      <c r="F17">
+        <v>15</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17" t="s">
+        <v>209</v>
+      </c>
+      <c r="I17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10">
+      <c r="A18" t="s">
+        <v>218</v>
+      </c>
+      <c r="B18" t="s">
+        <v>215</v>
+      </c>
+      <c r="C18" t="s">
+        <v>204</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18">
+        <v>30</v>
+      </c>
+      <c r="F18">
+        <v>15</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18" t="s">
+        <v>216</v>
+      </c>
+      <c r="I18" t="b">
+        <v>1</v>
+      </c>
+      <c r="J18" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10">
+      <c r="A19" t="s">
+        <v>219</v>
+      </c>
+      <c r="B19" t="s">
+        <v>220</v>
+      </c>
+      <c r="C19" t="s">
+        <v>212</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19">
+        <v>30</v>
+      </c>
+      <c r="F19">
+        <v>15</v>
+      </c>
+      <c r="G19">
+        <v>0.5</v>
+      </c>
+      <c r="H19" t="s">
+        <v>216</v>
+      </c>
+      <c r="I19" t="b">
+        <v>1</v>
+      </c>
+      <c r="J19" t="s">
+        <v>217</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UI polish: icon buttons, collapsible panels, expanded settings
- Left panel: replace All/None with Collapse All/Expand All group controls
- View Controls: compact icon buttons (⊙ ⏸ Aa) with tooltips; remove keyboard hint
- Right panel: collapsible with slide tab, mirrors left panel behaviour
- Settings: add Pause Flow on startup, Hide Labels on startup, floor separation distance
- CSS: add right-panel collapse rules; remove duplicate left-panel block
- FlowDrawer: layer dropdown populated from all flow-type layers
- Multiple flow layer support via system_config.xlsx

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/floor_1_data.xlsx
+++ b/assets/floor_1_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\M.Mead\9.FactoryView\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24607A47-283D-483C-8B16-4771D81F70D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{543A5AD1-9570-45C9-B6CC-9084DEFC06BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loc_name" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,9 @@
     <sheet name="inspect" sheetId="6" r:id="rId5"/>
     <sheet name="paper" sheetId="8" r:id="rId6"/>
     <sheet name="zones" sheetId="9" r:id="rId7"/>
-    <sheet name="flow" sheetId="10" r:id="rId8"/>
+    <sheet name="flow_pouch" sheetId="10" r:id="rId8"/>
+    <sheet name="flow_can" sheetId="12" r:id="rId9"/>
+    <sheet name="flow_rtd" sheetId="11" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -83,8 +85,94 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>User</author>
+  </authors>
+  <commentList>
+    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{FE8679F7-6CB3-41F3-ABA6-B528A83800BD}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color theme="1"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>User:
+Add Tension column to the flow sheet (0 to 1, default 0.5)
+0.0 = very round curves at corners (more organic)
+0.5 = balanced (default)
+1.0 = nearly straight lines between waypoints</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{3E9FBAE6-BF22-4840-97D8-0BC1E6C52CB8}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color theme="1"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>User:
+box, small_box, can, sack, powder</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>User</author>
+  </authors>
+  <commentList>
+    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{054815E8-2F7F-4F3E-ADFD-69179D5EA69A}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color theme="1"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>User:
+Add Tension column to the flow sheet (0 to 1, default 0.5)
+0.0 = very round curves at corners (more organic)
+0.5 = balanced (default)
+1.0 = nearly straight lines between waypoints</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{CD43AF9B-1A28-4684-B2BC-DA754D88B431}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="12"/>
+            <color theme="1"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>User:
+box, small_box, can, sack, powder</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="254">
   <si>
     <t>Name</t>
   </si>
@@ -716,18 +804,6 @@
     <t>#552fb5</t>
   </si>
   <si>
-    <t>powder1-&gt;foil1</t>
-  </si>
-  <si>
-    <t>powder2-&gt;foil2</t>
-  </si>
-  <si>
-    <t>powder3-&gt;foil3</t>
-  </si>
-  <si>
-    <t>powder4-&gt;foil4</t>
-  </si>
-  <si>
     <t>1737,-688;2038,-684;2037,-755;1758,-759;1758,-835;2093,-832;2095,-942;1890,-945;1890,-1108;1329,-1108;1244,-1192;633,-1191;491,-1051;-336,-1052;-358,-1070;-418,-1066;-435,-1090;-411,-1110;-392,-1084;-433,-1066;-431,-1166;-293,-1166</t>
   </si>
   <si>
@@ -819,6 +895,45 @@
   </si>
   <si>
     <t>#ff6600</t>
+  </si>
+  <si>
+    <t>-2047,831;-2046,979;-2153,979;-2155,1015;-2022,1017;-2023,1273;-2183,1271;-2183,998;-2561,998;-2561,984;-2183,983;-2182,866;-2269,865</t>
+  </si>
+  <si>
+    <t>#4b7cdd</t>
+  </si>
+  <si>
+    <t>Rtd-&gt;FinishGoods</t>
+  </si>
+  <si>
+    <t>-2351,874;-2473,871;-2471,742;-2464,565;-2456,452;-2456,237;-2480,210;-2480,173;-2464,155;-2422,155;-2407,174;-2407,244;-2402,272;-2400,402;-2416,424;-2461,423;-2475,405;-2474,342;-2481,327;-2480,235;-2451,201;-2452,139;-2446,85</t>
+  </si>
+  <si>
+    <t>#00aaff</t>
+  </si>
+  <si>
+    <t>Rtd-&gt;FinishGoodsBox</t>
+  </si>
+  <si>
+    <t>-2446,58;-2443,-166;-2496,-166</t>
+  </si>
+  <si>
+    <t>#ea9e48</t>
+  </si>
+  <si>
+    <t>Rtd-&gt;Fill</t>
+  </si>
+  <si>
+    <t>Sifter1-&gt;foil1</t>
+  </si>
+  <si>
+    <t>Sifter2-&gt;foil2</t>
+  </si>
+  <si>
+    <t>Sifter3-&gt;foil3</t>
+  </si>
+  <si>
+    <t>Sifter4-&gt;foil4</t>
   </si>
 </sst>
 </file>
@@ -909,7 +1024,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -924,6 +1039,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1301,6 +1417,140 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0ACF53D-E42F-4800-86E8-DC392D89187D}">
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18.33203125" customWidth="1"/>
+    <col min="2" max="2" width="54.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E1" t="s">
+        <v>159</v>
+      </c>
+      <c r="F1" t="s">
+        <v>160</v>
+      </c>
+      <c r="G1" t="s">
+        <v>161</v>
+      </c>
+      <c r="H1" t="s">
+        <v>162</v>
+      </c>
+      <c r="I1" t="s">
+        <v>163</v>
+      </c>
+      <c r="J1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="D2" s="8">
+        <v>1</v>
+      </c>
+      <c r="E2" s="8">
+        <v>30</v>
+      </c>
+      <c r="F2" s="8">
+        <v>15</v>
+      </c>
+      <c r="G2" s="8">
+        <v>0</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="I2" s="8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" t="s">
+        <v>243</v>
+      </c>
+      <c r="B3" t="s">
+        <v>244</v>
+      </c>
+      <c r="C3" t="s">
+        <v>245</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>30</v>
+      </c>
+      <c r="F3">
+        <v>15</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3" t="s">
+        <v>184</v>
+      </c>
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" t="s">
+        <v>246</v>
+      </c>
+      <c r="B4" t="s">
+        <v>247</v>
+      </c>
+      <c r="C4" t="s">
+        <v>248</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>30</v>
+      </c>
+      <c r="F4">
+        <v>15</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4" t="s">
+        <v>189</v>
+      </c>
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:N22"/>
@@ -2099,7 +2349,7 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>197</v>
@@ -2122,7 +2372,7 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>197</v>
@@ -2136,7 +2386,7 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>197</v>
@@ -2150,7 +2400,7 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>197</v>
@@ -2164,7 +2414,7 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>197</v>
@@ -2178,7 +2428,7 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>197</v>
@@ -2192,7 +2442,7 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>197</v>
@@ -2206,7 +2456,7 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>197</v>
@@ -2220,10 +2470,10 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
+        <v>230</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>234</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>238</v>
       </c>
       <c r="C10">
         <v>1160</v>
@@ -2232,15 +2482,15 @@
         <v>-971</v>
       </c>
       <c r="H10" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="C11">
         <v>1160</v>
@@ -2249,15 +2499,15 @@
         <v>-808</v>
       </c>
       <c r="H11" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="C12">
         <v>1160</v>
@@ -2266,15 +2516,15 @@
         <v>-627</v>
       </c>
       <c r="H12" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="C13">
         <v>1160</v>
@@ -2283,12 +2533,12 @@
         <v>-223</v>
       </c>
       <c r="H13" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="B14" s="7" t="s">
         <v>197</v>
@@ -2302,7 +2552,7 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>197</v>
@@ -2646,7 +2896,7 @@
         <v>-691</v>
       </c>
       <c r="H2" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -2663,7 +2913,7 @@
         <v>-560</v>
       </c>
       <c r="H3" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -2680,7 +2930,7 @@
         <v>-456</v>
       </c>
       <c r="H4" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -2697,7 +2947,7 @@
         <v>-280</v>
       </c>
       <c r="H5" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -2714,7 +2964,7 @@
         <v>-689</v>
       </c>
       <c r="H6" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -2731,7 +2981,7 @@
         <v>-556</v>
       </c>
       <c r="H7" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -2748,7 +2998,7 @@
         <v>-419</v>
       </c>
       <c r="H8" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -2765,7 +3015,7 @@
         <v>-770</v>
       </c>
       <c r="H9" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -2782,7 +3032,7 @@
         <v>-292</v>
       </c>
       <c r="H10" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -2799,7 +3049,7 @@
         <v>-117</v>
       </c>
       <c r="H11" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -2816,7 +3066,7 @@
         <v>-50</v>
       </c>
       <c r="H12" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -2833,7 +3083,7 @@
         <v>-51</v>
       </c>
       <c r="H13" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
   </sheetData>
@@ -3252,7 +3502,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.44140625" customWidth="1"/>
@@ -3294,13 +3544,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="B2" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="C2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -3558,16 +3808,16 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>204</v>
+        <v>250</v>
       </c>
       <c r="B11" t="s">
+        <v>215</v>
+      </c>
+      <c r="C11" t="s">
         <v>214</v>
       </c>
-      <c r="C11" t="s">
-        <v>183</v>
-      </c>
       <c r="D11">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="E11">
         <v>30</v>
@@ -3579,7 +3829,7 @@
         <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="I11" t="b">
         <v>1</v>
@@ -3587,16 +3837,16 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>205</v>
+        <v>251</v>
       </c>
       <c r="B12" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C12" t="s">
-        <v>185</v>
+        <v>214</v>
       </c>
       <c r="D12">
-        <v>0.3</v>
+        <v>2</v>
       </c>
       <c r="E12">
         <v>30</v>
@@ -3608,7 +3858,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="I12" t="b">
         <v>1</v>
@@ -3616,16 +3866,16 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>206</v>
+        <v>252</v>
       </c>
       <c r="B13" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C13" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="D13">
-        <v>0.2</v>
+        <v>2</v>
       </c>
       <c r="E13">
         <v>30</v>
@@ -3637,7 +3887,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="I13" t="b">
         <v>1</v>
@@ -3645,16 +3895,16 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>207</v>
+        <v>253</v>
       </c>
       <c r="B14" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C14" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="D14">
-        <v>0.3</v>
+        <v>2</v>
       </c>
       <c r="E14">
         <v>30</v>
@@ -3666,7 +3916,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="I14" t="b">
         <v>1</v>
@@ -3674,16 +3924,16 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>186</v>
+        <v>204</v>
       </c>
       <c r="B15" t="s">
-        <v>187</v>
+        <v>210</v>
       </c>
       <c r="C15" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="D15">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="E15">
         <v>30</v>
@@ -3695,7 +3945,7 @@
         <v>0</v>
       </c>
       <c r="H15" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="I15" t="b">
         <v>1</v>
@@ -3703,16 +3953,16 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="B16" t="s">
-        <v>191</v>
+        <v>211</v>
       </c>
       <c r="C16" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D16">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="E16">
         <v>30</v>
@@ -3724,7 +3974,7 @@
         <v>0</v>
       </c>
       <c r="H16" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="I16" t="b">
         <v>1</v>
@@ -3732,16 +3982,16 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="B17" t="s">
-        <v>195</v>
+        <v>212</v>
       </c>
       <c r="C17" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="D17">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="E17">
         <v>30</v>
@@ -3753,7 +4003,7 @@
         <v>0</v>
       </c>
       <c r="H17" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="I17" t="b">
         <v>1</v>
@@ -3761,16 +4011,16 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B18" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
       <c r="C18" t="s">
-        <v>188</v>
+        <v>209</v>
       </c>
       <c r="D18">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="E18">
         <v>30</v>
@@ -3782,24 +4032,21 @@
         <v>0</v>
       </c>
       <c r="H18" t="s">
-        <v>199</v>
+        <v>184</v>
       </c>
       <c r="I18" t="b">
         <v>1</v>
-      </c>
-      <c r="J18" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>202</v>
+        <v>186</v>
       </c>
       <c r="B19" t="s">
-        <v>203</v>
+        <v>187</v>
       </c>
       <c r="C19" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -3814,27 +4061,24 @@
         <v>0</v>
       </c>
       <c r="H19" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="I19" t="b">
         <v>1</v>
-      </c>
-      <c r="J19" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="B20" t="s">
-        <v>219</v>
+        <v>198</v>
       </c>
       <c r="C20" t="s">
-        <v>218</v>
+        <v>188</v>
       </c>
       <c r="D20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E20">
         <v>30</v>
@@ -3846,101 +4090,161 @@
         <v>0</v>
       </c>
       <c r="H20" t="s">
-        <v>165</v>
+        <v>199</v>
       </c>
       <c r="I20" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:10">
-      <c r="A21" t="s">
-        <v>211</v>
-      </c>
-      <c r="B21" t="s">
-        <v>220</v>
-      </c>
-      <c r="C21" t="s">
-        <v>218</v>
-      </c>
-      <c r="D21">
-        <v>2</v>
-      </c>
-      <c r="E21">
-        <v>30</v>
-      </c>
-      <c r="F21">
-        <v>15</v>
-      </c>
-      <c r="G21">
-        <v>0</v>
-      </c>
-      <c r="H21" t="s">
-        <v>165</v>
-      </c>
-      <c r="I21" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10">
-      <c r="A22" t="s">
-        <v>212</v>
-      </c>
-      <c r="B22" t="s">
-        <v>221</v>
-      </c>
-      <c r="C22" t="s">
-        <v>218</v>
-      </c>
-      <c r="D22">
-        <v>2</v>
-      </c>
-      <c r="E22">
-        <v>30</v>
-      </c>
-      <c r="F22">
-        <v>15</v>
-      </c>
-      <c r="G22">
-        <v>0</v>
-      </c>
-      <c r="H22" t="s">
-        <v>165</v>
-      </c>
-      <c r="I22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10">
-      <c r="A23" t="s">
-        <v>213</v>
-      </c>
-      <c r="B23" t="s">
-        <v>222</v>
-      </c>
-      <c r="C23" t="s">
-        <v>218</v>
-      </c>
-      <c r="D23">
-        <v>2</v>
-      </c>
-      <c r="E23">
-        <v>30</v>
-      </c>
-      <c r="F23">
-        <v>15</v>
-      </c>
-      <c r="G23">
-        <v>0</v>
-      </c>
-      <c r="H23" t="s">
-        <v>165</v>
-      </c>
-      <c r="I23" t="b">
-        <v>1</v>
+      <c r="J20" t="s">
+        <v>200</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6371DE79-3429-4A4A-870D-B4BFB7D5E0F2}">
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="132.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E1" t="s">
+        <v>159</v>
+      </c>
+      <c r="F1" t="s">
+        <v>160</v>
+      </c>
+      <c r="G1" t="s">
+        <v>161</v>
+      </c>
+      <c r="H1" t="s">
+        <v>162</v>
+      </c>
+      <c r="I1" t="s">
+        <v>163</v>
+      </c>
+      <c r="J1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>30</v>
+      </c>
+      <c r="F2">
+        <v>15</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s">
+        <v>193</v>
+      </c>
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B3" t="s">
+        <v>195</v>
+      </c>
+      <c r="C3" t="s">
+        <v>196</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>30</v>
+      </c>
+      <c r="F3">
+        <v>15</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3" t="s">
+        <v>193</v>
+      </c>
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" t="s">
+        <v>202</v>
+      </c>
+      <c r="B4" t="s">
+        <v>203</v>
+      </c>
+      <c r="C4" t="s">
+        <v>196</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>30</v>
+      </c>
+      <c r="F4">
+        <v>15</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4" t="s">
+        <v>199</v>
+      </c>
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" t="s">
+        <v>200</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix label-cycle button width and animation conflict with CSS2DRenderer
- Add width:auto to .label-cycle-btn to override global button{width:100%}
- Lazily wrap label text node in inner span; animate span instead of outer
  CSS2DObject element so CSS2DRenderer's positioning transform is unaffected

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/floor_1_data.xlsx
+++ b/assets/floor_1_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\M.Mead\9.FactoryView\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E89ECA3-0756-40EF-8A34-22B43ECB160D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECF5F1A2-FCE3-4D75-93B7-30C535A2C61A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loc_name" sheetId="1" r:id="rId1"/>
@@ -24,10 +24,11 @@
     <sheet name="form_pouch_2" sheetId="15" r:id="rId9"/>
     <sheet name="zones" sheetId="8" r:id="rId10"/>
     <sheet name="zones_noname" sheetId="9" r:id="rId11"/>
-    <sheet name="flow_powder" sheetId="10" r:id="rId12"/>
-    <sheet name="flow_pouch" sheetId="11" r:id="rId13"/>
-    <sheet name="flow_can" sheetId="12" r:id="rId14"/>
-    <sheet name="flow_rtd" sheetId="13" r:id="rId15"/>
+    <sheet name="zones_building" sheetId="16" r:id="rId12"/>
+    <sheet name="flow_powder" sheetId="10" r:id="rId13"/>
+    <sheet name="flow_pouch" sheetId="11" r:id="rId14"/>
+    <sheet name="flow_can" sheetId="12" r:id="rId15"/>
+    <sheet name="flow_rtd" sheetId="13" r:id="rId16"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -211,7 +212,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1408" uniqueCount="505">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1439" uniqueCount="513">
   <si>
     <t>Name</t>
   </si>
@@ -1726,6 +1727,30 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>milk_cans</t>
+  </si>
+  <si>
+    <t>Name1</t>
+  </si>
+  <si>
+    <t>FRM-00263</t>
+  </si>
+  <si>
+    <t>FRM-00242</t>
+  </si>
+  <si>
+    <t>SD011149</t>
+  </si>
+  <si>
+    <t>SD011163</t>
+  </si>
+  <si>
+    <t>SD011636</t>
+  </si>
+  <si>
+    <t>SD036012</t>
   </si>
 </sst>
 </file>
@@ -2984,6 +3009,338 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB6F1B60-63C1-4547-8A01-D2D6864F7BDB}">
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="21.44140625" style="8" customWidth="1"/>
+    <col min="2" max="7" width="8.88671875" style="8" customWidth="1"/>
+    <col min="8" max="8" width="7.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.88671875" style="8" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>306</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>307</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>308</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>311</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="B2" s="8">
+        <v>589</v>
+      </c>
+      <c r="C2" s="8">
+        <v>-1104</v>
+      </c>
+      <c r="D2" s="8">
+        <v>1229</v>
+      </c>
+      <c r="E2" s="8">
+        <v>-190</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="G2" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="H2" s="8">
+        <v>14</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="B3" s="8">
+        <v>1229</v>
+      </c>
+      <c r="C3" s="8">
+        <v>-759</v>
+      </c>
+      <c r="D3" s="8">
+        <v>1511</v>
+      </c>
+      <c r="E3" s="8">
+        <v>-190</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="G3" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="H3" s="8">
+        <v>14</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="B4" s="8">
+        <v>217</v>
+      </c>
+      <c r="C4" s="8">
+        <v>-190</v>
+      </c>
+      <c r="D4" s="8">
+        <v>1585</v>
+      </c>
+      <c r="E4" s="8">
+        <v>-5</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="G4" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="H4" s="8">
+        <v>14</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="B5" s="8">
+        <v>-1374</v>
+      </c>
+      <c r="C5" s="8">
+        <v>-1303</v>
+      </c>
+      <c r="D5" s="8">
+        <v>452</v>
+      </c>
+      <c r="E5" s="8">
+        <v>-971</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="G5" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="H5" s="8">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="B6" s="8">
+        <v>-173</v>
+      </c>
+      <c r="C6" s="8">
+        <v>-193</v>
+      </c>
+      <c r="D6" s="8">
+        <v>216</v>
+      </c>
+      <c r="E6" s="8">
+        <v>-5</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="G6" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="H6" s="8">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="B7" s="8">
+        <v>173</v>
+      </c>
+      <c r="C7" s="8">
+        <v>-5</v>
+      </c>
+      <c r="D7" s="8">
+        <v>726</v>
+      </c>
+      <c r="E7" s="8">
+        <v>320</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="G7" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="H7" s="8">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="B8" s="8">
+        <v>-468</v>
+      </c>
+      <c r="C8" s="8">
+        <v>-971</v>
+      </c>
+      <c r="D8" s="8">
+        <v>591</v>
+      </c>
+      <c r="E8" s="8">
+        <v>-190</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>324</v>
+      </c>
+      <c r="G8" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="H8" s="8">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="B9" s="8">
+        <v>-1540</v>
+      </c>
+      <c r="C9" s="8">
+        <v>-971</v>
+      </c>
+      <c r="D9" s="8">
+        <v>-468</v>
+      </c>
+      <c r="E9" s="8">
+        <v>-190</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="G9" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="H9" s="8">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="B10" s="8">
+        <v>-206</v>
+      </c>
+      <c r="C10" s="8">
+        <v>-8</v>
+      </c>
+      <c r="D10" s="8">
+        <v>119</v>
+      </c>
+      <c r="E10" s="8">
+        <v>728</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>328</v>
+      </c>
+      <c r="G10" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="H10" s="8">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="B11" s="8">
+        <v>119</v>
+      </c>
+      <c r="C11" s="8">
+        <v>488</v>
+      </c>
+      <c r="D11" s="8">
+        <v>535</v>
+      </c>
+      <c r="E11" s="8">
+        <v>728</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>328</v>
+      </c>
+      <c r="G11" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="H11" s="8">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="B12" s="8">
+        <v>-2703</v>
+      </c>
+      <c r="C12" s="8">
+        <v>-584</v>
+      </c>
+      <c r="D12" s="8">
+        <v>-1785</v>
+      </c>
+      <c r="E12" s="8">
+        <v>1308</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="G12" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="H12" s="8">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="B13" s="8">
+        <v>2121</v>
+      </c>
+      <c r="C13" s="8">
+        <v>-1169</v>
+      </c>
+      <c r="D13" s="8">
+        <v>2645</v>
+      </c>
+      <c r="E13" s="8">
+        <v>6</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>332</v>
+      </c>
+      <c r="G13" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="H13" s="8">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:K10"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3324,7 +3681,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:K11"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3695,7 +4052,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3864,7 +4221,7 @@
         <v>0</v>
       </c>
       <c r="H5" s="25" t="s">
-        <v>391</v>
+        <v>505</v>
       </c>
       <c r="I5" s="25" t="b">
         <v>1</v>
@@ -3879,7 +4236,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -5896,165 +6253,169 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:Q22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="11" customWidth="1"/>
-    <col min="2" max="2" width="43.77734375" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.77734375" customWidth="1"/>
-    <col min="5" max="5" width="5" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.77734375" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.88671875" style="8" customWidth="1"/>
-    <col min="11" max="11" width="80.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.21875" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="50.21875" style="8" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="63.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.77734375" style="8" customWidth="1"/>
+    <col min="3" max="3" width="26" style="8" customWidth="1"/>
+    <col min="4" max="4" width="10.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.77734375" customWidth="1"/>
+    <col min="6" max="6" width="5" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.77734375" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.88671875" style="8" customWidth="1"/>
+    <col min="12" max="12" width="80.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.21875" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9" style="8" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="50.21875" style="8" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="63.33203125" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16">
+    <row r="1" spans="1:17">
       <c r="A1" s="11" t="s">
         <v>167</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="8" t="s">
+        <v>506</v>
+      </c>
+      <c r="D1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>174</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>6</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>7</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>168</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>169</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>170</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>171</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>172</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="2" spans="1:16" s="13" customFormat="1">
+    <row r="2" spans="1:17" s="13" customFormat="1">
       <c r="A2" s="12">
         <v>1</v>
       </c>
       <c r="B2" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="C2" s="13" t="s">
-        <v>176</v>
-      </c>
       <c r="D2" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="E2" s="13" t="s">
         <v>413</v>
       </c>
-      <c r="E2" s="13">
+      <c r="F2" s="13">
         <v>420</v>
       </c>
-      <c r="F2" s="13">
+      <c r="G2" s="13">
         <v>-660</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="H2" s="13" t="s">
         <v>177</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="K2" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="L2" s="13" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="3" spans="1:16" s="13" customFormat="1">
+    <row r="3" spans="1:17" s="13" customFormat="1">
       <c r="A3" s="12">
         <v>2</v>
       </c>
       <c r="B3" s="13" t="s">
         <v>305</v>
       </c>
-      <c r="C3" s="13" t="s">
-        <v>176</v>
-      </c>
       <c r="D3" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="E3" s="13" t="s">
         <v>413</v>
       </c>
-      <c r="E3" s="13">
+      <c r="F3" s="13">
         <v>420</v>
       </c>
-      <c r="F3" s="13">
+      <c r="G3" s="13">
         <v>-630</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="H3" s="13" t="s">
         <v>299</v>
       </c>
-      <c r="J3" s="13" t="s">
+      <c r="K3" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="K3" s="13" t="s">
+      <c r="L3" s="13" t="s">
         <v>495</v>
       </c>
     </row>
-    <row r="4" spans="1:16" s="13" customFormat="1">
+    <row r="4" spans="1:17" s="13" customFormat="1">
       <c r="A4" s="12">
         <v>3</v>
       </c>
       <c r="B4" s="13" t="s">
         <v>180</v>
       </c>
-      <c r="C4" s="13" t="s">
-        <v>176</v>
-      </c>
       <c r="D4" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="E4" s="13" t="s">
         <v>413</v>
       </c>
-      <c r="E4" s="13">
+      <c r="F4" s="13">
         <v>420</v>
       </c>
-      <c r="F4" s="13">
+      <c r="G4" s="13">
         <v>-600</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="H4" s="13" t="s">
         <v>181</v>
       </c>
-      <c r="J4" s="13" t="s">
+      <c r="K4" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="K4" s="13" t="s">
+      <c r="L4" s="13" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="5" spans="1:16" s="13" customFormat="1">
+    <row r="5" spans="1:17" s="13" customFormat="1">
       <c r="A5" s="12">
         <v>4</v>
       </c>
@@ -6062,180 +6423,183 @@
         <v>183</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>176</v>
+        <v>508</v>
       </c>
       <c r="D5" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="E5" s="13" t="s">
         <v>413</v>
       </c>
-      <c r="E5" s="13">
+      <c r="F5" s="13">
         <v>420</v>
       </c>
-      <c r="F5" s="13">
+      <c r="G5" s="13">
         <v>-570</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="H5" s="13" t="s">
         <v>181</v>
       </c>
-      <c r="J5" s="13" t="s">
+      <c r="K5" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="K5" s="13" t="s">
+      <c r="L5" s="13" t="s">
         <v>184</v>
       </c>
-      <c r="L5" s="13" t="s">
+      <c r="M5" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="M5" s="13" t="s">
+      <c r="N5" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="N5" s="13" t="s">
+      <c r="O5" s="13" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="6" spans="1:16" s="13" customFormat="1">
+    <row r="6" spans="1:17" s="13" customFormat="1">
       <c r="A6" s="12">
         <v>5</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>187</v>
       </c>
-      <c r="C6" s="13" t="s">
-        <v>176</v>
-      </c>
       <c r="D6" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="E6" s="13" t="s">
         <v>413</v>
       </c>
-      <c r="E6" s="13">
+      <c r="F6" s="13">
         <v>420</v>
       </c>
-      <c r="F6" s="13">
+      <c r="G6" s="13">
         <v>-540</v>
       </c>
-      <c r="G6" s="13" t="s">
+      <c r="H6" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="J6" s="13" t="s">
+      <c r="K6" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="K6" s="13" t="s">
+      <c r="L6" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="L6" s="13" t="s">
+      <c r="M6" s="13" t="s">
         <v>185</v>
-      </c>
-      <c r="M6" s="13" t="s">
-        <v>186</v>
       </c>
       <c r="N6" s="13" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" s="13" customFormat="1">
+      <c r="O6" s="13" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" s="13" customFormat="1">
       <c r="A7" s="12">
         <v>6</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>190</v>
       </c>
-      <c r="C7" s="13" t="s">
-        <v>176</v>
-      </c>
       <c r="D7" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="E7" s="13" t="s">
         <v>413</v>
       </c>
-      <c r="E7" s="13">
+      <c r="F7" s="13">
         <v>420</v>
       </c>
-      <c r="F7" s="13">
+      <c r="G7" s="13">
         <v>-510</v>
       </c>
-      <c r="G7" s="13" t="s">
+      <c r="H7" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="J7" s="13" t="s">
+      <c r="K7" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="K7" s="13" t="s">
+      <c r="L7" s="13" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="8" spans="1:16" s="13" customFormat="1">
+    <row r="8" spans="1:17" s="13" customFormat="1">
       <c r="A8" s="12">
         <v>7</v>
       </c>
       <c r="B8" s="13" t="s">
         <v>192</v>
       </c>
-      <c r="C8" s="13" t="s">
-        <v>176</v>
-      </c>
       <c r="D8" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="E8" s="13" t="s">
         <v>413</v>
       </c>
-      <c r="E8" s="13">
+      <c r="F8" s="13">
         <v>420</v>
       </c>
-      <c r="F8" s="13">
+      <c r="G8" s="13">
         <v>-480</v>
       </c>
-      <c r="G8" s="13" t="s">
+      <c r="H8" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="J8" s="13" t="s">
+      <c r="K8" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="K8" s="13" t="s">
+      <c r="L8" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="L8" s="13" t="s">
+      <c r="M8" s="13" t="s">
         <v>185</v>
-      </c>
-      <c r="M8" s="13" t="s">
-        <v>186</v>
       </c>
       <c r="N8" s="13" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" s="13" customFormat="1">
+      <c r="O8" s="13" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" s="13" customFormat="1">
       <c r="A9" s="12">
         <v>8</v>
       </c>
       <c r="B9" s="13" t="s">
         <v>194</v>
       </c>
-      <c r="C9" s="13" t="s">
-        <v>176</v>
-      </c>
       <c r="D9" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="E9" s="13" t="s">
         <v>414</v>
       </c>
-      <c r="E9" s="13">
+      <c r="F9" s="13">
         <v>420</v>
       </c>
-      <c r="F9" s="13">
+      <c r="G9" s="13">
         <v>-450</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="H9" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="J9" s="13" t="s">
+      <c r="K9" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="K9" s="13" t="s">
+      <c r="L9" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="L9" s="13" t="s">
+      <c r="M9" s="13" t="s">
         <v>185</v>
-      </c>
-      <c r="M9" s="13" t="s">
-        <v>186</v>
       </c>
       <c r="N9" s="13" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="10" spans="1:16" s="9" customFormat="1">
+      <c r="O9" s="13" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" s="9" customFormat="1">
       <c r="A10" s="20">
         <v>9</v>
       </c>
@@ -6243,66 +6607,69 @@
         <v>196</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>176</v>
+        <v>507</v>
       </c>
       <c r="D10" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="E10" s="9" t="s">
         <v>414</v>
       </c>
-      <c r="E10" s="9">
+      <c r="F10" s="9">
         <v>686</v>
       </c>
-      <c r="F10" s="9">
+      <c r="G10" s="9">
         <v>-330</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="H10" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="J10" s="9" t="s">
+      <c r="K10" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="K10" s="9" t="s">
+      <c r="L10" s="9" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="11" spans="1:16" s="9" customFormat="1">
+    <row r="11" spans="1:17" s="9" customFormat="1">
       <c r="A11" s="20">
         <v>10</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="C11" s="9" t="s">
-        <v>176</v>
-      </c>
       <c r="D11" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="E11" s="9" t="s">
         <v>414</v>
       </c>
-      <c r="E11" s="9">
+      <c r="F11" s="9">
         <v>686</v>
       </c>
-      <c r="F11" s="9">
+      <c r="G11" s="9">
         <v>-300</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="H11" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="J11" s="9" t="s">
+      <c r="K11" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="K11" s="9" t="s">
+      <c r="L11" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="L11" s="9" t="s">
+      <c r="M11" s="9" t="s">
         <v>185</v>
-      </c>
-      <c r="M11" s="9" t="s">
-        <v>186</v>
       </c>
       <c r="N11" s="9" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" s="9" customFormat="1">
+      <c r="O11" s="9" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" s="9" customFormat="1">
       <c r="A12" s="20">
         <v>11</v>
       </c>
@@ -6310,28 +6677,31 @@
         <v>201</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>176</v>
+        <v>509</v>
       </c>
       <c r="D12" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="E12" s="9" t="s">
         <v>414</v>
       </c>
-      <c r="E12" s="9">
+      <c r="F12" s="9">
         <v>686</v>
       </c>
-      <c r="F12" s="9">
+      <c r="G12" s="9">
         <v>-270</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="H12" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="J12" s="9" t="s">
+      <c r="K12" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="K12" s="9" t="s">
+      <c r="L12" s="9" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="13" spans="1:16" s="9" customFormat="1">
+    <row r="13" spans="1:17" s="9" customFormat="1">
       <c r="A13" s="20">
         <v>12</v>
       </c>
@@ -6339,124 +6709,127 @@
         <v>203</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>176</v>
+        <v>512</v>
       </c>
       <c r="D13" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="E13" s="9" t="s">
         <v>414</v>
       </c>
-      <c r="E13" s="9">
+      <c r="F13" s="9">
         <v>1134</v>
       </c>
-      <c r="F13" s="9">
+      <c r="G13" s="9">
         <v>-330</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="H13" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="J13" s="9" t="s">
+      <c r="K13" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="K13" s="9" t="s">
+      <c r="L13" s="9" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="14" spans="1:16" s="9" customFormat="1">
+    <row r="14" spans="1:17" s="9" customFormat="1">
       <c r="A14" s="20">
         <v>13</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="C14" s="9" t="s">
-        <v>176</v>
-      </c>
       <c r="D14" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="E14" s="9" t="s">
         <v>414</v>
       </c>
-      <c r="E14" s="9">
+      <c r="F14" s="9">
         <v>1134</v>
       </c>
-      <c r="F14" s="9">
+      <c r="G14" s="9">
         <v>-300</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="H14" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="J14" s="9" t="s">
+      <c r="K14" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="K14" s="9" t="s">
+      <c r="L14" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="L14" s="9" t="s">
+      <c r="M14" s="9" t="s">
         <v>185</v>
-      </c>
-      <c r="M14" s="9" t="s">
-        <v>186</v>
       </c>
       <c r="N14" s="9" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="15" spans="1:16" s="9" customFormat="1">
+      <c r="O14" s="9" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" s="9" customFormat="1">
       <c r="A15" s="20">
         <v>14</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="C15" s="9" t="s">
-        <v>176</v>
-      </c>
       <c r="D15" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="E15" s="9" t="s">
         <v>414</v>
       </c>
-      <c r="E15" s="9">
+      <c r="F15" s="9">
         <v>1134</v>
       </c>
-      <c r="F15" s="9">
+      <c r="G15" s="9">
         <v>-270</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="H15" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="J15" s="9" t="s">
+      <c r="K15" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="K15" s="9" t="s">
+      <c r="L15" s="9" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="16" spans="1:16" s="9" customFormat="1">
+    <row r="16" spans="1:17" s="9" customFormat="1">
       <c r="A16" s="20">
         <v>15</v>
       </c>
       <c r="B16" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="C16" s="9" t="s">
-        <v>176</v>
-      </c>
       <c r="D16" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="E16" s="9" t="s">
         <v>411</v>
       </c>
-      <c r="E16" s="9">
+      <c r="F16" s="9">
         <v>1186</v>
       </c>
-      <c r="F16" s="9">
+      <c r="G16" s="9">
         <v>-240</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="H16" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="J16" s="9" t="s">
+      <c r="K16" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="K16" s="9" t="s">
+      <c r="L16" s="9" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="17" spans="1:14" s="9" customFormat="1">
+    <row r="17" spans="1:15" s="9" customFormat="1">
       <c r="A17" s="20">
         <v>16</v>
       </c>
@@ -6464,28 +6837,31 @@
         <v>213</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>176</v>
+        <v>511</v>
       </c>
       <c r="D17" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="E17" s="9" t="s">
         <v>413</v>
       </c>
-      <c r="E17" s="9">
+      <c r="F17" s="9">
         <v>1186</v>
       </c>
-      <c r="F17" s="9">
+      <c r="G17" s="9">
         <v>-210</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="H17" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="J17" s="9" t="s">
+      <c r="K17" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="K17" s="9" t="s">
+      <c r="L17" s="9" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="18" spans="1:14" s="9" customFormat="1">
+    <row r="18" spans="1:15" s="9" customFormat="1">
       <c r="A18" s="20">
         <v>17</v>
       </c>
@@ -6493,149 +6869,152 @@
         <v>215</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>176</v>
+        <v>510</v>
       </c>
       <c r="D18" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="E18" s="9" t="s">
         <v>412</v>
       </c>
-      <c r="E18" s="9">
+      <c r="F18" s="9">
         <v>1084</v>
       </c>
-      <c r="F18" s="9">
+      <c r="G18" s="9">
         <v>-210</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="H18" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="J18" s="9" t="s">
+      <c r="K18" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="K18" s="9" t="s">
+      <c r="L18" s="9" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="19" spans="1:14" s="17" customFormat="1">
+    <row r="19" spans="1:15" s="17" customFormat="1">
       <c r="A19" s="16">
         <v>18</v>
       </c>
       <c r="B19" s="17" t="s">
         <v>218</v>
       </c>
-      <c r="C19" s="17" t="s">
-        <v>176</v>
-      </c>
       <c r="D19" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="E19" s="17" t="s">
         <v>411</v>
       </c>
-      <c r="E19" s="17">
+      <c r="F19" s="17">
         <v>420</v>
       </c>
-      <c r="F19" s="17">
+      <c r="G19" s="17">
         <v>-330</v>
       </c>
-      <c r="G19" s="17" t="s">
+      <c r="H19" s="17" t="s">
         <v>177</v>
       </c>
-      <c r="J19" s="17" t="s">
+      <c r="K19" s="17" t="s">
         <v>211</v>
       </c>
-      <c r="K19" s="17" t="s">
+      <c r="L19" s="17" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="20" spans="1:14" s="17" customFormat="1">
+    <row r="20" spans="1:15" s="17" customFormat="1">
       <c r="A20" s="16">
         <v>19</v>
       </c>
       <c r="B20" s="17" t="s">
         <v>220</v>
       </c>
-      <c r="C20" s="17" t="s">
-        <v>176</v>
-      </c>
       <c r="D20" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="E20" s="17" t="s">
         <v>415</v>
       </c>
-      <c r="E20" s="17">
+      <c r="F20" s="17">
         <v>420</v>
       </c>
-      <c r="F20" s="17">
+      <c r="G20" s="17">
         <v>-300</v>
       </c>
-      <c r="G20" s="17" t="s">
+      <c r="H20" s="17" t="s">
         <v>181</v>
       </c>
-      <c r="J20" s="17" t="s">
+      <c r="K20" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="K20" s="17" t="s">
+      <c r="L20" s="17" t="s">
         <v>221</v>
       </c>
-      <c r="L20" s="17" t="s">
+      <c r="M20" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="M20" s="17" t="s">
+      <c r="N20" s="17" t="s">
         <v>186</v>
       </c>
-      <c r="N20" s="17" t="s">
+      <c r="O20" s="17" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="21" spans="1:14" s="17" customFormat="1">
+    <row r="21" spans="1:15" s="17" customFormat="1">
       <c r="A21" s="16">
         <v>20</v>
       </c>
       <c r="B21" s="17" t="s">
         <v>222</v>
       </c>
-      <c r="C21" s="17" t="s">
-        <v>176</v>
-      </c>
       <c r="D21" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="E21" s="17" t="s">
         <v>415</v>
       </c>
-      <c r="E21" s="17">
+      <c r="F21" s="17">
         <v>420</v>
       </c>
-      <c r="F21" s="17">
+      <c r="G21" s="17">
         <v>-270</v>
       </c>
-      <c r="G21" s="17" t="s">
+      <c r="H21" s="17" t="s">
         <v>223</v>
       </c>
-      <c r="J21" s="17" t="s">
+      <c r="K21" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="K21" s="17" t="s">
+      <c r="L21" s="17" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="22" spans="1:14" s="17" customFormat="1">
+    <row r="22" spans="1:15" s="17" customFormat="1">
       <c r="A22" s="16">
         <v>21</v>
       </c>
       <c r="B22" s="17" t="s">
         <v>225</v>
       </c>
-      <c r="C22" s="17" t="s">
-        <v>176</v>
-      </c>
       <c r="D22" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="E22" s="17" t="s">
         <v>415</v>
       </c>
-      <c r="E22" s="17">
+      <c r="F22" s="17">
         <v>420</v>
       </c>
-      <c r="F22" s="17">
+      <c r="G22" s="17">
         <v>-240</v>
       </c>
-      <c r="G22" s="17" t="s">
+      <c r="H22" s="17" t="s">
         <v>223</v>
       </c>
-      <c r="J22" s="17" t="s">
+      <c r="K22" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="K22" s="17" t="s">
+      <c r="L22" s="17" t="s">
         <v>226</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 4 features: local PDF serving, item popup, Name3/obsolete, admin data panel
- Fix PDF overlay to serve directly from assets/docs/ when running on localhost
  (python -m http.server) instead of routing through /api/docs/
- Add ItemPopup component for machine/equipment layers: photo + specs card
  with CSS spring animation (cubic-bezier overshoot); enabled per layer via
  Popup column in system_config.xlsx Layers sheet
- Add Name3 label cycle mode; if Name3='-' hides label and greys mesh (obsolete)
  with red diagonal OBSOLETE stamp on PDF overlay
- Add admin Data Files panel (left panel) with download buttons and upload-to-
  Vercel-Blob for floor/config/preset xlsx files; DataLoader auto-prefers blob
  versions over static assets when available

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/floor_1_data.xlsx
+++ b/assets/floor_1_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\M.Mead\9.FactoryView\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29DDC3B8-B778-4C06-970D-9A156208230F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFB826D4-458A-405A-85F0-5E7B4024863F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="695" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="807" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loc_name" sheetId="1" r:id="rId1"/>
@@ -212,7 +212,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1435" uniqueCount="516">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1467" uniqueCount="523">
   <si>
     <t>Name</t>
   </si>
@@ -1681,9 +1681,6 @@
     <t>assets/docs/1000381996+1000381979_POUCH/0.Overall/P_071_079.pdf</t>
   </si>
   <si>
-    <t>assets/docs/1000381996+1000381979_POUCH/0.Overall/P_080_092.pdf</t>
-  </si>
-  <si>
     <t>assets/docs/1000381996+1000381979_POUCH/1.Batch%20Preparation/P_106_110.pdf</t>
   </si>
   <si>
@@ -1760,6 +1757,30 @@
   </si>
   <si>
     <t>Alacta f1</t>
+  </si>
+  <si>
+    <t>Flush Line &amp; Dry Clean Record</t>
+  </si>
+  <si>
+    <t>Name2</t>
+  </si>
+  <si>
+    <t>Name3</t>
+  </si>
+  <si>
+    <t>Optiva</t>
+  </si>
+  <si>
+    <t>SAP</t>
+  </si>
+  <si>
+    <t>Op-Once</t>
+  </si>
+  <si>
+    <t>Continuous</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
 </sst>
 </file>
@@ -2367,7 +2388,7 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B2">
         <v>589</v>
@@ -2382,7 +2403,7 @@
         <v>-190</v>
       </c>
       <c r="F2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="G2">
         <v>0.2</v>
@@ -2391,12 +2412,12 @@
         <v>14</v>
       </c>
       <c r="I2" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="8" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B3">
         <v>1229</v>
@@ -2420,7 +2441,7 @@
         <v>14</v>
       </c>
       <c r="I3" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -2451,7 +2472,7 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B5">
         <v>217</v>
@@ -2697,7 +2718,7 @@
         <v>6</v>
       </c>
       <c r="F14" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="G14">
         <v>0.2</v>
@@ -2766,7 +2787,7 @@
         <v>-190</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="G2" s="8">
         <v>0.2</v>
@@ -2775,7 +2796,7 @@
         <v>14</v>
       </c>
       <c r="I2" s="8" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -2801,7 +2822,7 @@
         <v>14</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -3051,7 +3072,7 @@
         <v>6</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="G14" s="8">
         <v>0.2</v>
@@ -3108,7 +3129,7 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="8" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B2" s="8">
         <v>-2703</v>
@@ -3134,7 +3155,7 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="8" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B3" s="8">
         <v>-1782</v>
@@ -3149,7 +3170,7 @@
         <v>930</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="G3" s="8">
         <v>0.2</v>
@@ -3160,7 +3181,7 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="8" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B4" s="8">
         <v>-1782</v>
@@ -3175,7 +3196,7 @@
         <v>-194</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="G4" s="8">
         <v>0.2</v>
@@ -3198,7 +3219,7 @@
         <v>733</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="G5" s="8">
         <v>0.2</v>
@@ -3221,7 +3242,7 @@
         <v>198</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="G6" s="8">
         <v>0.2</v>
@@ -4002,7 +4023,7 @@
         <v>383</v>
       </c>
       <c r="B2" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C2" t="s">
         <v>384</v>
@@ -4095,13 +4116,13 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="25" t="s">
+        <v>491</v>
+      </c>
+      <c r="B5" s="25" t="s">
         <v>492</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="C5" s="25" t="s">
         <v>493</v>
-      </c>
-      <c r="C5" s="25" t="s">
-        <v>494</v>
       </c>
       <c r="D5" s="25">
         <v>1</v>
@@ -4116,13 +4137,13 @@
         <v>0</v>
       </c>
       <c r="H5" s="25" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="I5" s="25" t="b">
         <v>1</v>
       </c>
       <c r="J5" s="25" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
   </sheetData>
@@ -6148,29 +6169,30 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:Q22"/>
+  <dimension ref="A1:S22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="11" customWidth="1"/>
     <col min="2" max="2" width="32.77734375" style="8" customWidth="1"/>
-    <col min="3" max="3" width="26" style="8" customWidth="1"/>
-    <col min="4" max="4" width="10.109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.77734375" customWidth="1"/>
-    <col min="6" max="6" width="5" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.77734375" style="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.88671875" style="8" customWidth="1"/>
-    <col min="12" max="12" width="80.5546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.21875" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="50.21875" style="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="63.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="20.6640625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="20.6640625" style="11" customWidth="1"/>
+    <col min="6" max="6" width="10.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.77734375" customWidth="1"/>
+    <col min="8" max="8" width="5" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.77734375" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.88671875" style="8" customWidth="1"/>
+    <col min="14" max="14" width="80.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.21875" style="8" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9" style="8" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="50.21875" style="8" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="63.33203125" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:19">
       <c r="A1" s="11" t="s">
         <v>167</v>
       </c>
@@ -6178,52 +6200,58 @@
         <v>0</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>497</v>
-      </c>
-      <c r="D1" t="s">
+        <v>496</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>516</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>517</v>
+      </c>
+      <c r="F1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>174</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>2</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>4</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>5</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>6</v>
       </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>7</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>168</v>
       </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>169</v>
       </c>
-      <c r="N1" t="s">
+      <c r="P1" t="s">
         <v>170</v>
       </c>
-      <c r="O1" t="s">
+      <c r="Q1" t="s">
         <v>171</v>
       </c>
-      <c r="P1" t="s">
+      <c r="R1" t="s">
         <v>172</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="S1" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="2" spans="1:17" s="13" customFormat="1">
+    <row r="2" spans="1:19" s="13" customFormat="1">
       <c r="A2" s="12">
         <v>1</v>
       </c>
@@ -6231,28 +6259,34 @@
         <v>175</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="E2" s="13" t="s">
+        <v>518</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>522</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="G2" s="13" t="s">
         <v>404</v>
       </c>
-      <c r="F2" s="13">
+      <c r="H2" s="13">
         <v>420</v>
       </c>
-      <c r="G2" s="13">
+      <c r="I2" s="13">
         <v>-660</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="J2" s="13" t="s">
         <v>177</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="M2" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="L2" s="13" t="s">
+      <c r="N2" s="13" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="3" spans="1:17" s="13" customFormat="1">
+    <row r="3" spans="1:19" s="13" customFormat="1">
       <c r="A3" s="12">
         <v>2</v>
       </c>
@@ -6260,28 +6294,34 @@
         <v>305</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="E3" s="13" t="s">
+        <v>518</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>522</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="G3" s="13" t="s">
         <v>404</v>
       </c>
-      <c r="F3" s="13">
+      <c r="H3" s="13">
         <v>420</v>
       </c>
-      <c r="G3" s="13">
+      <c r="I3" s="13">
         <v>-630</v>
       </c>
-      <c r="H3" s="13" t="s">
+      <c r="J3" s="13" t="s">
         <v>299</v>
       </c>
-      <c r="K3" s="13" t="s">
+      <c r="M3" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="L3" s="13" t="s">
+      <c r="N3" s="13" t="s">
         <v>486</v>
       </c>
     </row>
-    <row r="4" spans="1:17" s="13" customFormat="1">
+    <row r="4" spans="1:19" s="13" customFormat="1">
       <c r="A4" s="12">
         <v>3</v>
       </c>
@@ -6289,28 +6329,34 @@
         <v>180</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="E4" s="13" t="s">
+        <v>519</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>522</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="G4" s="13" t="s">
         <v>404</v>
       </c>
-      <c r="F4" s="13">
+      <c r="H4" s="13">
         <v>420</v>
       </c>
-      <c r="G4" s="13">
+      <c r="I4" s="13">
         <v>-600</v>
       </c>
-      <c r="H4" s="13" t="s">
+      <c r="J4" s="13" t="s">
         <v>181</v>
       </c>
-      <c r="K4" s="13" t="s">
+      <c r="M4" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="L4" s="13" t="s">
+      <c r="N4" s="13" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="5" spans="1:17" s="13" customFormat="1">
+    <row r="5" spans="1:19" s="13" customFormat="1">
       <c r="A5" s="12">
         <v>4</v>
       </c>
@@ -6318,40 +6364,43 @@
         <v>183</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>499</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="E5" s="13" t="s">
+        <v>498</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>522</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="G5" s="13" t="s">
         <v>404</v>
       </c>
-      <c r="F5" s="13">
+      <c r="H5" s="13">
         <v>420</v>
       </c>
-      <c r="G5" s="13">
+      <c r="I5" s="13">
         <v>-570</v>
       </c>
-      <c r="H5" s="13" t="s">
+      <c r="J5" s="13" t="s">
         <v>181</v>
       </c>
-      <c r="K5" s="13" t="s">
+      <c r="M5" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="L5" s="13" t="s">
+      <c r="N5" s="13" t="s">
         <v>184</v>
       </c>
-      <c r="M5" s="13" t="s">
+      <c r="O5" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="N5" s="13" t="s">
+      <c r="P5" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="O5" s="13" t="s">
+      <c r="Q5" s="13" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="6" spans="1:17" s="13" customFormat="1">
+    <row r="6" spans="1:19" s="13" customFormat="1">
       <c r="A6" s="12">
         <v>5</v>
       </c>
@@ -6359,37 +6408,43 @@
         <v>187</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="E6" s="13" t="s">
+        <v>519</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>522</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="G6" s="13" t="s">
         <v>404</v>
       </c>
-      <c r="F6" s="13">
+      <c r="H6" s="13">
         <v>420</v>
       </c>
-      <c r="G6" s="13">
+      <c r="I6" s="13">
         <v>-540</v>
       </c>
-      <c r="H6" s="13" t="s">
+      <c r="J6" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="K6" s="13" t="s">
+      <c r="M6" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="L6" s="13" t="s">
+      <c r="N6" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="M6" s="13" t="s">
+      <c r="O6" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="N6" s="13" t="s">
+      <c r="P6" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="O6" s="13" t="s">
+      <c r="Q6" s="13" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="7" spans="1:17" s="13" customFormat="1">
+    <row r="7" spans="1:19" s="13" customFormat="1">
       <c r="A7" s="12">
         <v>6</v>
       </c>
@@ -6397,28 +6452,34 @@
         <v>190</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="E7" s="13" t="s">
+        <v>519</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>522</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="G7" s="13" t="s">
         <v>404</v>
       </c>
-      <c r="F7" s="13">
+      <c r="H7" s="13">
         <v>420</v>
       </c>
-      <c r="G7" s="13">
+      <c r="I7" s="13">
         <v>-510</v>
       </c>
-      <c r="H7" s="13" t="s">
+      <c r="J7" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="K7" s="13" t="s">
+      <c r="M7" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="L7" s="13" t="s">
+      <c r="N7" s="13" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="8" spans="1:17" s="13" customFormat="1">
+    <row r="8" spans="1:19" s="13" customFormat="1">
       <c r="A8" s="12">
         <v>7</v>
       </c>
@@ -6426,37 +6487,43 @@
         <v>192</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="E8" s="13" t="s">
+        <v>519</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>522</v>
+      </c>
+      <c r="F8" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="G8" s="13" t="s">
         <v>404</v>
       </c>
-      <c r="F8" s="13">
+      <c r="H8" s="13">
         <v>420</v>
       </c>
-      <c r="G8" s="13">
+      <c r="I8" s="13">
         <v>-480</v>
       </c>
-      <c r="H8" s="13" t="s">
+      <c r="J8" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="K8" s="13" t="s">
+      <c r="M8" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="L8" s="13" t="s">
+      <c r="N8" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="M8" s="13" t="s">
+      <c r="O8" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="N8" s="13" t="s">
+      <c r="P8" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="O8" s="13" t="s">
+      <c r="Q8" s="13" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="9" spans="1:17" s="13" customFormat="1">
+    <row r="9" spans="1:19" s="13" customFormat="1">
       <c r="A9" s="12">
         <v>8</v>
       </c>
@@ -6464,37 +6531,43 @@
         <v>194</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="E9" s="13" t="s">
+        <v>520</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>522</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="G9" s="13" t="s">
         <v>405</v>
       </c>
-      <c r="F9" s="13">
+      <c r="H9" s="13">
         <v>420</v>
       </c>
-      <c r="G9" s="13">
+      <c r="I9" s="13">
         <v>-450</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="J9" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="K9" s="13" t="s">
+      <c r="M9" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="L9" s="13" t="s">
+      <c r="N9" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="M9" s="13" t="s">
+      <c r="O9" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="N9" s="13" t="s">
+      <c r="P9" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="O9" s="13" t="s">
+      <c r="Q9" s="13" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="10" spans="1:17" s="9" customFormat="1">
+    <row r="10" spans="1:19" s="9" customFormat="1">
       <c r="A10" s="20">
         <v>9</v>
       </c>
@@ -6502,31 +6575,37 @@
         <v>196</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="E10" s="9" t="s">
+        <v>520</v>
+      </c>
+      <c r="E10" s="20" t="s">
+        <v>522</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="G10" s="9" t="s">
         <v>405</v>
       </c>
-      <c r="F10" s="9">
+      <c r="H10" s="9">
         <v>686</v>
       </c>
-      <c r="G10" s="9">
+      <c r="I10" s="9">
         <v>-330</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="J10" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="K10" s="9" t="s">
+      <c r="M10" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="L10" s="9" t="s">
+      <c r="N10" s="9" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="11" spans="1:17" s="9" customFormat="1">
+    <row r="11" spans="1:19" s="9" customFormat="1">
       <c r="A11" s="20">
         <v>10</v>
       </c>
@@ -6534,37 +6613,43 @@
         <v>199</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="E11" s="9" t="s">
+        <v>520</v>
+      </c>
+      <c r="E11" s="20" t="s">
+        <v>522</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="G11" s="9" t="s">
         <v>405</v>
       </c>
-      <c r="F11" s="9">
+      <c r="H11" s="9">
         <v>686</v>
       </c>
-      <c r="G11" s="9">
+      <c r="I11" s="9">
         <v>-300</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="J11" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="K11" s="9" t="s">
+      <c r="M11" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="L11" s="9" t="s">
+      <c r="N11" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="M11" s="9" t="s">
+      <c r="O11" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="N11" s="9" t="s">
+      <c r="P11" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="O11" s="9" t="s">
+      <c r="Q11" s="9" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="12" spans="1:17" s="9" customFormat="1">
+    <row r="12" spans="1:19" s="9" customFormat="1">
       <c r="A12" s="20">
         <v>11</v>
       </c>
@@ -6572,31 +6657,37 @@
         <v>201</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="E12" s="9" t="s">
+        <v>520</v>
+      </c>
+      <c r="E12" s="20" t="s">
+        <v>522</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="G12" s="9" t="s">
         <v>405</v>
       </c>
-      <c r="F12" s="9">
+      <c r="H12" s="9">
         <v>686</v>
       </c>
-      <c r="G12" s="9">
+      <c r="I12" s="9">
         <v>-270</v>
       </c>
-      <c r="H12" s="9" t="s">
+      <c r="J12" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="K12" s="9" t="s">
+      <c r="M12" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="L12" s="9" t="s">
+      <c r="N12" s="9" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="13" spans="1:17" s="9" customFormat="1">
+    <row r="13" spans="1:19" s="9" customFormat="1">
       <c r="A13" s="20">
         <v>12</v>
       </c>
@@ -6604,31 +6695,37 @@
         <v>203</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="E13" s="9" t="s">
+        <v>520</v>
+      </c>
+      <c r="E13" s="20" t="s">
+        <v>522</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="G13" s="9" t="s">
         <v>405</v>
       </c>
-      <c r="F13" s="9">
+      <c r="H13" s="9">
         <v>1134</v>
       </c>
-      <c r="G13" s="9">
+      <c r="I13" s="9">
         <v>-330</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="J13" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="K13" s="9" t="s">
+      <c r="M13" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="L13" s="9" t="s">
+      <c r="N13" s="9" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="14" spans="1:17" s="9" customFormat="1">
+    <row r="14" spans="1:19" s="9" customFormat="1">
       <c r="A14" s="20">
         <v>13</v>
       </c>
@@ -6636,37 +6733,43 @@
         <v>206</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="E14" s="9" t="s">
+        <v>520</v>
+      </c>
+      <c r="E14" s="20" t="s">
+        <v>522</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="G14" s="9" t="s">
         <v>405</v>
       </c>
-      <c r="F14" s="9">
+      <c r="H14" s="9">
         <v>1134</v>
       </c>
-      <c r="G14" s="9">
+      <c r="I14" s="9">
         <v>-300</v>
       </c>
-      <c r="H14" s="9" t="s">
+      <c r="J14" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="K14" s="9" t="s">
+      <c r="M14" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="L14" s="9" t="s">
+      <c r="N14" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="M14" s="9" t="s">
+      <c r="O14" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="N14" s="9" t="s">
+      <c r="P14" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="O14" s="9" t="s">
+      <c r="Q14" s="9" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="15" spans="1:17" s="9" customFormat="1">
+    <row r="15" spans="1:19" s="9" customFormat="1">
       <c r="A15" s="20">
         <v>14</v>
       </c>
@@ -6674,28 +6777,34 @@
         <v>208</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="E15" s="9" t="s">
+        <v>520</v>
+      </c>
+      <c r="E15" s="20" t="s">
+        <v>522</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="G15" s="9" t="s">
         <v>405</v>
       </c>
-      <c r="F15" s="9">
+      <c r="H15" s="9">
         <v>1134</v>
       </c>
-      <c r="G15" s="9">
+      <c r="I15" s="9">
         <v>-270</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="J15" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="K15" s="9" t="s">
+      <c r="M15" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="L15" s="9" t="s">
+      <c r="N15" s="9" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="16" spans="1:17" s="9" customFormat="1">
+    <row r="16" spans="1:19" s="9" customFormat="1">
       <c r="A16" s="20">
         <v>15</v>
       </c>
@@ -6703,28 +6812,34 @@
         <v>210</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="E16" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="E16" s="20" t="s">
+        <v>522</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="G16" s="9" t="s">
         <v>402</v>
       </c>
-      <c r="F16" s="9">
+      <c r="H16" s="9">
         <v>1186</v>
       </c>
-      <c r="G16" s="9">
+      <c r="I16" s="9">
         <v>-240</v>
       </c>
-      <c r="H16" s="9" t="s">
+      <c r="J16" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="K16" s="9" t="s">
+      <c r="M16" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="L16" s="9" t="s">
+      <c r="N16" s="9" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="17" spans="1:15" s="9" customFormat="1">
+    <row r="17" spans="1:17" s="9" customFormat="1">
       <c r="A17" s="20">
         <v>16</v>
       </c>
@@ -6732,31 +6847,37 @@
         <v>213</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="E17" s="9" t="s">
+        <v>520</v>
+      </c>
+      <c r="E17" s="20" t="s">
+        <v>522</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="G17" s="9" t="s">
         <v>404</v>
       </c>
-      <c r="F17" s="9">
+      <c r="H17" s="9">
         <v>1186</v>
       </c>
-      <c r="G17" s="9">
+      <c r="I17" s="9">
         <v>-210</v>
       </c>
-      <c r="H17" s="9" t="s">
+      <c r="J17" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="K17" s="9" t="s">
+      <c r="M17" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="L17" s="9" t="s">
+      <c r="N17" s="9" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="18" spans="1:15" s="9" customFormat="1">
+    <row r="18" spans="1:17" s="9" customFormat="1">
       <c r="A18" s="20">
         <v>17</v>
       </c>
@@ -6764,152 +6885,172 @@
         <v>215</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="E18" s="9" t="s">
+        <v>521</v>
+      </c>
+      <c r="E18" s="20"/>
+      <c r="F18" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="G18" s="9" t="s">
         <v>403</v>
       </c>
-      <c r="F18" s="9">
+      <c r="H18" s="9">
         <v>1084</v>
       </c>
-      <c r="G18" s="9">
+      <c r="I18" s="9">
         <v>-210</v>
       </c>
-      <c r="H18" s="9" t="s">
+      <c r="J18" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="K18" s="9" t="s">
+      <c r="M18" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="L18" s="9" t="s">
+      <c r="N18" s="9" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="19" spans="1:15" s="17" customFormat="1">
+    <row r="19" spans="1:17" s="17" customFormat="1">
       <c r="A19" s="16">
         <v>18</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>218</v>
+        <v>515</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>176</v>
-      </c>
-      <c r="E19" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="E19" s="16"/>
+      <c r="F19" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="G19" s="17" t="s">
         <v>402</v>
       </c>
-      <c r="F19" s="17">
+      <c r="H19" s="17">
         <v>420</v>
       </c>
-      <c r="G19" s="17">
+      <c r="I19" s="17">
         <v>-330</v>
       </c>
-      <c r="H19" s="17" t="s">
+      <c r="J19" s="17" t="s">
         <v>177</v>
       </c>
-      <c r="K19" s="17" t="s">
+      <c r="M19" s="17" t="s">
         <v>211</v>
       </c>
-      <c r="L19" s="17" t="s">
+      <c r="N19" s="17" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="20" spans="1:15" s="17" customFormat="1">
+    <row r="20" spans="1:17" s="17" customFormat="1">
       <c r="A20" s="16">
         <v>19</v>
       </c>
       <c r="B20" s="17" t="s">
         <v>220</v>
       </c>
-      <c r="D20" s="17" t="s">
-        <v>176</v>
-      </c>
-      <c r="E20" s="17" t="s">
+      <c r="D20" s="9" t="s">
+        <v>520</v>
+      </c>
+      <c r="E20" s="16"/>
+      <c r="F20" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="G20" s="17" t="s">
         <v>406</v>
       </c>
-      <c r="F20" s="17">
+      <c r="H20" s="17">
         <v>420</v>
       </c>
-      <c r="G20" s="17">
+      <c r="I20" s="17">
         <v>-300</v>
       </c>
-      <c r="H20" s="17" t="s">
+      <c r="J20" s="17" t="s">
         <v>181</v>
       </c>
-      <c r="K20" s="17" t="s">
+      <c r="M20" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="L20" s="17" t="s">
+      <c r="N20" s="17" t="s">
         <v>221</v>
       </c>
-      <c r="M20" s="17" t="s">
+      <c r="O20" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="N20" s="17" t="s">
+      <c r="P20" s="17" t="s">
         <v>186</v>
       </c>
-      <c r="O20" s="17" t="s">
+      <c r="Q20" s="17" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="21" spans="1:15" s="17" customFormat="1">
+    <row r="21" spans="1:17" s="17" customFormat="1">
       <c r="A21" s="16">
         <v>20</v>
       </c>
       <c r="B21" s="17" t="s">
         <v>222</v>
       </c>
-      <c r="D21" s="17" t="s">
-        <v>176</v>
-      </c>
-      <c r="E21" s="17" t="s">
+      <c r="D21" s="9" t="s">
+        <v>520</v>
+      </c>
+      <c r="E21" s="16"/>
+      <c r="F21" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="G21" s="17" t="s">
         <v>406</v>
       </c>
-      <c r="F21" s="17">
+      <c r="H21" s="17">
         <v>420</v>
       </c>
-      <c r="G21" s="17">
+      <c r="I21" s="17">
         <v>-270</v>
       </c>
-      <c r="H21" s="17" t="s">
+      <c r="J21" s="17" t="s">
         <v>223</v>
       </c>
-      <c r="K21" s="17" t="s">
+      <c r="M21" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="L21" s="17" t="s">
+      <c r="N21" s="17" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="22" spans="1:15" s="17" customFormat="1">
+    <row r="22" spans="1:17" s="17" customFormat="1">
       <c r="A22" s="16">
         <v>21</v>
       </c>
       <c r="B22" s="17" t="s">
         <v>225</v>
       </c>
-      <c r="D22" s="17" t="s">
-        <v>176</v>
-      </c>
-      <c r="E22" s="17" t="s">
+      <c r="D22" s="9" t="s">
+        <v>520</v>
+      </c>
+      <c r="E22" s="16"/>
+      <c r="F22" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="G22" s="17" t="s">
         <v>406</v>
       </c>
-      <c r="F22" s="17">
+      <c r="H22" s="17">
         <v>420</v>
       </c>
-      <c r="G22" s="17">
+      <c r="I22" s="17">
         <v>-240</v>
       </c>
-      <c r="H22" s="17" t="s">
+      <c r="J22" s="17" t="s">
         <v>223</v>
       </c>
-      <c r="K22" s="17" t="s">
+      <c r="M22" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="L22" s="17" t="s">
+      <c r="N22" s="17" t="s">
         <v>226</v>
       </c>
     </row>
@@ -6923,7 +7064,7 @@
   <dimension ref="A1:P37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="11" customWidth="1"/>
+    <col min="1" max="1" width="5.109375" style="11" customWidth="1"/>
     <col min="2" max="2" width="43.77734375" style="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.109375" style="8" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.88671875" style="8" customWidth="1"/>
@@ -6992,62 +7133,62 @@
         <v>173</v>
       </c>
     </row>
-    <row r="2" spans="1:16" s="13" customFormat="1">
-      <c r="A2" s="12">
+    <row r="2" spans="1:16" s="15" customFormat="1">
+      <c r="A2" s="14">
         <v>1</v>
       </c>
-      <c r="B2" s="13" t="s">
-        <v>303</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="D2" s="13" t="s">
-        <v>404</v>
-      </c>
-      <c r="E2" s="13">
-        <v>-140</v>
-      </c>
-      <c r="F2" s="13">
-        <v>-105</v>
-      </c>
-      <c r="G2" s="13" t="s">
-        <v>299</v>
-      </c>
-      <c r="J2" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="K2" s="13" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" s="13" customFormat="1">
-      <c r="A3" s="12">
+      <c r="B2" s="15" t="s">
+        <v>230</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>402</v>
+      </c>
+      <c r="E2" s="15">
+        <v>1186</v>
+      </c>
+      <c r="F2" s="15">
+        <v>-165</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>211</v>
+      </c>
+      <c r="K2" s="15" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" s="15" customFormat="1">
+      <c r="A3" s="14">
         <v>2</v>
       </c>
-      <c r="B3" s="13" t="s">
-        <v>295</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>404</v>
-      </c>
-      <c r="E3" s="13">
-        <v>270</v>
-      </c>
-      <c r="F3" s="13">
+      <c r="B3" s="15" t="s">
+        <v>232</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>402</v>
+      </c>
+      <c r="E3" s="15">
+        <v>695</v>
+      </c>
+      <c r="F3" s="15">
         <v>-165</v>
       </c>
-      <c r="G3" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="J3" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="K3" s="13" t="s">
-        <v>296</v>
+      <c r="G3" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J3" s="15" t="s">
+        <v>211</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="4" spans="1:16" s="15" customFormat="1">
@@ -7055,16 +7196,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="C4" s="15" t="s">
         <v>176</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E4" s="15">
-        <v>1186</v>
+        <v>840</v>
       </c>
       <c r="F4" s="15">
         <v>-165</v>
@@ -7073,10 +7214,10 @@
         <v>228</v>
       </c>
       <c r="J4" s="15" t="s">
-        <v>211</v>
+        <v>178</v>
       </c>
       <c r="K4" s="15" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
     </row>
     <row r="5" spans="1:16" s="15" customFormat="1">
@@ -7084,28 +7225,28 @@
         <v>4</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="C5" s="15" t="s">
         <v>176</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="E5" s="15">
-        <v>695</v>
+        <v>1245</v>
       </c>
       <c r="F5" s="15">
-        <v>-165</v>
+        <v>-110</v>
       </c>
       <c r="G5" s="15" t="s">
         <v>228</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>211</v>
+        <v>178</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
     </row>
     <row r="6" spans="1:16" s="15" customFormat="1">
@@ -7113,19 +7254,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="C6" s="15" t="s">
         <v>176</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="E6" s="15">
-        <v>840</v>
+        <v>1245</v>
       </c>
       <c r="F6" s="15">
-        <v>-165</v>
+        <v>-80</v>
       </c>
       <c r="G6" s="15" t="s">
         <v>228</v>
@@ -7134,7 +7275,16 @@
         <v>178</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>235</v>
+        <v>239</v>
+      </c>
+      <c r="L6" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="M6" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="N6" s="15" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="7" spans="1:16" s="15" customFormat="1">
@@ -7142,7 +7292,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>176</v>
@@ -7154,7 +7304,7 @@
         <v>1245</v>
       </c>
       <c r="F7" s="15">
-        <v>-110</v>
+        <v>-50</v>
       </c>
       <c r="G7" s="15" t="s">
         <v>228</v>
@@ -7163,7 +7313,7 @@
         <v>178</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
     </row>
     <row r="8" spans="1:16" s="15" customFormat="1">
@@ -7171,37 +7321,28 @@
         <v>7</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C8" s="15" t="s">
         <v>176</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="E8" s="15">
         <v>1245</v>
       </c>
       <c r="F8" s="15">
-        <v>-80</v>
+        <v>-20</v>
       </c>
       <c r="G8" s="15" t="s">
         <v>228</v>
       </c>
       <c r="J8" s="15" t="s">
-        <v>178</v>
+        <v>216</v>
       </c>
       <c r="K8" s="15" t="s">
-        <v>239</v>
-      </c>
-      <c r="L8" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="M8" s="15" t="s">
-        <v>186</v>
-      </c>
-      <c r="N8" s="15" t="s">
-        <v>186</v>
+        <v>243</v>
       </c>
     </row>
     <row r="9" spans="1:16" s="15" customFormat="1">
@@ -7209,28 +7350,28 @@
         <v>8</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="C9" s="15" t="s">
         <v>176</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="E9" s="15">
-        <v>1245</v>
+        <v>1025</v>
       </c>
       <c r="F9" s="15">
-        <v>-50</v>
+        <v>-135</v>
       </c>
       <c r="G9" s="15" t="s">
         <v>228</v>
       </c>
       <c r="J9" s="15" t="s">
-        <v>178</v>
+        <v>216</v>
       </c>
       <c r="K9" s="15" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="10" spans="1:16" s="15" customFormat="1">
@@ -7238,7 +7379,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>242</v>
+        <v>262</v>
       </c>
       <c r="C10" s="15" t="s">
         <v>176</v>
@@ -7247,10 +7388,10 @@
         <v>403</v>
       </c>
       <c r="E10" s="15">
-        <v>1245</v>
+        <v>1025</v>
       </c>
       <c r="F10" s="15">
-        <v>-20</v>
+        <v>-165</v>
       </c>
       <c r="G10" s="15" t="s">
         <v>228</v>
@@ -7259,7 +7400,7 @@
         <v>216</v>
       </c>
       <c r="K10" s="15" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
     </row>
     <row r="11" spans="1:16" s="15" customFormat="1">
@@ -7267,28 +7408,28 @@
         <v>10</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C11" s="15" t="s">
         <v>176</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E11" s="15">
-        <v>1025</v>
+        <v>836</v>
       </c>
       <c r="F11" s="15">
-        <v>-135</v>
+        <v>-100</v>
       </c>
       <c r="G11" s="15" t="s">
         <v>228</v>
       </c>
       <c r="J11" s="15" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="K11" s="15" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="12" spans="1:16" s="15" customFormat="1">
@@ -7296,28 +7437,43 @@
         <v>11</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>262</v>
+        <v>248</v>
       </c>
       <c r="C12" s="15" t="s">
         <v>176</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E12" s="15">
-        <v>1025</v>
+        <v>836</v>
       </c>
       <c r="F12" s="15">
-        <v>-165</v>
+        <v>-70</v>
       </c>
       <c r="G12" s="15" t="s">
         <v>228</v>
       </c>
       <c r="J12" s="15" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="K12" s="15" t="s">
-        <v>263</v>
+        <v>249</v>
+      </c>
+      <c r="L12" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="M12" s="15" t="s">
+        <v>250</v>
+      </c>
+      <c r="N12" s="15" t="s">
+        <v>251</v>
+      </c>
+      <c r="O12" s="15" t="s">
+        <v>252</v>
+      </c>
+      <c r="P12" s="15" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="13" spans="1:16" s="15" customFormat="1">
@@ -7325,28 +7481,28 @@
         <v>12</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="C13" s="15" t="s">
         <v>176</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E13" s="15">
         <v>836</v>
       </c>
       <c r="F13" s="15">
-        <v>-100</v>
+        <v>-40</v>
       </c>
       <c r="G13" s="15" t="s">
         <v>228</v>
       </c>
       <c r="J13" s="15" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="K13" s="15" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
     </row>
     <row r="14" spans="1:16" s="15" customFormat="1">
@@ -7354,43 +7510,28 @@
         <v>13</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>248</v>
+        <v>258</v>
       </c>
       <c r="C14" s="15" t="s">
         <v>176</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E14" s="15">
-        <v>836</v>
+        <v>1305</v>
       </c>
       <c r="F14" s="15">
-        <v>-70</v>
+        <v>-170</v>
       </c>
       <c r="G14" s="15" t="s">
         <v>228</v>
       </c>
       <c r="J14" s="15" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="K14" s="15" t="s">
-        <v>249</v>
-      </c>
-      <c r="L14" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="M14" s="15" t="s">
-        <v>250</v>
-      </c>
-      <c r="N14" s="15" t="s">
-        <v>251</v>
-      </c>
-      <c r="O14" s="15" t="s">
-        <v>252</v>
-      </c>
-      <c r="P14" s="15" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
     </row>
     <row r="15" spans="1:16" s="15" customFormat="1">
@@ -7398,7 +7539,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="C15" s="15" t="s">
         <v>176</v>
@@ -7407,10 +7548,10 @@
         <v>403</v>
       </c>
       <c r="E15" s="15">
-        <v>836</v>
+        <v>1485</v>
       </c>
       <c r="F15" s="15">
-        <v>-40</v>
+        <v>-165</v>
       </c>
       <c r="G15" s="15" t="s">
         <v>228</v>
@@ -7419,7 +7560,7 @@
         <v>216</v>
       </c>
       <c r="K15" s="15" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
     </row>
     <row r="16" spans="1:16" s="15" customFormat="1">
@@ -7427,7 +7568,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="C16" s="15" t="s">
         <v>176</v>
@@ -7436,10 +7577,10 @@
         <v>403</v>
       </c>
       <c r="E16" s="15">
-        <v>1305</v>
+        <v>1485</v>
       </c>
       <c r="F16" s="15">
-        <v>-170</v>
+        <v>-135</v>
       </c>
       <c r="G16" s="15" t="s">
         <v>228</v>
@@ -7448,7 +7589,7 @@
         <v>216</v>
       </c>
       <c r="K16" s="15" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
     </row>
     <row r="17" spans="1:11" s="15" customFormat="1">
@@ -7456,7 +7597,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="C17" s="15" t="s">
         <v>176</v>
@@ -7468,7 +7609,7 @@
         <v>1485</v>
       </c>
       <c r="F17" s="15">
-        <v>-165</v>
+        <v>-100</v>
       </c>
       <c r="G17" s="15" t="s">
         <v>228</v>
@@ -7477,7 +7618,7 @@
         <v>216</v>
       </c>
       <c r="K17" s="15" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
     </row>
     <row r="18" spans="1:11" s="15" customFormat="1">
@@ -7485,7 +7626,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="C18" s="15" t="s">
         <v>176</v>
@@ -7497,7 +7638,7 @@
         <v>1485</v>
       </c>
       <c r="F18" s="15">
-        <v>-135</v>
+        <v>-70</v>
       </c>
       <c r="G18" s="15" t="s">
         <v>228</v>
@@ -7506,7 +7647,7 @@
         <v>216</v>
       </c>
       <c r="K18" s="15" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
     </row>
     <row r="19" spans="1:11" s="15" customFormat="1">
@@ -7514,28 +7655,28 @@
         <v>18</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>266</v>
+        <v>227</v>
       </c>
       <c r="C19" s="15" t="s">
         <v>176</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E19" s="15">
-        <v>1485</v>
+        <v>1428</v>
       </c>
       <c r="F19" s="15">
-        <v>-100</v>
+        <v>-50</v>
       </c>
       <c r="G19" s="15" t="s">
         <v>228</v>
       </c>
       <c r="J19" s="15" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="K19" s="15" t="s">
-        <v>267</v>
+        <v>229</v>
       </c>
     </row>
     <row r="20" spans="1:11" s="15" customFormat="1">
@@ -7543,7 +7684,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>268</v>
+        <v>256</v>
       </c>
       <c r="C20" s="15" t="s">
         <v>176</v>
@@ -7552,10 +7693,10 @@
         <v>403</v>
       </c>
       <c r="E20" s="15">
-        <v>1485</v>
+        <v>1428</v>
       </c>
       <c r="F20" s="15">
-        <v>-70</v>
+        <v>-20</v>
       </c>
       <c r="G20" s="15" t="s">
         <v>228</v>
@@ -7564,7 +7705,7 @@
         <v>216</v>
       </c>
       <c r="K20" s="15" t="s">
-        <v>269</v>
+        <v>257</v>
       </c>
     </row>
     <row r="21" spans="1:11" s="15" customFormat="1">
@@ -7572,28 +7713,28 @@
         <v>20</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>227</v>
+        <v>270</v>
       </c>
       <c r="C21" s="15" t="s">
         <v>176</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E21" s="15">
-        <v>1428</v>
+        <v>695</v>
       </c>
       <c r="F21" s="15">
-        <v>-50</v>
+        <v>-70</v>
       </c>
       <c r="G21" s="15" t="s">
         <v>228</v>
       </c>
       <c r="J21" s="15" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="K21" s="15" t="s">
-        <v>229</v>
+        <v>271</v>
       </c>
     </row>
     <row r="22" spans="1:11" s="15" customFormat="1">
@@ -7601,7 +7742,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>256</v>
+        <v>272</v>
       </c>
       <c r="C22" s="15" t="s">
         <v>176</v>
@@ -7610,10 +7751,10 @@
         <v>403</v>
       </c>
       <c r="E22" s="15">
-        <v>1428</v>
+        <v>695</v>
       </c>
       <c r="F22" s="15">
-        <v>-20</v>
+        <v>-40</v>
       </c>
       <c r="G22" s="15" t="s">
         <v>228</v>
@@ -7622,7 +7763,7 @@
         <v>216</v>
       </c>
       <c r="K22" s="15" t="s">
-        <v>257</v>
+        <v>273</v>
       </c>
     </row>
     <row r="23" spans="1:11" s="15" customFormat="1">
@@ -7630,86 +7771,86 @@
         <v>22</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="C23" s="15" t="s">
         <v>176</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="E23" s="15">
         <v>695</v>
       </c>
       <c r="F23" s="15">
-        <v>-70</v>
+        <v>-10</v>
       </c>
       <c r="G23" s="15" t="s">
         <v>228</v>
       </c>
       <c r="J23" s="15" t="s">
-        <v>216</v>
+        <v>178</v>
       </c>
       <c r="K23" s="15" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" s="15" customFormat="1">
-      <c r="A24" s="14">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" s="22" customFormat="1">
+      <c r="A24" s="21">
         <v>23</v>
       </c>
-      <c r="B24" s="15" t="s">
-        <v>272</v>
-      </c>
-      <c r="C24" s="15" t="s">
-        <v>176</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>403</v>
-      </c>
-      <c r="E24" s="15">
-        <v>695</v>
-      </c>
-      <c r="F24" s="15">
-        <v>-40</v>
-      </c>
-      <c r="G24" s="15" t="s">
-        <v>228</v>
-      </c>
-      <c r="J24" s="15" t="s">
-        <v>216</v>
-      </c>
-      <c r="K24" s="15" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" s="15" customFormat="1">
-      <c r="A25" s="14">
+      <c r="B24" s="22" t="s">
+        <v>276</v>
+      </c>
+      <c r="C24" s="22" t="s">
+        <v>176</v>
+      </c>
+      <c r="D24" s="22" t="s">
+        <v>402</v>
+      </c>
+      <c r="E24" s="22">
+        <v>550</v>
+      </c>
+      <c r="F24" s="22">
+        <v>40</v>
+      </c>
+      <c r="G24" s="22" t="s">
+        <v>277</v>
+      </c>
+      <c r="J24" s="22" t="s">
+        <v>211</v>
+      </c>
+      <c r="K24" s="22" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" s="22" customFormat="1">
+      <c r="A25" s="21">
         <v>24</v>
       </c>
-      <c r="B25" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="C25" s="15" t="s">
-        <v>176</v>
-      </c>
-      <c r="D25" s="15" t="s">
-        <v>406</v>
-      </c>
-      <c r="E25" s="15">
-        <v>695</v>
-      </c>
-      <c r="F25" s="15">
-        <v>-10</v>
-      </c>
-      <c r="G25" s="15" t="s">
-        <v>228</v>
-      </c>
-      <c r="J25" s="15" t="s">
+      <c r="B25" s="22" t="s">
+        <v>279</v>
+      </c>
+      <c r="C25" s="22" t="s">
+        <v>176</v>
+      </c>
+      <c r="D25" s="22" t="s">
+        <v>405</v>
+      </c>
+      <c r="E25" s="22">
+        <v>550</v>
+      </c>
+      <c r="F25" s="22">
+        <v>70</v>
+      </c>
+      <c r="G25" s="22" t="s">
+        <v>277</v>
+      </c>
+      <c r="J25" s="22" t="s">
         <v>178</v>
       </c>
-      <c r="K25" s="15" t="s">
-        <v>275</v>
+      <c r="K25" s="22" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="26" spans="1:11" s="22" customFormat="1">
@@ -7717,86 +7858,86 @@
         <v>25</v>
       </c>
       <c r="B26" s="22" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C26" s="22" t="s">
         <v>176</v>
       </c>
       <c r="D26" s="22" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E26" s="22">
         <v>550</v>
       </c>
       <c r="F26" s="22">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="G26" s="22" t="s">
         <v>277</v>
       </c>
       <c r="J26" s="22" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="K26" s="22" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" s="22" customFormat="1">
-      <c r="A27" s="21">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" s="13" customFormat="1">
+      <c r="A27" s="12">
         <v>26</v>
       </c>
-      <c r="B27" s="22" t="s">
-        <v>279</v>
-      </c>
-      <c r="C27" s="22" t="s">
-        <v>176</v>
-      </c>
-      <c r="D27" s="22" t="s">
-        <v>405</v>
-      </c>
-      <c r="E27" s="22">
-        <v>550</v>
-      </c>
-      <c r="F27" s="22">
-        <v>70</v>
-      </c>
-      <c r="G27" s="22" t="s">
-        <v>277</v>
-      </c>
-      <c r="J27" s="22" t="s">
+      <c r="B27" s="13" t="s">
+        <v>295</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>404</v>
+      </c>
+      <c r="E27" s="13">
+        <v>270</v>
+      </c>
+      <c r="F27" s="13">
+        <v>-165</v>
+      </c>
+      <c r="G27" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="J27" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="K27" s="22" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" s="22" customFormat="1">
-      <c r="A28" s="21">
+      <c r="K27" s="13" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" s="13" customFormat="1">
+      <c r="A28" s="12">
         <v>27</v>
       </c>
-      <c r="B28" s="22" t="s">
-        <v>281</v>
-      </c>
-      <c r="C28" s="22" t="s">
-        <v>176</v>
-      </c>
-      <c r="D28" s="22" t="s">
+      <c r="B28" s="13" t="s">
+        <v>283</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="D28" s="13" t="s">
         <v>403</v>
       </c>
-      <c r="E28" s="22">
-        <v>550</v>
-      </c>
-      <c r="F28" s="22">
-        <v>100</v>
-      </c>
-      <c r="G28" s="22" t="s">
-        <v>277</v>
-      </c>
-      <c r="J28" s="22" t="s">
+      <c r="E28" s="13">
+        <v>270</v>
+      </c>
+      <c r="F28" s="13">
+        <v>-100</v>
+      </c>
+      <c r="G28" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="J28" s="13" t="s">
         <v>216</v>
       </c>
-      <c r="K28" s="22" t="s">
-        <v>282</v>
+      <c r="K28" s="13" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="29" spans="1:11" s="13" customFormat="1">
@@ -7804,7 +7945,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C29" s="13" t="s">
         <v>176</v>
@@ -7816,7 +7957,7 @@
         <v>270</v>
       </c>
       <c r="F29" s="13">
-        <v>-100</v>
+        <v>-70</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>158</v>
@@ -7825,7 +7966,7 @@
         <v>216</v>
       </c>
       <c r="K29" s="13" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="30" spans="1:11" s="13" customFormat="1">
@@ -7833,28 +7974,28 @@
         <v>29</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C30" s="13" t="s">
         <v>176</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E30" s="13">
-        <v>270</v>
+        <v>420</v>
       </c>
       <c r="F30" s="13">
-        <v>-70</v>
+        <v>-165</v>
       </c>
       <c r="G30" s="13" t="s">
         <v>158</v>
       </c>
       <c r="J30" s="13" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="K30" s="13" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="31" spans="1:11" s="13" customFormat="1">
@@ -7862,28 +8003,28 @@
         <v>30</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C31" s="13" t="s">
         <v>176</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="E31" s="13">
         <v>420</v>
       </c>
       <c r="F31" s="13">
-        <v>-165</v>
+        <v>-135</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>158</v>
       </c>
       <c r="J31" s="13" t="s">
-        <v>211</v>
+        <v>178</v>
       </c>
       <c r="K31" s="13" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="32" spans="1:11" s="13" customFormat="1">
@@ -7891,7 +8032,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C32" s="13" t="s">
         <v>176</v>
@@ -7903,7 +8044,7 @@
         <v>420</v>
       </c>
       <c r="F32" s="13">
-        <v>-135</v>
+        <v>-100</v>
       </c>
       <c r="G32" s="13" t="s">
         <v>158</v>
@@ -7912,7 +8053,7 @@
         <v>178</v>
       </c>
       <c r="K32" s="13" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="33" spans="1:11" s="13" customFormat="1">
@@ -7920,28 +8061,28 @@
         <v>32</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="C33" s="13" t="s">
         <v>176</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="E33" s="13">
         <v>420</v>
       </c>
       <c r="F33" s="13">
-        <v>-100</v>
+        <v>-70</v>
       </c>
       <c r="G33" s="13" t="s">
         <v>158</v>
       </c>
       <c r="J33" s="13" t="s">
-        <v>178</v>
+        <v>216</v>
       </c>
       <c r="K33" s="13" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="34" spans="1:11" s="13" customFormat="1">
@@ -7949,7 +8090,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="C34" s="13" t="s">
         <v>176</v>
@@ -7961,7 +8102,7 @@
         <v>420</v>
       </c>
       <c r="F34" s="13">
-        <v>-70</v>
+        <v>-40</v>
       </c>
       <c r="G34" s="13" t="s">
         <v>158</v>
@@ -7970,36 +8111,36 @@
         <v>216</v>
       </c>
       <c r="K34" s="13" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" s="13" customFormat="1">
-      <c r="A35" s="12">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" s="24" customFormat="1">
+      <c r="A35" s="23">
         <v>34</v>
       </c>
-      <c r="B35" s="13" t="s">
-        <v>297</v>
-      </c>
-      <c r="C35" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="D35" s="13" t="s">
-        <v>403</v>
-      </c>
-      <c r="E35" s="13">
-        <v>420</v>
-      </c>
-      <c r="F35" s="13">
-        <v>-40</v>
-      </c>
-      <c r="G35" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="J35" s="13" t="s">
-        <v>216</v>
-      </c>
-      <c r="K35" s="13" t="s">
-        <v>298</v>
+      <c r="B35" s="24" t="s">
+        <v>287</v>
+      </c>
+      <c r="C35" s="24" t="s">
+        <v>176</v>
+      </c>
+      <c r="D35" s="24" t="s">
+        <v>402</v>
+      </c>
+      <c r="E35" s="24">
+        <v>-140</v>
+      </c>
+      <c r="F35" s="24">
+        <v>-165</v>
+      </c>
+      <c r="G35" s="24" t="s">
+        <v>299</v>
+      </c>
+      <c r="J35" s="24" t="s">
+        <v>211</v>
+      </c>
+      <c r="K35" s="24" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="36" spans="1:11" s="24" customFormat="1">
@@ -8007,28 +8148,28 @@
         <v>35</v>
       </c>
       <c r="B36" s="24" t="s">
-        <v>287</v>
+        <v>301</v>
       </c>
       <c r="C36" s="24" t="s">
         <v>176</v>
       </c>
       <c r="D36" s="24" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="E36" s="24">
         <v>-140</v>
       </c>
       <c r="F36" s="24">
-        <v>-165</v>
+        <v>-135</v>
       </c>
       <c r="G36" s="24" t="s">
         <v>299</v>
       </c>
       <c r="J36" s="24" t="s">
-        <v>211</v>
+        <v>178</v>
       </c>
       <c r="K36" s="24" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="37" spans="1:11" s="24" customFormat="1">
@@ -8036,19 +8177,19 @@
         <v>36</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="C37" s="24" t="s">
         <v>176</v>
       </c>
       <c r="D37" s="24" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="E37" s="24">
         <v>-140</v>
       </c>
       <c r="F37" s="24">
-        <v>-135</v>
+        <v>-105</v>
       </c>
       <c r="G37" s="24" t="s">
         <v>299</v>
@@ -8057,7 +8198,7 @@
         <v>178</v>
       </c>
       <c r="K37" s="24" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
   </sheetData>
@@ -8067,10 +8208,10 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DDE8CCF-D616-44F3-8678-E353565AE52E}">
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" style="11" customWidth="1"/>
+    <col min="1" max="1" width="6.6640625" style="11" customWidth="1"/>
     <col min="2" max="2" width="35.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="23.109375" bestFit="1" customWidth="1"/>
@@ -8132,7 +8273,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="C2" s="13" t="s">
         <v>176</v>
@@ -8144,16 +8285,16 @@
         <v>420</v>
       </c>
       <c r="F2" s="13">
-        <v>-690</v>
+        <v>-600</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="J2" s="13" t="s">
         <v>178</v>
       </c>
       <c r="K2" s="13" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="3" spans="1:16" s="13" customFormat="1">
@@ -8161,7 +8302,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>305</v>
+        <v>412</v>
       </c>
       <c r="C3" s="13" t="s">
         <v>176</v>
@@ -8173,16 +8314,16 @@
         <v>420</v>
       </c>
       <c r="F3" s="13">
-        <v>-660</v>
+        <v>-570</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>299</v>
+        <v>188</v>
       </c>
       <c r="J3" s="13" t="s">
         <v>178</v>
       </c>
       <c r="K3" s="13" t="s">
-        <v>487</v>
+        <v>413</v>
       </c>
     </row>
     <row r="4" spans="1:16" s="13" customFormat="1">
@@ -8190,7 +8331,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>408</v>
+        <v>183</v>
       </c>
       <c r="C4" s="13" t="s">
         <v>176</v>
@@ -8202,7 +8343,7 @@
         <v>420</v>
       </c>
       <c r="F4" s="13">
-        <v>-630</v>
+        <v>-540</v>
       </c>
       <c r="G4" s="13" t="s">
         <v>181</v>
@@ -8211,7 +8352,16 @@
         <v>178</v>
       </c>
       <c r="K4" s="13" t="s">
-        <v>409</v>
+        <v>414</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="M4" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="N4" s="13" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="5" spans="1:16" s="13" customFormat="1">
@@ -8219,7 +8369,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>176</v>
@@ -8231,16 +8381,25 @@
         <v>420</v>
       </c>
       <c r="F5" s="13">
-        <v>-600</v>
+        <v>-510</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="J5" s="13" t="s">
         <v>178</v>
       </c>
       <c r="K5" s="13" t="s">
-        <v>488</v>
+        <v>481</v>
+      </c>
+      <c r="L5" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="M5" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="N5" s="13" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="6" spans="1:16" s="13" customFormat="1">
@@ -8248,7 +8407,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>412</v>
+        <v>190</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>176</v>
@@ -8260,7 +8419,7 @@
         <v>420</v>
       </c>
       <c r="F6" s="13">
-        <v>-570</v>
+        <v>-480</v>
       </c>
       <c r="G6" s="13" t="s">
         <v>188</v>
@@ -8269,7 +8428,16 @@
         <v>178</v>
       </c>
       <c r="K6" s="13" t="s">
-        <v>413</v>
+        <v>489</v>
+      </c>
+      <c r="L6" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="M6" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="N6" s="13" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="7" spans="1:16" s="13" customFormat="1">
@@ -8277,7 +8445,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>183</v>
+        <v>411</v>
       </c>
       <c r="C7" s="13" t="s">
         <v>176</v>
@@ -8289,16 +8457,16 @@
         <v>420</v>
       </c>
       <c r="F7" s="13">
-        <v>-540</v>
+        <v>-450</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="J7" s="13" t="s">
         <v>178</v>
       </c>
       <c r="K7" s="13" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
       <c r="L7" s="13" t="s">
         <v>185</v>
@@ -8307,7 +8475,7 @@
         <v>186</v>
       </c>
       <c r="N7" s="13" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8" spans="1:16" s="13" customFormat="1">
@@ -8315,19 +8483,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="C8" s="13" t="s">
         <v>176</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="E8" s="13">
         <v>420</v>
       </c>
       <c r="F8" s="13">
-        <v>-510</v>
+        <v>-420</v>
       </c>
       <c r="G8" s="13" t="s">
         <v>188</v>
@@ -8336,7 +8504,7 @@
         <v>178</v>
       </c>
       <c r="K8" s="13" t="s">
-        <v>481</v>
+        <v>415</v>
       </c>
       <c r="L8" s="13" t="s">
         <v>185</v>
@@ -8349,70 +8517,65 @@
       </c>
     </row>
     <row r="9" spans="1:16" s="13" customFormat="1">
-      <c r="A9" s="12">
+      <c r="A9" s="14">
         <v>8</v>
       </c>
-      <c r="B9" s="13" t="s">
-        <v>190</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>404</v>
-      </c>
-      <c r="E9" s="13">
-        <v>420</v>
-      </c>
-      <c r="F9" s="13">
-        <v>-480</v>
-      </c>
-      <c r="G9" s="13" t="s">
-        <v>188</v>
-      </c>
-      <c r="J9" s="13" t="s">
+      <c r="B9" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>405</v>
+      </c>
+      <c r="E9" s="15">
+        <v>686</v>
+      </c>
+      <c r="F9" s="15">
+        <v>-750</v>
+      </c>
+      <c r="G9" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15" t="s">
         <v>178</v>
       </c>
-      <c r="K9" s="13" t="s">
-        <v>490</v>
-      </c>
-      <c r="L9" s="13" t="s">
-        <v>185</v>
-      </c>
-      <c r="M9" s="13" t="s">
-        <v>186</v>
-      </c>
-      <c r="N9" s="13" t="s">
-        <v>186</v>
+      <c r="K9" s="15" t="s">
+        <v>416</v>
       </c>
     </row>
     <row r="10" spans="1:16" s="13" customFormat="1">
-      <c r="A10" s="12">
+      <c r="A10" s="14">
         <v>9</v>
       </c>
-      <c r="B10" s="13" t="s">
-        <v>411</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>404</v>
-      </c>
-      <c r="E10" s="13">
-        <v>420</v>
-      </c>
-      <c r="F10" s="13">
-        <v>-450</v>
-      </c>
-      <c r="G10" s="13" t="s">
-        <v>188</v>
-      </c>
-      <c r="J10" s="13" t="s">
+      <c r="B10" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>405</v>
+      </c>
+      <c r="E10" s="15">
+        <v>686</v>
+      </c>
+      <c r="F10" s="15">
+        <v>-720</v>
+      </c>
+      <c r="G10" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15" t="s">
         <v>178</v>
       </c>
-      <c r="K10" s="13" t="s">
-        <v>410</v>
+      <c r="K10" s="15" t="s">
+        <v>417</v>
       </c>
       <c r="L10" s="13" t="s">
         <v>185</v>
@@ -8425,41 +8588,34 @@
       </c>
     </row>
     <row r="11" spans="1:16" s="13" customFormat="1">
-      <c r="A11" s="12">
+      <c r="A11" s="14">
         <v>10</v>
       </c>
-      <c r="B11" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="D11" s="13" t="s">
+      <c r="B11" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="D11" s="15" t="s">
         <v>405</v>
       </c>
-      <c r="E11" s="13">
-        <v>420</v>
-      </c>
-      <c r="F11" s="13">
-        <v>-420</v>
-      </c>
-      <c r="G11" s="13" t="s">
-        <v>188</v>
-      </c>
-      <c r="J11" s="13" t="s">
+      <c r="E11" s="15">
+        <v>686</v>
+      </c>
+      <c r="F11" s="15">
+        <v>-690</v>
+      </c>
+      <c r="G11" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15" t="s">
         <v>178</v>
       </c>
-      <c r="K11" s="13" t="s">
-        <v>415</v>
-      </c>
-      <c r="L11" s="13" t="s">
-        <v>185</v>
-      </c>
-      <c r="M11" s="13" t="s">
-        <v>186</v>
-      </c>
-      <c r="N11" s="13" t="s">
-        <v>186</v>
+      <c r="K11" s="15" t="s">
+        <v>418</v>
       </c>
     </row>
     <row r="12" spans="1:16" s="13" customFormat="1">
@@ -8467,7 +8623,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="C12" s="15" t="s">
         <v>176</v>
@@ -8476,13 +8632,13 @@
         <v>405</v>
       </c>
       <c r="E12" s="15">
-        <v>686</v>
+        <v>1134</v>
       </c>
       <c r="F12" s="15">
         <v>-750</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="H12" s="15"/>
       <c r="I12" s="15"/>
@@ -8490,7 +8646,7 @@
         <v>178</v>
       </c>
       <c r="K12" s="15" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
     </row>
     <row r="13" spans="1:16" s="13" customFormat="1">
@@ -8498,7 +8654,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="C13" s="15" t="s">
         <v>176</v>
@@ -8507,13 +8663,13 @@
         <v>405</v>
       </c>
       <c r="E13" s="15">
-        <v>686</v>
+        <v>1134</v>
       </c>
       <c r="F13" s="15">
         <v>-720</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="H13" s="15"/>
       <c r="I13" s="15"/>
@@ -8521,7 +8677,7 @@
         <v>178</v>
       </c>
       <c r="K13" s="15" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="L13" s="13" t="s">
         <v>185</v>
@@ -8538,7 +8694,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C14" s="15" t="s">
         <v>176</v>
@@ -8547,13 +8703,13 @@
         <v>405</v>
       </c>
       <c r="E14" s="15">
-        <v>686</v>
+        <v>1134</v>
       </c>
       <c r="F14" s="15">
         <v>-690</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="H14" s="15"/>
       <c r="I14" s="15"/>
@@ -8561,7 +8717,7 @@
         <v>178</v>
       </c>
       <c r="K14" s="15" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
     </row>
     <row r="15" spans="1:16" s="13" customFormat="1">
@@ -8569,19 +8725,19 @@
         <v>14</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="C15" s="15" t="s">
         <v>176</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="E15" s="15">
-        <v>1134</v>
+        <v>1186</v>
       </c>
       <c r="F15" s="15">
-        <v>-750</v>
+        <v>-660</v>
       </c>
       <c r="G15" s="15" t="s">
         <v>204</v>
@@ -8589,10 +8745,10 @@
       <c r="H15" s="15"/>
       <c r="I15" s="15"/>
       <c r="J15" s="15" t="s">
-        <v>178</v>
+        <v>211</v>
       </c>
       <c r="K15" s="15" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
     </row>
     <row r="16" spans="1:16" s="13" customFormat="1">
@@ -8600,39 +8756,30 @@
         <v>15</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>206</v>
+        <v>427</v>
       </c>
       <c r="C16" s="15" t="s">
         <v>176</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="E16" s="15">
-        <v>1134</v>
+        <v>1186</v>
       </c>
       <c r="F16" s="15">
-        <v>-720</v>
+        <v>-630</v>
       </c>
       <c r="G16" s="15" t="s">
-        <v>204</v>
+        <v>425</v>
       </c>
       <c r="H16" s="15"/>
       <c r="I16" s="15"/>
       <c r="J16" s="15" t="s">
-        <v>178</v>
+        <v>211</v>
       </c>
       <c r="K16" s="15" t="s">
-        <v>419</v>
-      </c>
-      <c r="L16" s="13" t="s">
-        <v>185</v>
-      </c>
-      <c r="M16" s="13" t="s">
-        <v>186</v>
-      </c>
-      <c r="N16" s="13" t="s">
-        <v>186</v>
+        <v>426</v>
       </c>
     </row>
     <row r="17" spans="1:14" s="13" customFormat="1">
@@ -8640,19 +8787,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="C17" s="15" t="s">
         <v>176</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="E17" s="15">
-        <v>1134</v>
+        <v>1186</v>
       </c>
       <c r="F17" s="15">
-        <v>-690</v>
+        <v>-600</v>
       </c>
       <c r="G17" s="15" t="s">
         <v>204</v>
@@ -8663,7 +8810,7 @@
         <v>178</v>
       </c>
       <c r="K17" s="15" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="18" spans="1:14" s="13" customFormat="1">
@@ -8671,19 +8818,19 @@
         <v>17</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="C18" s="15" t="s">
         <v>176</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E18" s="15">
-        <v>1186</v>
+        <v>1084</v>
       </c>
       <c r="F18" s="15">
-        <v>-660</v>
+        <v>-630</v>
       </c>
       <c r="G18" s="15" t="s">
         <v>204</v>
@@ -8691,103 +8838,112 @@
       <c r="H18" s="15"/>
       <c r="I18" s="15"/>
       <c r="J18" s="15" t="s">
+        <v>216</v>
+      </c>
+      <c r="K18" s="15" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" s="13" customFormat="1">
+      <c r="A19" s="16">
+        <v>18</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="C19" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>402</v>
+      </c>
+      <c r="E19" s="17">
+        <v>160</v>
+      </c>
+      <c r="F19" s="17">
+        <v>-420</v>
+      </c>
+      <c r="G19" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="H19" s="17"/>
+      <c r="I19" s="17"/>
+      <c r="J19" s="17" t="s">
         <v>211</v>
       </c>
-      <c r="K18" s="15" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" s="13" customFormat="1">
-      <c r="A19" s="14">
-        <v>18</v>
-      </c>
-      <c r="B19" s="15" t="s">
-        <v>427</v>
-      </c>
-      <c r="C19" s="15" t="s">
-        <v>176</v>
-      </c>
-      <c r="D19" s="15" t="s">
-        <v>402</v>
-      </c>
-      <c r="E19" s="15">
-        <v>1186</v>
-      </c>
-      <c r="F19" s="15">
-        <v>-630</v>
-      </c>
-      <c r="G19" s="15" t="s">
-        <v>425</v>
-      </c>
-      <c r="H19" s="15"/>
-      <c r="I19" s="15"/>
-      <c r="J19" s="15" t="s">
-        <v>211</v>
-      </c>
-      <c r="K19" s="15" t="s">
-        <v>426</v>
+      <c r="K19" s="17" t="s">
+        <v>474</v>
       </c>
     </row>
     <row r="20" spans="1:14" s="13" customFormat="1">
-      <c r="A20" s="14">
+      <c r="A20" s="16">
         <v>19</v>
       </c>
-      <c r="B20" s="15" t="s">
-        <v>213</v>
-      </c>
-      <c r="C20" s="15" t="s">
-        <v>176</v>
-      </c>
-      <c r="D20" s="15" t="s">
-        <v>404</v>
-      </c>
-      <c r="E20" s="15">
-        <v>1186</v>
-      </c>
-      <c r="F20" s="15">
-        <v>-600</v>
-      </c>
-      <c r="G20" s="15" t="s">
-        <v>204</v>
-      </c>
-      <c r="H20" s="15"/>
-      <c r="I20" s="15"/>
-      <c r="J20" s="15" t="s">
+      <c r="B20" s="17" t="s">
+        <v>220</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="D20" s="17" t="s">
+        <v>406</v>
+      </c>
+      <c r="E20" s="17">
+        <v>160</v>
+      </c>
+      <c r="F20" s="17">
+        <v>-390</v>
+      </c>
+      <c r="G20" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+      <c r="J20" s="17" t="s">
         <v>178</v>
       </c>
-      <c r="K20" s="15" t="s">
-        <v>420</v>
+      <c r="K20" s="17" t="s">
+        <v>407</v>
+      </c>
+      <c r="L20" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="M20" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="N20" s="13" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="21" spans="1:14" s="13" customFormat="1">
-      <c r="A21" s="14">
+      <c r="A21" s="16">
         <v>20</v>
       </c>
-      <c r="B21" s="15" t="s">
-        <v>215</v>
-      </c>
-      <c r="C21" s="15" t="s">
-        <v>176</v>
-      </c>
-      <c r="D21" s="15" t="s">
-        <v>403</v>
-      </c>
-      <c r="E21" s="15">
-        <v>1084</v>
-      </c>
-      <c r="F21" s="15">
-        <v>-630</v>
-      </c>
-      <c r="G21" s="15" t="s">
-        <v>204</v>
-      </c>
-      <c r="H21" s="15"/>
-      <c r="I21" s="15"/>
-      <c r="J21" s="15" t="s">
-        <v>216</v>
-      </c>
-      <c r="K21" s="15" t="s">
-        <v>424</v>
+      <c r="B21" s="17" t="s">
+        <v>475</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>406</v>
+      </c>
+      <c r="E21" s="17">
+        <v>160</v>
+      </c>
+      <c r="F21" s="17">
+        <v>-360</v>
+      </c>
+      <c r="G21" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="H21" s="17"/>
+      <c r="I21" s="17"/>
+      <c r="J21" s="17" t="s">
+        <v>178</v>
+      </c>
+      <c r="K21" s="17" t="s">
+        <v>476</v>
       </c>
     </row>
     <row r="22" spans="1:14" s="13" customFormat="1">
@@ -8795,30 +8951,30 @@
         <v>21</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>218</v>
+        <v>477</v>
       </c>
       <c r="C22" s="17" t="s">
         <v>176</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="E22" s="17">
         <v>160</v>
       </c>
       <c r="F22" s="17">
-        <v>-420</v>
+        <v>-330</v>
       </c>
       <c r="G22" s="17" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="H22" s="17"/>
       <c r="I22" s="17"/>
       <c r="J22" s="17" t="s">
-        <v>211</v>
+        <v>178</v>
       </c>
       <c r="K22" s="17" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
     </row>
     <row r="23" spans="1:14" s="13" customFormat="1">
@@ -8826,7 +8982,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>220</v>
+        <v>479</v>
       </c>
       <c r="C23" s="17" t="s">
         <v>176</v>
@@ -8838,7 +8994,7 @@
         <v>160</v>
       </c>
       <c r="F23" s="17">
-        <v>-390</v>
+        <v>-300</v>
       </c>
       <c r="G23" s="17" t="s">
         <v>181</v>
@@ -8849,16 +9005,7 @@
         <v>178</v>
       </c>
       <c r="K23" s="17" t="s">
-        <v>407</v>
-      </c>
-      <c r="L23" s="13" t="s">
-        <v>185</v>
-      </c>
-      <c r="M23" s="13" t="s">
-        <v>186</v>
-      </c>
-      <c r="N23" s="13" t="s">
-        <v>181</v>
+        <v>480</v>
       </c>
     </row>
     <row r="24" spans="1:14" s="13" customFormat="1">
@@ -8866,7 +9013,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>475</v>
+        <v>484</v>
       </c>
       <c r="C24" s="17" t="s">
         <v>176</v>
@@ -8878,7 +9025,7 @@
         <v>160</v>
       </c>
       <c r="F24" s="17">
-        <v>-360</v>
+        <v>-270</v>
       </c>
       <c r="G24" s="17" t="s">
         <v>181</v>
@@ -8889,7 +9036,7 @@
         <v>178</v>
       </c>
       <c r="K24" s="17" t="s">
-        <v>476</v>
+        <v>485</v>
       </c>
     </row>
     <row r="25" spans="1:14" s="13" customFormat="1">
@@ -8897,7 +9044,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>477</v>
+        <v>482</v>
       </c>
       <c r="C25" s="17" t="s">
         <v>176</v>
@@ -8909,7 +9056,7 @@
         <v>160</v>
       </c>
       <c r="F25" s="17">
-        <v>-330</v>
+        <v>-240</v>
       </c>
       <c r="G25" s="17" t="s">
         <v>181</v>
@@ -8920,99 +9067,6 @@
         <v>178</v>
       </c>
       <c r="K25" s="17" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14" s="13" customFormat="1">
-      <c r="A26" s="16">
-        <v>25</v>
-      </c>
-      <c r="B26" s="17" t="s">
-        <v>479</v>
-      </c>
-      <c r="C26" s="17" t="s">
-        <v>176</v>
-      </c>
-      <c r="D26" s="17" t="s">
-        <v>406</v>
-      </c>
-      <c r="E26" s="17">
-        <v>160</v>
-      </c>
-      <c r="F26" s="17">
-        <v>-300</v>
-      </c>
-      <c r="G26" s="17" t="s">
-        <v>181</v>
-      </c>
-      <c r="H26" s="17"/>
-      <c r="I26" s="17"/>
-      <c r="J26" s="17" t="s">
-        <v>178</v>
-      </c>
-      <c r="K26" s="17" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" s="13" customFormat="1">
-      <c r="A27" s="16">
-        <v>26</v>
-      </c>
-      <c r="B27" s="17" t="s">
-        <v>484</v>
-      </c>
-      <c r="C27" s="17" t="s">
-        <v>176</v>
-      </c>
-      <c r="D27" s="17" t="s">
-        <v>406</v>
-      </c>
-      <c r="E27" s="17">
-        <v>160</v>
-      </c>
-      <c r="F27" s="17">
-        <v>-270</v>
-      </c>
-      <c r="G27" s="17" t="s">
-        <v>181</v>
-      </c>
-      <c r="H27" s="17"/>
-      <c r="I27" s="17"/>
-      <c r="J27" s="17" t="s">
-        <v>178</v>
-      </c>
-      <c r="K27" s="17" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="28" spans="1:14" s="13" customFormat="1">
-      <c r="A28" s="16">
-        <v>27</v>
-      </c>
-      <c r="B28" s="17" t="s">
-        <v>482</v>
-      </c>
-      <c r="C28" s="17" t="s">
-        <v>176</v>
-      </c>
-      <c r="D28" s="17" t="s">
-        <v>406</v>
-      </c>
-      <c r="E28" s="17">
-        <v>160</v>
-      </c>
-      <c r="F28" s="17">
-        <v>-240</v>
-      </c>
-      <c r="G28" s="17" t="s">
-        <v>181</v>
-      </c>
-      <c r="H28" s="17"/>
-      <c r="I28" s="17"/>
-      <c r="J28" s="17" t="s">
-        <v>178</v>
-      </c>
-      <c r="K28" s="17" t="s">
         <v>483</v>
       </c>
     </row>
@@ -9023,10 +9077,10 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBF48B15-98CD-4572-AF47-284D31EEEF23}">
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="11"/>
+    <col min="1" max="1" width="8.21875" style="11" customWidth="1"/>
     <col min="2" max="2" width="49.77734375" style="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.88671875" style="8"/>
     <col min="4" max="4" width="10" style="8" bestFit="1" customWidth="1"/>
@@ -9092,7 +9146,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>295</v>
+        <v>408</v>
       </c>
       <c r="C2" s="13" t="s">
         <v>176</v>
@@ -9104,7 +9158,7 @@
         <v>1280</v>
       </c>
       <c r="F2" s="13">
-        <v>-335</v>
+        <v>-365</v>
       </c>
       <c r="G2" s="13" t="s">
         <v>228</v>
@@ -9113,7 +9167,7 @@
         <v>178</v>
       </c>
       <c r="K2" s="13" t="s">
-        <v>452</v>
+        <v>409</v>
       </c>
     </row>
     <row r="3" spans="1:16" s="13" customFormat="1">
@@ -9121,19 +9175,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>429</v>
+        <v>295</v>
       </c>
       <c r="C3" s="13" t="s">
         <v>176</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="E3" s="13">
         <v>1280</v>
       </c>
       <c r="F3" s="13">
-        <v>-305</v>
+        <v>-335</v>
       </c>
       <c r="G3" s="13" t="s">
         <v>228</v>
@@ -9142,7 +9196,7 @@
         <v>178</v>
       </c>
       <c r="K3" s="13" t="s">
-        <v>437</v>
+        <v>452</v>
       </c>
     </row>
     <row r="4" spans="1:16" s="13" customFormat="1">
@@ -9150,7 +9204,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>238</v>
+        <v>429</v>
       </c>
       <c r="C4" s="13" t="s">
         <v>176</v>
@@ -9162,7 +9216,7 @@
         <v>1280</v>
       </c>
       <c r="F4" s="13">
-        <v>-275</v>
+        <v>-305</v>
       </c>
       <c r="G4" s="13" t="s">
         <v>228</v>
@@ -9171,16 +9225,7 @@
         <v>178</v>
       </c>
       <c r="K4" s="13" t="s">
-        <v>431</v>
-      </c>
-      <c r="L4" s="13" t="s">
-        <v>185</v>
-      </c>
-      <c r="M4" s="13" t="s">
-        <v>186</v>
-      </c>
-      <c r="N4" s="13" t="s">
-        <v>186</v>
+        <v>437</v>
       </c>
     </row>
     <row r="5" spans="1:16" s="13" customFormat="1">
@@ -9188,7 +9233,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>176</v>
@@ -9200,7 +9245,7 @@
         <v>1280</v>
       </c>
       <c r="F5" s="13">
-        <v>-245</v>
+        <v>-275</v>
       </c>
       <c r="G5" s="13" t="s">
         <v>228</v>
@@ -9209,7 +9254,16 @@
         <v>178</v>
       </c>
       <c r="K5" s="13" t="s">
-        <v>432</v>
+        <v>431</v>
+      </c>
+      <c r="L5" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="M5" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="N5" s="13" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="6" spans="1:16" s="13" customFormat="1">
@@ -9217,28 +9271,28 @@
         <v>5</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>428</v>
+        <v>240</v>
       </c>
       <c r="C6" s="13" t="s">
         <v>176</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="E6" s="13">
         <v>1280</v>
       </c>
       <c r="F6" s="13">
-        <v>-215</v>
+        <v>-245</v>
       </c>
       <c r="G6" s="13" t="s">
         <v>228</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>211</v>
+        <v>178</v>
       </c>
       <c r="K6" s="13" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
     </row>
     <row r="7" spans="1:16" s="13" customFormat="1">
@@ -9246,28 +9300,28 @@
         <v>6</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="C7" s="13" t="s">
         <v>176</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E7" s="13">
-        <v>1495</v>
+        <v>1280</v>
       </c>
       <c r="F7" s="13">
-        <v>-335</v>
+        <v>-215</v>
       </c>
       <c r="G7" s="13" t="s">
         <v>228</v>
       </c>
       <c r="J7" s="13" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="K7" s="13" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
     </row>
     <row r="8" spans="1:16" s="13" customFormat="1">
@@ -9275,7 +9329,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>262</v>
+        <v>434</v>
       </c>
       <c r="C8" s="13" t="s">
         <v>176</v>
@@ -9287,7 +9341,7 @@
         <v>1495</v>
       </c>
       <c r="F8" s="13">
-        <v>-305</v>
+        <v>-335</v>
       </c>
       <c r="G8" s="13" t="s">
         <v>228</v>
@@ -9296,7 +9350,7 @@
         <v>216</v>
       </c>
       <c r="K8" s="13" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
     </row>
     <row r="9" spans="1:16" s="13" customFormat="1">
@@ -9304,7 +9358,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>436</v>
+        <v>262</v>
       </c>
       <c r="C9" s="13" t="s">
         <v>176</v>
@@ -9316,7 +9370,7 @@
         <v>1495</v>
       </c>
       <c r="F9" s="13">
-        <v>-275</v>
+        <v>-305</v>
       </c>
       <c r="G9" s="13" t="s">
         <v>228</v>
@@ -9325,7 +9379,7 @@
         <v>216</v>
       </c>
       <c r="K9" s="13" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="10" spans="1:16" s="13" customFormat="1">
@@ -9333,7 +9387,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C10" s="13" t="s">
         <v>176</v>
@@ -9345,7 +9399,7 @@
         <v>1495</v>
       </c>
       <c r="F10" s="13">
-        <v>-245</v>
+        <v>-275</v>
       </c>
       <c r="G10" s="13" t="s">
         <v>228</v>
@@ -9354,7 +9408,7 @@
         <v>216</v>
       </c>
       <c r="K10" s="13" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="11" spans="1:16" s="13" customFormat="1">
@@ -9362,86 +9416,86 @@
         <v>10</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>461</v>
+        <v>435</v>
       </c>
       <c r="C11" s="13" t="s">
         <v>176</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="E11" s="13">
-        <v>1665</v>
+        <v>1495</v>
       </c>
       <c r="F11" s="13">
-        <v>-365</v>
+        <v>-245</v>
       </c>
       <c r="G11" s="13" t="s">
         <v>228</v>
       </c>
       <c r="J11" s="13" t="s">
+        <v>216</v>
+      </c>
+      <c r="K11" s="13" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" s="13" customFormat="1">
+      <c r="A12" s="12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>404</v>
+      </c>
+      <c r="E12" s="13">
+        <v>1665</v>
+      </c>
+      <c r="F12" s="13">
+        <v>-395</v>
+      </c>
+      <c r="G12" s="13" t="s">
+        <v>445</v>
+      </c>
+      <c r="J12" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="K11" s="13" t="s">
+      <c r="K12" s="13" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" s="13" customFormat="1">
+      <c r="A13" s="12">
+        <v>12</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>461</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>405</v>
+      </c>
+      <c r="E13" s="13">
+        <v>1665</v>
+      </c>
+      <c r="F13" s="13">
+        <v>-365</v>
+      </c>
+      <c r="G13" s="13" t="s">
+        <v>445</v>
+      </c>
+      <c r="J13" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="K13" s="13" t="s">
         <v>462</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" s="17" customFormat="1">
-      <c r="A12" s="16">
-        <v>11</v>
-      </c>
-      <c r="B12" s="17" t="s">
-        <v>291</v>
-      </c>
-      <c r="C12" s="17" t="s">
-        <v>176</v>
-      </c>
-      <c r="D12" s="17" t="s">
-        <v>405</v>
-      </c>
-      <c r="E12" s="17">
-        <v>1665</v>
-      </c>
-      <c r="F12" s="17">
-        <v>-335</v>
-      </c>
-      <c r="G12" s="17" t="s">
-        <v>445</v>
-      </c>
-      <c r="J12" s="17" t="s">
-        <v>178</v>
-      </c>
-      <c r="K12" s="17" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" s="17" customFormat="1">
-      <c r="A13" s="16">
-        <v>12</v>
-      </c>
-      <c r="B13" s="17" t="s">
-        <v>450</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>176</v>
-      </c>
-      <c r="D13" s="17" t="s">
-        <v>403</v>
-      </c>
-      <c r="E13" s="17">
-        <v>1665</v>
-      </c>
-      <c r="F13" s="17">
-        <v>-305</v>
-      </c>
-      <c r="G13" s="17" t="s">
-        <v>445</v>
-      </c>
-      <c r="J13" s="17" t="s">
-        <v>216</v>
-      </c>
-      <c r="K13" s="17" t="s">
-        <v>451</v>
       </c>
     </row>
     <row r="14" spans="1:16" s="17" customFormat="1">
@@ -9449,28 +9503,28 @@
         <v>13</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>459</v>
+        <v>291</v>
       </c>
       <c r="C14" s="17" t="s">
         <v>176</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="E14" s="17">
         <v>1665</v>
       </c>
       <c r="F14" s="17">
-        <v>-275</v>
+        <v>-335</v>
       </c>
       <c r="G14" s="17" t="s">
         <v>445</v>
       </c>
       <c r="J14" s="17" t="s">
-        <v>216</v>
+        <v>178</v>
       </c>
       <c r="K14" s="17" t="s">
-        <v>460</v>
+        <v>448</v>
       </c>
     </row>
     <row r="15" spans="1:16" s="17" customFormat="1">
@@ -9478,43 +9532,28 @@
         <v>14</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>248</v>
+        <v>450</v>
       </c>
       <c r="C15" s="17" t="s">
         <v>176</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E15" s="17">
         <v>1665</v>
       </c>
       <c r="F15" s="17">
-        <v>-245</v>
+        <v>-305</v>
       </c>
       <c r="G15" s="17" t="s">
         <v>445</v>
       </c>
       <c r="J15" s="17" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="K15" s="17" t="s">
-        <v>453</v>
-      </c>
-      <c r="L15" s="17" t="s">
-        <v>185</v>
-      </c>
-      <c r="M15" s="17" t="s">
-        <v>250</v>
-      </c>
-      <c r="N15" s="17" t="s">
-        <v>251</v>
-      </c>
-      <c r="O15" s="17" t="s">
-        <v>252</v>
-      </c>
-      <c r="P15" s="17" t="s">
-        <v>253</v>
+        <v>451</v>
       </c>
     </row>
     <row r="16" spans="1:16" s="17" customFormat="1">
@@ -9522,7 +9561,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>254</v>
+        <v>459</v>
       </c>
       <c r="C16" s="17" t="s">
         <v>176</v>
@@ -9534,7 +9573,7 @@
         <v>1665</v>
       </c>
       <c r="F16" s="17">
-        <v>-215</v>
+        <v>-275</v>
       </c>
       <c r="G16" s="17" t="s">
         <v>445</v>
@@ -9543,15 +9582,15 @@
         <v>216</v>
       </c>
       <c r="K16" s="17" t="s">
-        <v>454</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" s="17" customFormat="1">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" s="17" customFormat="1">
       <c r="A17" s="16">
         <v>16</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>444</v>
+        <v>248</v>
       </c>
       <c r="C17" s="17" t="s">
         <v>176</v>
@@ -9560,10 +9599,10 @@
         <v>402</v>
       </c>
       <c r="E17" s="17">
-        <v>1910</v>
+        <v>1665</v>
       </c>
       <c r="F17" s="17">
-        <v>-210</v>
+        <v>-245</v>
       </c>
       <c r="G17" s="17" t="s">
         <v>445</v>
@@ -9572,44 +9611,59 @@
         <v>211</v>
       </c>
       <c r="K17" s="17" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" s="17" customFormat="1">
+        <v>453</v>
+      </c>
+      <c r="L17" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="M17" s="17" t="s">
+        <v>250</v>
+      </c>
+      <c r="N17" s="17" t="s">
+        <v>251</v>
+      </c>
+      <c r="O17" s="17" t="s">
+        <v>252</v>
+      </c>
+      <c r="P17" s="17" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" s="17" customFormat="1">
       <c r="A18" s="16">
         <v>17</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>442</v>
+        <v>254</v>
       </c>
       <c r="C18" s="17" t="s">
         <v>176</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E18" s="17">
-        <v>1910</v>
+        <v>1665</v>
       </c>
       <c r="F18" s="17">
-        <v>-180</v>
+        <v>-215</v>
       </c>
       <c r="G18" s="17" t="s">
         <v>445</v>
       </c>
       <c r="J18" s="17" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="K18" s="17" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" s="17" customFormat="1">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" s="17" customFormat="1">
       <c r="A19" s="16">
         <v>18</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>227</v>
+        <v>444</v>
       </c>
       <c r="C19" s="17" t="s">
         <v>176</v>
@@ -9618,10 +9672,10 @@
         <v>402</v>
       </c>
       <c r="E19" s="17">
-        <v>1700</v>
+        <v>1910</v>
       </c>
       <c r="F19" s="17">
-        <v>-140</v>
+        <v>-210</v>
       </c>
       <c r="G19" s="17" t="s">
         <v>445</v>
@@ -9630,73 +9684,73 @@
         <v>211</v>
       </c>
       <c r="K19" s="17" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" s="17" customFormat="1">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" s="17" customFormat="1">
       <c r="A20" s="16">
         <v>19</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>455</v>
+        <v>442</v>
       </c>
       <c r="C20" s="17" t="s">
         <v>176</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E20" s="17">
-        <v>1610</v>
+        <v>1910</v>
       </c>
       <c r="F20" s="17">
-        <v>-100</v>
+        <v>-180</v>
       </c>
       <c r="G20" s="17" t="s">
         <v>445</v>
       </c>
       <c r="J20" s="17" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="K20" s="17" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" s="17" customFormat="1">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" s="17" customFormat="1">
       <c r="A21" s="16">
         <v>20</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>457</v>
+        <v>227</v>
       </c>
       <c r="C21" s="17" t="s">
         <v>176</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E21" s="17">
-        <v>1610</v>
+        <v>1700</v>
       </c>
       <c r="F21" s="17">
-        <v>-70</v>
+        <v>-140</v>
       </c>
       <c r="G21" s="17" t="s">
         <v>445</v>
       </c>
       <c r="J21" s="17" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="K21" s="17" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" s="17" customFormat="1">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" s="17" customFormat="1">
       <c r="A22" s="16">
         <v>21</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>447</v>
+        <v>455</v>
       </c>
       <c r="C22" s="17" t="s">
         <v>176</v>
@@ -9708,7 +9762,7 @@
         <v>1610</v>
       </c>
       <c r="F22" s="17">
-        <v>-40</v>
+        <v>-100</v>
       </c>
       <c r="G22" s="17" t="s">
         <v>445</v>
@@ -9717,102 +9771,102 @@
         <v>216</v>
       </c>
       <c r="K22" s="17" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" s="17" customFormat="1">
+      <c r="A23" s="16">
+        <v>22</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>457</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="D23" s="17" t="s">
+        <v>403</v>
+      </c>
+      <c r="E23" s="17">
+        <v>1610</v>
+      </c>
+      <c r="F23" s="17">
+        <v>-70</v>
+      </c>
+      <c r="G23" s="17" t="s">
+        <v>445</v>
+      </c>
+      <c r="J23" s="17" t="s">
+        <v>216</v>
+      </c>
+      <c r="K23" s="17" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" s="17" customFormat="1">
+      <c r="A24" s="16">
+        <v>23</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>447</v>
+      </c>
+      <c r="C24" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="D24" s="17" t="s">
+        <v>403</v>
+      </c>
+      <c r="E24" s="17">
+        <v>1610</v>
+      </c>
+      <c r="F24" s="17">
+        <v>-40</v>
+      </c>
+      <c r="G24" s="17" t="s">
+        <v>445</v>
+      </c>
+      <c r="J24" s="17" t="s">
+        <v>216</v>
+      </c>
+      <c r="K24" s="17" t="s">
         <v>449</v>
       </c>
     </row>
-    <row r="23" spans="1:11" s="19" customFormat="1">
-      <c r="A23" s="18">
-        <v>22</v>
-      </c>
-      <c r="B23" s="19" t="s">
-        <v>466</v>
-      </c>
-      <c r="C23" s="19" t="s">
-        <v>176</v>
-      </c>
-      <c r="D23" s="19" t="s">
-        <v>402</v>
-      </c>
-      <c r="E23" s="19">
-        <v>60</v>
-      </c>
-      <c r="F23" s="19">
-        <v>-1245</v>
-      </c>
-      <c r="G23" s="19" t="s">
-        <v>463</v>
-      </c>
-      <c r="J23" s="19" t="s">
-        <v>211</v>
-      </c>
-      <c r="K23" s="19" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" s="19" customFormat="1">
-      <c r="A24" s="18">
-        <v>23</v>
-      </c>
-      <c r="B24" s="19" t="s">
-        <v>464</v>
-      </c>
-      <c r="C24" s="19" t="s">
-        <v>176</v>
-      </c>
-      <c r="D24" s="19" t="s">
-        <v>403</v>
-      </c>
-      <c r="E24" s="19">
-        <v>60</v>
-      </c>
-      <c r="F24" s="19">
-        <v>-1150</v>
-      </c>
-      <c r="G24" s="19" t="s">
-        <v>463</v>
-      </c>
-      <c r="J24" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="K24" s="19" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" s="19" customFormat="1">
+    <row r="25" spans="1:16" s="19" customFormat="1">
       <c r="A25" s="18">
         <v>24</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="C25" s="19" t="s">
         <v>176</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E25" s="19">
         <v>60</v>
       </c>
       <c r="F25" s="19">
-        <v>-1120</v>
+        <v>-1245</v>
       </c>
       <c r="G25" s="19" t="s">
         <v>463</v>
       </c>
       <c r="J25" s="19" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="K25" s="19" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" s="19" customFormat="1">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" s="19" customFormat="1">
       <c r="A26" s="18">
         <v>25</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="C26" s="19" t="s">
         <v>176</v>
@@ -9824,7 +9878,7 @@
         <v>60</v>
       </c>
       <c r="F26" s="19">
-        <v>-1090</v>
+        <v>-1150</v>
       </c>
       <c r="G26" s="19" t="s">
         <v>463</v>
@@ -9833,64 +9887,122 @@
         <v>216</v>
       </c>
       <c r="K26" s="19" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" s="19" customFormat="1">
+      <c r="A27" s="18">
+        <v>26</v>
+      </c>
+      <c r="B27" s="19" t="s">
+        <v>468</v>
+      </c>
+      <c r="C27" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="D27" s="19" t="s">
+        <v>403</v>
+      </c>
+      <c r="E27" s="19">
+        <v>60</v>
+      </c>
+      <c r="F27" s="19">
+        <v>-1120</v>
+      </c>
+      <c r="G27" s="19" t="s">
+        <v>463</v>
+      </c>
+      <c r="J27" s="19" t="s">
+        <v>216</v>
+      </c>
+      <c r="K27" s="19" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" s="19" customFormat="1">
+      <c r="A28" s="18">
+        <v>27</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>470</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="D28" s="19" t="s">
+        <v>403</v>
+      </c>
+      <c r="E28" s="19">
+        <v>60</v>
+      </c>
+      <c r="F28" s="19">
+        <v>-1090</v>
+      </c>
+      <c r="G28" s="19" t="s">
+        <v>463</v>
+      </c>
+      <c r="J28" s="19" t="s">
+        <v>216</v>
+      </c>
+      <c r="K28" s="19" t="s">
         <v>471</v>
       </c>
     </row>
-    <row r="27" spans="1:11" s="9" customFormat="1">
-      <c r="A27" s="20">
-        <v>26</v>
-      </c>
-      <c r="B27" s="9" t="s">
+    <row r="29" spans="1:16" s="9" customFormat="1">
+      <c r="A29" s="20">
+        <v>28</v>
+      </c>
+      <c r="B29" s="9" t="s">
         <v>303</v>
       </c>
-      <c r="C27" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="D27" s="9" t="s">
+      <c r="C29" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="D29" s="9" t="s">
         <v>404</v>
       </c>
-      <c r="E27" s="9">
+      <c r="E29" s="9">
         <v>-505</v>
       </c>
-      <c r="F27" s="9">
+      <c r="F29" s="9">
         <v>-1150</v>
       </c>
-      <c r="G27" s="9" t="s">
+      <c r="G29" s="9" t="s">
         <v>463</v>
       </c>
-      <c r="J27" s="9" t="s">
+      <c r="J29" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="K27" s="9" t="s">
+      <c r="K29" s="9" t="s">
         <v>473</v>
       </c>
     </row>
-    <row r="28" spans="1:11" s="9" customFormat="1">
-      <c r="A28" s="20">
-        <v>27</v>
-      </c>
-      <c r="B28" s="9" t="s">
+    <row r="30" spans="1:16" s="9" customFormat="1">
+      <c r="A30" s="20">
+        <v>29</v>
+      </c>
+      <c r="B30" s="9" t="s">
         <v>301</v>
       </c>
-      <c r="C28" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="D28" s="9" t="s">
+      <c r="C30" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="D30" s="9" t="s">
         <v>406</v>
       </c>
-      <c r="E28" s="9">
+      <c r="E30" s="9">
         <v>-505</v>
       </c>
-      <c r="F28" s="9">
+      <c r="F30" s="9">
         <v>-1120</v>
       </c>
-      <c r="G28" s="9" t="s">
+      <c r="G30" s="9" t="s">
         <v>463</v>
       </c>
-      <c r="J28" s="9" t="s">
+      <c r="J30" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="K28" s="9" t="s">
+      <c r="K30" s="9" t="s">
         <v>472</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update area and machine
</commit_message>
<xml_diff>
--- a/assets/floor_1_data.xlsx
+++ b/assets/floor_1_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\M.Mead\9.FactoryView\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D05224D3-FEB3-4974-A1AD-1F71AF21BCE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70D81C1E-F75F-48D7-A5C6-C7937D308E6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="807" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="807" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="loc_name" sheetId="1" r:id="rId1"/>
@@ -212,7 +212,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1468" uniqueCount="522">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1471" uniqueCount="523">
   <si>
     <t>Name</t>
   </si>
@@ -1778,6 +1778,9 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>#34a4eb</t>
   </si>
 </sst>
 </file>
@@ -2346,7 +2349,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="21.44140625" style="8" customWidth="1"/>
@@ -2548,30 +2551,30 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
-      <c r="A8" t="s">
-        <v>180</v>
-      </c>
-      <c r="B8">
-        <v>-468</v>
-      </c>
-      <c r="C8">
-        <v>-971</v>
-      </c>
-      <c r="D8">
-        <v>591</v>
-      </c>
-      <c r="E8">
-        <v>-190</v>
-      </c>
-      <c r="F8" t="s">
-        <v>317</v>
-      </c>
-      <c r="G8">
+    <row r="8" spans="1:9" s="8" customFormat="1">
+      <c r="A8" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="B8" s="8">
+        <v>314</v>
+      </c>
+      <c r="C8" s="8">
+        <v>-584</v>
+      </c>
+      <c r="D8" s="8">
+        <v>451</v>
+      </c>
+      <c r="E8" s="8">
+        <v>-443</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>522</v>
+      </c>
+      <c r="G8" s="8">
         <v>0.2</v>
       </c>
-      <c r="H8">
-        <v>14</v>
+      <c r="H8" s="8">
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -2579,18 +2582,18 @@
         <v>180</v>
       </c>
       <c r="B9">
-        <v>-1540</v>
+        <v>-468</v>
       </c>
       <c r="C9">
         <v>-971</v>
       </c>
       <c r="D9">
-        <v>-468</v>
+        <v>451</v>
       </c>
       <c r="E9">
         <v>-190</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" t="s">
         <v>317</v>
       </c>
       <c r="G9">
@@ -2600,64 +2603,67 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:9" s="8" customFormat="1">
-      <c r="B10" s="8">
-        <v>-1097</v>
-      </c>
-      <c r="C10" s="8">
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>180</v>
+      </c>
+      <c r="B10">
+        <v>-1540</v>
+      </c>
+      <c r="C10">
+        <v>-971</v>
+      </c>
+      <c r="D10">
+        <v>-468</v>
+      </c>
+      <c r="E10">
         <v>-190</v>
-      </c>
-      <c r="D10" s="8">
-        <v>-90</v>
-      </c>
-      <c r="E10" s="8">
-        <v>-10</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>317</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10">
         <v>0.2</v>
       </c>
-      <c r="H10" s="8">
+      <c r="H10">
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
-      <c r="A11" t="s">
+    <row r="11" spans="1:9" s="8" customFormat="1">
+      <c r="B11" s="8">
+        <v>-1097</v>
+      </c>
+      <c r="C11" s="8">
+        <v>-190</v>
+      </c>
+      <c r="D11" s="8">
+        <v>-90</v>
+      </c>
+      <c r="E11" s="8">
+        <v>-10</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="G11" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="H11" s="8">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" t="s">
         <v>318</v>
       </c>
-      <c r="B11">
+      <c r="B12">
         <v>-206</v>
       </c>
-      <c r="C11">
+      <c r="C12">
         <v>-8</v>
       </c>
-      <c r="D11">
+      <c r="D12">
         <v>119</v>
-      </c>
-      <c r="E11">
-        <v>728</v>
-      </c>
-      <c r="F11" t="s">
-        <v>319</v>
-      </c>
-      <c r="G11">
-        <v>0.2</v>
-      </c>
-      <c r="H11">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="B12">
-        <v>119</v>
-      </c>
-      <c r="C12">
-        <v>488</v>
-      </c>
-      <c r="D12">
-        <v>535</v>
       </c>
       <c r="E12">
         <v>728</v>
@@ -2673,54 +2679,77 @@
       </c>
     </row>
     <row r="13" spans="1:9">
-      <c r="A13" t="s">
-        <v>320</v>
-      </c>
       <c r="B13">
-        <v>-2703</v>
+        <v>119</v>
       </c>
       <c r="C13">
-        <v>-584</v>
+        <v>488</v>
       </c>
       <c r="D13">
-        <v>-1785</v>
+        <v>535</v>
       </c>
       <c r="E13">
-        <v>1308</v>
+        <v>728</v>
       </c>
       <c r="F13" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="G13">
         <v>0.2</v>
       </c>
       <c r="H13">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B14">
-        <v>2121</v>
+        <v>-2703</v>
       </c>
       <c r="C14">
-        <v>-1169</v>
+        <v>-584</v>
       </c>
       <c r="D14">
-        <v>2645</v>
+        <v>-1785</v>
       </c>
       <c r="E14">
-        <v>6</v>
+        <v>1308</v>
       </c>
       <c r="F14" t="s">
-        <v>505</v>
+        <v>321</v>
       </c>
       <c r="G14">
         <v>0.2</v>
       </c>
       <c r="H14">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" t="s">
+        <v>322</v>
+      </c>
+      <c r="B15">
+        <v>2121</v>
+      </c>
+      <c r="C15">
+        <v>-1169</v>
+      </c>
+      <c r="D15">
+        <v>2645</v>
+      </c>
+      <c r="E15">
+        <v>6</v>
+      </c>
+      <c r="F15" t="s">
+        <v>505</v>
+      </c>
+      <c r="G15">
+        <v>0.2</v>
+      </c>
+      <c r="H15">
         <v>14</v>
       </c>
     </row>
@@ -2731,7 +2760,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72DBCD41-868E-493C-81E0-24F62877FB8D}">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="21.44140625" style="8" customWidth="1"/>
@@ -2919,36 +2948,36 @@
     </row>
     <row r="8" spans="1:9">
       <c r="B8" s="8">
-        <v>-468</v>
+        <v>314</v>
       </c>
       <c r="C8" s="8">
-        <v>-971</v>
+        <v>-584</v>
       </c>
       <c r="D8" s="8">
-        <v>591</v>
+        <v>451</v>
       </c>
       <c r="E8" s="8">
-        <v>-190</v>
+        <v>-443</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>317</v>
+        <v>522</v>
       </c>
       <c r="G8" s="8">
         <v>0.2</v>
       </c>
       <c r="H8" s="8">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="B9" s="8">
-        <v>-1540</v>
+        <v>-468</v>
       </c>
       <c r="C9" s="8">
         <v>-971</v>
       </c>
       <c r="D9" s="8">
-        <v>-468</v>
+        <v>591</v>
       </c>
       <c r="E9" s="8">
         <v>-190</v>
@@ -2965,16 +2994,16 @@
     </row>
     <row r="10" spans="1:9">
       <c r="B10" s="8">
-        <v>-1097</v>
+        <v>-1540</v>
       </c>
       <c r="C10" s="8">
+        <v>-971</v>
+      </c>
+      <c r="D10" s="8">
+        <v>-468</v>
+      </c>
+      <c r="E10" s="8">
         <v>-190</v>
-      </c>
-      <c r="D10" s="8">
-        <v>-90</v>
-      </c>
-      <c r="E10" s="8">
-        <v>-10</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>317</v>
@@ -2988,19 +3017,19 @@
     </row>
     <row r="11" spans="1:9">
       <c r="B11" s="8">
-        <v>-206</v>
+        <v>-1097</v>
       </c>
       <c r="C11" s="8">
-        <v>-8</v>
+        <v>-190</v>
       </c>
       <c r="D11" s="8">
-        <v>119</v>
+        <v>-90</v>
       </c>
       <c r="E11" s="8">
-        <v>728</v>
+        <v>-10</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="G11" s="8">
         <v>0.2</v>
@@ -3011,13 +3040,13 @@
     </row>
     <row r="12" spans="1:9">
       <c r="B12" s="8">
+        <v>-206</v>
+      </c>
+      <c r="C12" s="8">
+        <v>-8</v>
+      </c>
+      <c r="D12" s="8">
         <v>119</v>
-      </c>
-      <c r="C12" s="8">
-        <v>488</v>
-      </c>
-      <c r="D12" s="8">
-        <v>535</v>
       </c>
       <c r="E12" s="8">
         <v>728</v>
@@ -3034,47 +3063,70 @@
     </row>
     <row r="13" spans="1:9">
       <c r="B13" s="8">
-        <v>-2703</v>
+        <v>119</v>
       </c>
       <c r="C13" s="8">
-        <v>-584</v>
+        <v>488</v>
       </c>
       <c r="D13" s="8">
-        <v>-1785</v>
+        <v>535</v>
       </c>
       <c r="E13" s="8">
-        <v>1308</v>
+        <v>728</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="G13" s="8">
         <v>0.2</v>
       </c>
       <c r="H13" s="8">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:9">
       <c r="B14" s="8">
-        <v>2121</v>
+        <v>-2703</v>
       </c>
       <c r="C14" s="8">
-        <v>-1169</v>
+        <v>-584</v>
       </c>
       <c r="D14" s="8">
-        <v>2645</v>
+        <v>-1785</v>
       </c>
       <c r="E14" s="8">
-        <v>6</v>
+        <v>1308</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>505</v>
+        <v>321</v>
       </c>
       <c r="G14" s="8">
         <v>0.2</v>
       </c>
       <c r="H14" s="8">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="B15" s="8">
+        <v>2121</v>
+      </c>
+      <c r="C15" s="8">
+        <v>-1169</v>
+      </c>
+      <c r="D15" s="8">
+        <v>2645</v>
+      </c>
+      <c r="E15" s="8">
+        <v>6</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>505</v>
+      </c>
+      <c r="G15" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="H15" s="8">
         <v>14</v>
       </c>
     </row>

</xml_diff>